<commit_message>
Review Nebius compute economics, PUE and structured financing
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R31c4f4b9b00d4ab9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R49fc04845fc44ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R8288f841dca0496c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rfe9e0885443d435d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R596c12a194584f1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R76e382eb87ab4a2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rc26c46b89db744b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0c4b3283f05541f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R1f4545370fcc4234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rd25de35d7b094d53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R49cdfcf44e0c4109"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R5b90e5cf421848c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R78b23928c7c64a87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rba4c0d29382543ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -330,7 +330,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompanyMethodsTable" displayName="CompanyMethodsTable" ref="A4:G17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompanyMethodsTable" displayName="CompanyMethodsTable" ref="A4:G19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Method ID"/>
     <x:tableColumn id="2" name="Company"/>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -638,7 +638,7 @@
         <x:v>Companies configured</x:v>
       </x:c>
       <x:c r="B6" s="19" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D6" s="19" t="str">
         <x:v>Spot compute revenue ($B / IT GW-year)</x:v>
@@ -661,7 +661,7 @@
         <x:v>Operator outputs calculated</x:v>
       </x:c>
       <x:c r="B7" s="19" t="n">
-        <x:f>COUNT('Company Models'!S5:S17)</x:f>
+        <x:f>COUNT('Company Models'!S5:S19)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D7" s="19" t="str">
@@ -758,7 +758,7 @@
         <x:v>SEGMENT-AZURE</x:v>
       </x:c>
       <x:c r="C13" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B13,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B13,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D13" s="19" t="str">
@@ -783,7 +783,7 @@
         <x:v>SEGMENT-AWS</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B14,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B14,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str">
@@ -808,7 +808,7 @@
         <x:v>SEGMENT-GCP</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B15,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B15,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D15" s="19" t="str">
@@ -833,7 +833,7 @@
         <x:v>INTERNAL-META</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B16,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B16,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Internal compute</x:v>
       </x:c>
       <x:c r="D16" s="19" t="str">
@@ -858,7 +858,7 @@
         <x:v>SEGMENT-OCI</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B17,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B17,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D17" s="19" t="str">
@@ -883,7 +883,7 @@
         <x:v>MERCHANT-CRWV</x:v>
       </x:c>
       <x:c r="C18" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B18,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B18,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Neocloud</x:v>
       </x:c>
       <x:c r="D18" s="19" t="str">
@@ -908,12 +908,12 @@
         <x:v>MERCHANT-NBIS</x:v>
       </x:c>
       <x:c r="C19" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B19,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B19,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Neocloud</x:v>
       </x:c>
       <x:c r="D19" s="19" t="str">
         <x:f>'Company Models'!N11</x:f>
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E19" s="58" t="str">
         <x:f>IF('Company Models'!S11="","",'Company Models'!S11)</x:f>
@@ -933,7 +933,7 @@
         <x:v>MERCHANT-IREN</x:v>
       </x:c>
       <x:c r="C20" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B20,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B20,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Neocloud</x:v>
       </x:c>
       <x:c r="D20" s="19" t="str">
@@ -958,7 +958,7 @@
         <x:v>CONTRACT-NSCALE</x:v>
       </x:c>
       <x:c r="C21" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B21,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B21,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Contracted compute</x:v>
       </x:c>
       <x:c r="D21" s="19" t="str">
@@ -984,7 +984,7 @@
         <x:v>PROJECT-XAI</x:v>
       </x:c>
       <x:c r="C22" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B22,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B22,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Reference operator</x:v>
       </x:c>
       <x:c r="D22" s="19" t="str">
@@ -1009,7 +1009,7 @@
         <x:v>PROJECT-STARGATE</x:v>
       </x:c>
       <x:c r="C23" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B23,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B23,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Reference project</x:v>
       </x:c>
       <x:c r="D23" s="19" t="str">
@@ -1034,7 +1034,7 @@
         <x:v>VENDOR-NVDA</x:v>
       </x:c>
       <x:c r="C24" s="19" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B24,Methods!$A$5:$A$17,0)),"")</x:f>
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B24,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Silicon vendor</x:v>
       </x:c>
       <x:c r="D24" s="19" t="str">
@@ -1050,27 +1050,77 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="20" t="str">
+      <x:c r="A25" s="19" t="str">
         <x:f>'Company Models'!A17</x:f>
         <x:v>Broadcom</x:v>
       </x:c>
-      <x:c r="B25" s="20" t="str">
+      <x:c r="B25" s="19" t="str">
         <x:f>'Company Models'!B17</x:f>
         <x:v>VENDOR-AVGO</x:v>
       </x:c>
-      <x:c r="C25" s="20" t="str">
-        <x:f>IFERROR(INDEX(Methods!$C$5:$C$17,MATCH(B25,Methods!$A$5:$A$17,0)),"")</x:f>
+      <x:c r="C25" s="19" t="str">
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B25,Methods!$A$5:$A$19,0)),"")</x:f>
         <x:v>Silicon vendor</x:v>
       </x:c>
-      <x:c r="D25" s="20" t="str">
+      <x:c r="D25" s="19" t="str">
         <x:f>'Company Models'!N17</x:f>
         <x:v>VENDOR ONLY</x:v>
       </x:c>
-      <x:c r="E25" s="59" t="str">
+      <x:c r="E25" s="58" t="str">
         <x:f>IF('Company Models'!S17="","",'Company Models'!S17)</x:f>
       </x:c>
-      <x:c r="F25" s="20" t="str">
+      <x:c r="F25" s="19" t="str">
         <x:f>'Company Models'!T17</x:f>
+        <x:v>Not an operator output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="19" t="str">
+        <x:f>'Company Models'!A18</x:f>
+        <x:v>Bloom Energy</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="str">
+        <x:f>'Company Models'!B18</x:f>
+        <x:v>SUPPLIER-BLOOM</x:v>
+      </x:c>
+      <x:c r="C26" s="19" t="str">
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B26,Methods!$A$5:$A$19,0)),"")</x:f>
+        <x:v>Power supplier</x:v>
+      </x:c>
+      <x:c r="D26" s="19" t="str">
+        <x:f>'Company Models'!N18</x:f>
+        <x:v>VENDOR ONLY</x:v>
+      </x:c>
+      <x:c r="E26" s="58" t="str">
+        <x:f>IF('Company Models'!S18="","",'Company Models'!S18)</x:f>
+      </x:c>
+      <x:c r="F26" s="19" t="str">
+        <x:f>'Company Models'!T18</x:f>
+        <x:v>Not an operator output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="20" t="str">
+        <x:f>'Company Models'!A19</x:f>
+        <x:v>Palantir</x:v>
+      </x:c>
+      <x:c r="B27" s="20" t="str">
+        <x:f>'Company Models'!B19</x:f>
+        <x:v>SOFTWARE-PLTR</x:v>
+      </x:c>
+      <x:c r="C27" s="20" t="str">
+        <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B27,Methods!$A$5:$A$19,0)),"")</x:f>
+        <x:v>Software</x:v>
+      </x:c>
+      <x:c r="D27" s="20" t="str">
+        <x:f>'Company Models'!N19</x:f>
+        <x:v>VENDOR ONLY</x:v>
+      </x:c>
+      <x:c r="E27" s="59" t="str">
+        <x:f>IF('Company Models'!S19="","",'Company Models'!S19)</x:f>
+      </x:c>
+      <x:c r="F27" s="20" t="str">
+        <x:f>'Company Models'!T19</x:f>
         <x:v>Not an operator output</x:v>
       </x:c>
     </x:row>
@@ -1532,10 +1582,14 @@
         <x:v>MERCHANT-NBIS</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D11" s="27"/>
-      <x:c r="E11" s="29"/>
+        <x:v>Q2 2026</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="n">
+        <x:v>574900000</x:v>
+      </x:c>
+      <x:c r="E11" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F11" s="31"/>
       <x:c r="G11" s="33"/>
       <x:c r="H11" s="23"/>
@@ -1544,13 +1598,13 @@
       <x:c r="K11" s="35"/>
       <x:c r="L11" s="35"/>
       <x:c r="M11" s="19" t="str">
-        <x:v>SRC-CHAT-001</x:v>
+        <x:v>SRC-NBIS-Q2FY26-FS</x:v>
       </x:c>
       <x:c r="N11" s="19" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O11" s="43" t="str">
-        <x:v>Needs active connected MW on matching revenue period</x:v>
+        <x:v>Raw segment includes internal/noncompute; Q2 active IT MW and utilization open. PUE 1.25 is 2025 only.</x:v>
       </x:c>
       <x:c r="P11" s="37" t="str">
         <x:f>IF(OR(D11="",E11="",F11=""),"",D11*E11*F11)</x:f>
@@ -1850,63 +1904,153 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="20" t="str">
+      <x:c r="A17" s="19" t="str">
         <x:v>Broadcom</x:v>
       </x:c>
-      <x:c r="B17" s="20" t="str">
+      <x:c r="B17" s="19" t="str">
         <x:v>VENDOR-AVGO</x:v>
       </x:c>
-      <x:c r="C17" s="20" t="str">
+      <x:c r="C17" s="19" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="32"/>
-      <x:c r="G17" s="34" t="n">
+      <x:c r="D17" s="27"/>
+      <x:c r="E17" s="29"/>
+      <x:c r="F17" s="31"/>
+      <x:c r="G17" s="33" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="H17" s="24" t="str">
+      <x:c r="H17" s="23" t="str">
         <x:v>IT load</x:v>
       </x:c>
-      <x:c r="I17" s="36" t="n">
+      <x:c r="I17" s="35" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J17" s="36" t="n">
+      <x:c r="J17" s="35" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K17" s="36" t="n">
+      <x:c r="K17" s="35" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L17" s="36"/>
-      <x:c r="M17" s="20" t="str">
+      <x:c r="L17" s="35"/>
+      <x:c r="M17" s="19" t="str">
         <x:v>SRC-WB-P2S-001</x:v>
       </x:c>
-      <x:c r="N17" s="20" t="str">
+      <x:c r="N17" s="19" t="str">
         <x:v>VENDOR ONLY</x:v>
       </x:c>
-      <x:c r="O17" s="44" t="str">
+      <x:c r="O17" s="43" t="str">
         <x:v>Custom silicon only; architecture mix required</x:v>
       </x:c>
-      <x:c r="P17" s="38" t="str">
+      <x:c r="P17" s="37" t="str">
         <x:f>IF(OR(D17="",E17="",F17=""),"",D17*E17*F17)</x:f>
       </x:c>
-      <x:c r="Q17" s="40" t="n">
+      <x:c r="Q17" s="39" t="n">
         <x:f>IF(G17="","",IF(H17="IT load",G17,IF(H17="Facility power",IF(I17="","",G17/I17),IF(H17="Generation",IF(OR(I17="",J17="",K17=""),"",G17*J17*K17/I17),IF(H17="Effective utilized IT",G17,"")))))</x:f>
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="R17" s="40" t="str">
+      <x:c r="R17" s="39" t="str">
         <x:f>IF(Q17="","",IF(H17="Effective utilized IT",Q17,IF(L17="","",Q17*L17)))</x:f>
       </x:c>
-      <x:c r="S17" s="42" t="str">
+      <x:c r="S17" s="41" t="str">
         <x:f>IF(OR(P17="",R17="",R17=0),"",P17/R17/1000000)</x:f>
       </x:c>
-      <x:c r="T17" s="26" t="str">
+      <x:c r="T17" s="25" t="str">
         <x:f>IF(S17&lt;&gt;"","Calculated",IF(OR(N17="VENDOR ONLY",N17="CAPEX ONLY"),"Not an operator output","Missing numerator or denominator"))</x:f>
         <x:v>Not an operator output</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="19" t="str">
+        <x:v>Bloom Energy</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="str">
+        <x:v>SUPPLIER-BLOOM</x:v>
+      </x:c>
+      <x:c r="C18" s="19" t="str">
+        <x:v>Not reviewed</x:v>
+      </x:c>
+      <x:c r="D18" s="27"/>
+      <x:c r="E18" s="29"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="33"/>
+      <x:c r="H18" s="23"/>
+      <x:c r="I18" s="35"/>
+      <x:c r="J18" s="35"/>
+      <x:c r="K18" s="35"/>
+      <x:c r="L18" s="35"/>
+      <x:c r="M18" s="19" t="str">
+        <x:v>SRC-NBIS-BLOOM-CONTRACT</x:v>
+      </x:c>
+      <x:c r="N18" s="19" t="str">
+        <x:v>VENDOR ONLY</x:v>
+      </x:c>
+      <x:c r="O18" s="43" t="str">
+        <x:v>Power supplier; PUE not applicable; queued via Nebius agreement.</x:v>
+      </x:c>
+      <x:c r="P18" s="37" t="str">
+        <x:f>IF(OR(D18="",E18="",F18=""),"",D18*E18*F18)</x:f>
+      </x:c>
+      <x:c r="Q18" s="39" t="str">
+        <x:f>IF(G18="","",IF(H18="IT load",G18,IF(H18="Facility power",IF(I18="","",G18/I18),IF(H18="Generation",IF(OR(I18="",J18="",K18=""),"",G18*J18*K18/I18),IF(H18="Effective utilized IT",G18,"")))))</x:f>
+      </x:c>
+      <x:c r="R18" s="39" t="str">
+        <x:f>IF(Q18="","",IF(H18="Effective utilized IT",Q18,IF(L18="","",Q18*L18)))</x:f>
+      </x:c>
+      <x:c r="S18" s="41" t="str">
+        <x:f>IF(OR(P18="",R18="",R18=0),"",P18/R18/1000000)</x:f>
+      </x:c>
+      <x:c r="T18" s="25" t="str">
+        <x:f>IF(S18&lt;&gt;"","Calculated",IF(OR(N18="VENDOR ONLY",N18="CAPEX ONLY"),"Not an operator output","Missing numerator or denominator"))</x:f>
+        <x:v>Not an operator output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="20" t="str">
+        <x:v>Palantir</x:v>
+      </x:c>
+      <x:c r="B19" s="20" t="str">
+        <x:v>SOFTWARE-PLTR</x:v>
+      </x:c>
+      <x:c r="C19" s="20" t="str">
+        <x:v>Not reviewed</x:v>
+      </x:c>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="32"/>
+      <x:c r="G19" s="34"/>
+      <x:c r="H19" s="24"/>
+      <x:c r="I19" s="36"/>
+      <x:c r="J19" s="36"/>
+      <x:c r="K19" s="36"/>
+      <x:c r="L19" s="36"/>
+      <x:c r="M19" s="20" t="str">
+        <x:v>SRC-NBIS-PALANTIR-20260908</x:v>
+      </x:c>
+      <x:c r="N19" s="20" t="str">
+        <x:v>VENDOR ONLY</x:v>
+      </x:c>
+      <x:c r="O19" s="44" t="str">
+        <x:v>Software attribution; own PUE not applicable; queued via Nebius partnership.</x:v>
+      </x:c>
+      <x:c r="P19" s="38" t="str">
+        <x:f>IF(OR(D19="",E19="",F19=""),"",D19*E19*F19)</x:f>
+      </x:c>
+      <x:c r="Q19" s="40" t="str">
+        <x:f>IF(G19="","",IF(H19="IT load",G19,IF(H19="Facility power",IF(I19="","",G19/I19),IF(H19="Generation",IF(OR(I19="",J19="",K19=""),"",G19*J19*K19/I19),IF(H19="Effective utilized IT",G19,"")))))</x:f>
+      </x:c>
+      <x:c r="R19" s="40" t="str">
+        <x:f>IF(Q19="","",IF(H19="Effective utilized IT",Q19,IF(L19="","",Q19*L19)))</x:f>
+      </x:c>
+      <x:c r="S19" s="42" t="str">
+        <x:f>IF(OR(P19="",R19="",R19=0),"",P19/R19/1000000)</x:f>
+      </x:c>
+      <x:c r="T19" s="26" t="str">
+        <x:f>IF(S19&lt;&gt;"","Calculated",IF(OR(N19="VENDOR ONLY",N19="CAPEX ONLY"),"Not an operator output","Missing numerator or denominator"))</x:f>
+        <x:v>Not an operator output</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="T5:T17">
+  <x:conditionalFormatting sqref="T5:T19">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Missing"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Calculated"/>
   </x:conditionalFormatting>
@@ -2124,16 +2268,16 @@
         <x:v>Neocloud</x:v>
       </x:c>
       <x:c r="D11" s="43" t="str">
-        <x:v>Annualized AI infrastructure revenue</x:v>
+        <x:v>Annualized external compute-only revenue</x:v>
       </x:c>
       <x:c r="E11" s="43" t="str">
-        <x:v>Weighted-average connected active IT MW times utilization</x:v>
+        <x:v>Time-weighted effective IT MW</x:v>
       </x:c>
       <x:c r="F11" s="43" t="str">
-        <x:v>Separate active reserved and planned capacity</x:v>
+        <x:v>Exclude internal/noncompute; no exit MW; historical PUE not current</x:v>
       </x:c>
       <x:c r="G11" s="43" t="str">
-        <x:v>Configured; inputs open</x:v>
+        <x:v>Partial; numerator and denominator open</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2252,32 +2396,78 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="20" t="str">
+      <x:c r="A17" s="19" t="str">
         <x:v>VENDOR-AVGO</x:v>
       </x:c>
-      <x:c r="B17" s="20" t="str">
+      <x:c r="B17" s="19" t="str">
         <x:v>Broadcom</x:v>
       </x:c>
-      <x:c r="C17" s="44" t="str">
+      <x:c r="C17" s="43" t="str">
         <x:v>Silicon vendor</x:v>
       </x:c>
-      <x:c r="D17" s="44" t="str">
+      <x:c r="D17" s="43" t="str">
         <x:v>Custom accelerator and networking revenue attributable to capacity</x:v>
       </x:c>
-      <x:c r="E17" s="44" t="str">
+      <x:c r="E17" s="43" t="str">
         <x:v>Deployed IT-load GW</x:v>
       </x:c>
-      <x:c r="F17" s="44" t="str">
+      <x:c r="F17" s="43" t="str">
         <x:v>Preserve custom-only perimeter and architecture mix</x:v>
       </x:c>
-      <x:c r="G17" s="44" t="str">
+      <x:c r="G17" s="43" t="str">
         <x:v>Configured; inputs partial</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="19" t="str">
+        <x:v>SUPPLIER-BLOOM</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="str">
+        <x:v>Bloom Energy</x:v>
+      </x:c>
+      <x:c r="C18" s="43" t="str">
+        <x:v>Power supplier</x:v>
+      </x:c>
+      <x:c r="D18" s="43" t="str">
+        <x:v>Attributable capacity service fees</x:v>
+      </x:c>
+      <x:c r="E18" s="43" t="str">
+        <x:v>Guaranteed generation MW service-years</x:v>
+      </x:c>
+      <x:c r="F18" s="43" t="str">
+        <x:v>Fuel and generation scope; not operator revenue; PUE not applicable</x:v>
+      </x:c>
+      <x:c r="G18" s="43" t="str">
+        <x:v>Queued; not reviewed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="20" t="str">
+        <x:v>SOFTWARE-PLTR</x:v>
+      </x:c>
+      <x:c r="B19" s="20" t="str">
+        <x:v>Palantir</x:v>
+      </x:c>
+      <x:c r="C19" s="44" t="str">
+        <x:v>Software</x:v>
+      </x:c>
+      <x:c r="D19" s="44" t="str">
+        <x:v>Attributed incremental AI software revenue</x:v>
+      </x:c>
+      <x:c r="E19" s="44" t="str">
+        <x:v>Matching associated average IT MW</x:v>
+      </x:c>
+      <x:c r="F19" s="44" t="str">
+        <x:v>No total-company revenue; separate third-party compute</x:v>
+      </x:c>
+      <x:c r="G19" s="44" t="str">
+        <x:v>Queued; not reviewed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R473e72239eb340db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53b70c1f9e394b1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2901,7 +3091,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re014a0c2a70c4cd8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0536ca08fe794681"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4325,38 +4515,531 @@
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="20" t="str">
+      <x:c r="A38" s="19" t="str">
         <x:v>SRC-CRWV-META-20260409</x:v>
       </x:c>
-      <x:c r="B38" s="46" t="n">
+      <x:c r="B38" s="45" t="n">
         <x:v>46121</x:v>
       </x:c>
-      <x:c r="C38" s="20" t="str">
+      <x:c r="C38" s="19" t="str">
         <x:v>CoreWeave</x:v>
       </x:c>
-      <x:c r="D38" s="44" t="str">
+      <x:c r="D38" s="43" t="str">
         <x:v>CoreWeave and Meta Announce USD21 Billion Expanded AI Infrastructure Agreement</x:v>
       </x:c>
-      <x:c r="E38" s="44" t="str">
+      <x:c r="E38" s="43" t="str">
         <x:v>issuer_customer_agreement</x:v>
       </x:c>
-      <x:c r="F38" s="44" t="str">
+      <x:c r="F38" s="43" t="str">
         <x:v>https://investors.coreweave.com/news/news-details/2026/CoreWeave-and-Meta-Announce-21-Billion-Expanded-AI-Infrastructure-Agreement/default.aspx</x:v>
       </x:c>
-      <x:c r="G38" s="44" t="str">
+      <x:c r="G38" s="43" t="str">
         <x:v>CoreWeave Meta agreement</x:v>
       </x:c>
-      <x:c r="H38" s="44" t="str">
+      <x:c r="H38" s="43" t="str">
         <x:v>primary_read</x:v>
       </x:c>
-      <x:c r="I38" s="44" t="str">
+      <x:c r="I38" s="43" t="str">
         <x:v>Dedicated multi-location capacity through December 2032; initial Vera Rubin deployments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="19" t="str">
+        <x:v>SRC-NBIS-20F-FY25</x:v>
+      </x:c>
+      <x:c r="B39" s="45" t="n">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C39" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D39" s="43" t="str">
+        <x:v>FY2025 Form 20-F</x:v>
+      </x:c>
+      <x:c r="E39" s="43" t="str">
+        <x:v>20-F</x:v>
+      </x:c>
+      <x:c r="F39" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926052948/nbis-20251231x20f.htm</x:v>
+      </x:c>
+      <x:c r="G39" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H39" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I39" s="43" t="str">
+        <x:v>Item 4.B capacity definitions; Item 5.E off-balance-sheet arrangements; Note 2 revenue F-17–F-18; Note 11 commitments; exhibit index</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="19" t="str">
+        <x:v>SRC-NBIS-Q2FY26-FS</x:v>
+      </x:c>
+      <x:c r="B40" s="45" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="C40" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D40" s="43" t="str">
+        <x:v>Q2/H1 2026 financial statements</x:v>
+      </x:c>
+      <x:c r="E40" s="43" t="str">
+        <x:v>6-K_exhibit</x:v>
+      </x:c>
+      <x:c r="F40" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926094844/nbis-20260812xex99d2.htm</x:v>
+      </x:c>
+      <x:c r="G40" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H40" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I40" s="43" t="str">
+        <x:v>Cash-flow statement; Note 2 F-10; Note 4 F-19; Note 8 F-24–F-25; Note 11 F-26; Notes 14–16 F-31–F-34</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="19" t="str">
+        <x:v>SRC-NBIS-Q2FY26-MDNA</x:v>
+      </x:c>
+      <x:c r="B41" s="45" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="C41" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D41" s="43" t="str">
+        <x:v>Q2/H1 2026 management discussion</x:v>
+      </x:c>
+      <x:c r="E41" s="43" t="str">
+        <x:v>6-K_exhibit</x:v>
+      </x:c>
+      <x:c r="F41" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926094844/nbis-20260812xex99d1.htm</x:v>
+      </x:c>
+      <x:c r="G41" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H41" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I41" s="43" t="str">
+        <x:v>p.4 revenue table; liquidity and capital resources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="19" t="str">
+        <x:v>SRC-NBIS-Q2FY26-ER</x:v>
+      </x:c>
+      <x:c r="B42" s="45" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="C42" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D42" s="43" t="str">
+        <x:v>Q2 2026 earnings release</x:v>
+      </x:c>
+      <x:c r="E42" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F42" s="43" t="str">
+        <x:v>https://assets.nebius.com/assets/72a8c258-bbb7-4df7-ab9d-8698f6cb88fc/PR.pdf</x:v>
+      </x:c>
+      <x:c r="G42" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H42" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I42" s="43" t="str">
+        <x:v>Consolidated results and cash-flow tables, 10-page release</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="19" t="str">
+        <x:v>SRC-NBIS-Q2FY26-LETTER</x:v>
+      </x:c>
+      <x:c r="B43" s="45" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="C43" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D43" s="43" t="str">
+        <x:v>Q2 2026 shareholder letter</x:v>
+      </x:c>
+      <x:c r="E43" s="43" t="str">
+        <x:v>shareholder_letter</x:v>
+      </x:c>
+      <x:c r="F43" s="43" t="str">
+        <x:v>https://assets.nebius.com/assets/a6ecfd85-a6cb-4967-8ef7-9a25bd261f9c/SHLQ226.pdf</x:v>
+      </x:c>
+      <x:c r="G43" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H43" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I43" s="43" t="str">
+        <x:v>pp.2–4 pricing and deal economics; p.5 capacity; pp.10–11 financing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="19" t="str">
+        <x:v>SRC-NBIS-ESG-FY25</x:v>
+      </x:c>
+      <x:c r="B44" s="45" t="n">
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="C44" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D44" s="43" t="str">
+        <x:v>2025 Sustainability Report</x:v>
+      </x:c>
+      <x:c r="E44" s="43" t="str">
+        <x:v>sustainability_report</x:v>
+      </x:c>
+      <x:c r="F44" s="43" t="str">
+        <x:v>https://assets.nebius.com/assets/79cf11ba-bb23-4cb8-802e-21dc155be31c/Nebius%202025%20Sustainability%20Report.pdf</x:v>
+      </x:c>
+      <x:c r="G44" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H44" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I44" s="43" t="str">
+        <x:v>p.14 PUE panel and footnotes 1–6; publication date confirmed at nebius.com/sustainability</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="19" t="str">
+        <x:v>SRC-NBIS-MSFT-SOW</x:v>
+      </x:c>
+      <x:c r="B45" s="45" t="n">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C45" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D45" s="43" t="str">
+        <x:v>Microsoft SOW dated September 7 2025, Exhibit 4.4</x:v>
+      </x:c>
+      <x:c r="E45" s="43" t="str">
+        <x:v>contract_exhibit</x:v>
+      </x:c>
+      <x:c r="F45" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926052948/nbis-20251231xex4d4.htm</x:v>
+      </x:c>
+      <x:c r="G45" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H45" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I45" s="43" t="str">
+        <x:v>Sections 2 acceptance and delivery; 3.1 pricing; 3.2 payment; 3.3 termination</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="19" t="str">
+        <x:v>SRC-NBIS-MSFT-ADDENDUM</x:v>
+      </x:c>
+      <x:c r="B46" s="45" t="n">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C46" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D46" s="43" t="str">
+        <x:v>Microsoft January 21 2026 addendum, Exhibit 4.5</x:v>
+      </x:c>
+      <x:c r="E46" s="43" t="str">
+        <x:v>contract_exhibit</x:v>
+      </x:c>
+      <x:c r="F46" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926052948/nbis-20251231xex4d5.htm</x:v>
+      </x:c>
+      <x:c r="G46" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H46" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I46" s="43" t="str">
+        <x:v>Section 2(d) additional tranches no upfront payment; 2(e) monthly GPU fee formula</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="19" t="str">
+        <x:v>SRC-NBIS-META-CONTRACT</x:v>
+      </x:c>
+      <x:c r="B47" s="45" t="n">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="C47" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D47" s="43" t="str">
+        <x:v>Meta March 13 2026 infrastructure agreement, Exhibit 4.3</x:v>
+      </x:c>
+      <x:c r="E47" s="43" t="str">
+        <x:v>contract_exhibit</x:v>
+      </x:c>
+      <x:c r="F47" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926052948/nbis-20251231xex4d3.htm</x:v>
+      </x:c>
+      <x:c r="G47" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H47" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I47" s="43" t="str">
+        <x:v>Sections 2.2 affiliate orders; 14.9 force majeure; 15 financing matters</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="19" t="str">
+        <x:v>SRC-NBIS-META-20260316</x:v>
+      </x:c>
+      <x:c r="B48" s="45" t="n">
+        <x:v>46097</x:v>
+      </x:c>
+      <x:c r="C48" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D48" s="43" t="str">
+        <x:v>New AI infrastructure agreement with Meta</x:v>
+      </x:c>
+      <x:c r="E48" s="43" t="str">
+        <x:v>issuer_press_release</x:v>
+      </x:c>
+      <x:c r="F48" s="43" t="str">
+        <x:v>https://www.businesswire.com/news/home/20260316469367/en/Nebius-Signs-New-AI-Infrastructure-Agreement-with-Meta</x:v>
+      </x:c>
+      <x:c r="G48" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H48" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I48" s="43" t="str">
+        <x:v>Opening three substantive paragraphs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="19" t="str">
+        <x:v>SRC-NBIS-BLOOM-CONTRACT</x:v>
+      </x:c>
+      <x:c r="B49" s="45" t="n">
+        <x:v>46162</x:v>
+      </x:c>
+      <x:c r="C49" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D49" s="43" t="str">
+        <x:v>Q1 financials subsequent event: Bloom fuel-cell capacity agreement</x:v>
+      </x:c>
+      <x:c r="E49" s="43" t="str">
+        <x:v>6-K_exhibit</x:v>
+      </x:c>
+      <x:c r="F49" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926064092/nbis-20260331xex99d2.htm</x:v>
+      </x:c>
+      <x:c r="G49" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H49" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I49" s="43" t="str">
+        <x:v>Note 16 Subsequent Events, F-30, Fuel Cell Capacity Agreement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="19" t="str">
+        <x:v>SRC-NBIS-ABS-20260717</x:v>
+      </x:c>
+      <x:c r="B50" s="45" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+      <x:c r="C50" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D50" s="43" t="str">
+        <x:v>Asset-backed facility signed July 10</x:v>
+      </x:c>
+      <x:c r="E50" s="43" t="str">
+        <x:v>6-K</x:v>
+      </x:c>
+      <x:c r="F50" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926084452/tm2620683d1_6k.htm</x:v>
+      </x:c>
+      <x:c r="G50" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H50" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I50" s="43" t="str">
+        <x:v>ASSET-BACKED FACILITY terms, security, covenants and guarantee paragraphs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="19" t="str">
+        <x:v>SRC-NBIS-CONVERT-20260824</x:v>
+      </x:c>
+      <x:c r="B51" s="45" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="C51" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D51" s="43" t="str">
+        <x:v>Closing of $5.75B convertible senior notes</x:v>
+      </x:c>
+      <x:c r="E51" s="43" t="str">
+        <x:v>6-K_exhibit</x:v>
+      </x:c>
+      <x:c r="F51" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926100347/tm2623863d1_ex99-1.htm</x:v>
+      </x:c>
+      <x:c r="G51" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H51" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I51" s="43" t="str">
+        <x:v>Proceeds, accretion and exchange transaction paragraphs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="19" t="str">
+        <x:v>SRC-NBIS-INDENTURE-2030</x:v>
+      </x:c>
+      <x:c r="B52" s="45" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="C52" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D52" s="43" t="str">
+        <x:v>0.500% notes due 2030 indenture</x:v>
+      </x:c>
+      <x:c r="E52" s="43" t="str">
+        <x:v>indenture</x:v>
+      </x:c>
+      <x:c r="F52" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926100347/tm2623863d1_ex4-1.htm</x:v>
+      </x:c>
+      <x:c r="G52" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H52" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I52" s="43" t="str">
+        <x:v>Section 2.21 and Exhibit C C-1 accreted principal schedule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="19" t="str">
+        <x:v>SRC-NBIS-INDENTURE-2034</x:v>
+      </x:c>
+      <x:c r="B53" s="45" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="C53" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D53" s="43" t="str">
+        <x:v>4.500% notes due 2034 indenture</x:v>
+      </x:c>
+      <x:c r="E53" s="43" t="str">
+        <x:v>indenture</x:v>
+      </x:c>
+      <x:c r="F53" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926100347/tm2623863d1_ex4-3.htm</x:v>
+      </x:c>
+      <x:c r="G53" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H53" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I53" s="43" t="str">
+        <x:v>Sections 1.02(L), 2.21 and Exhibit C C-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="19" t="str">
+        <x:v>SRC-NBIS-PALANTIR-20260908</x:v>
+      </x:c>
+      <x:c r="B54" s="45" t="n">
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="C54" s="19" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D54" s="43" t="str">
+        <x:v>Palantir/Nebius sovereign AI partnership</x:v>
+      </x:c>
+      <x:c r="E54" s="43" t="str">
+        <x:v>6-K_exhibit</x:v>
+      </x:c>
+      <x:c r="F54" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1513845/000110465926105749/tm2624958d1_ex99-1.htm</x:v>
+      </x:c>
+      <x:c r="G54" s="43" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H54" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I54" s="43" t="str">
+        <x:v>Opening partnership and integration description</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="20" t="str">
+        <x:v>SRC-NBIS-NEWSROOM-20260915</x:v>
+      </x:c>
+      <x:c r="B55" s="46" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="C55" s="20" t="str">
+        <x:v>Nebius Group N.V.</x:v>
+      </x:c>
+      <x:c r="D55" s="44" t="str">
+        <x:v>Issuer news index checked September 15</x:v>
+      </x:c>
+      <x:c r="E55" s="44" t="str">
+        <x:v>issuer_index</x:v>
+      </x:c>
+      <x:c r="F55" s="44" t="str">
+        <x:v>https://nebius.com/newsroom</x:v>
+      </x:c>
+      <x:c r="G55" s="44" t="str">
+        <x:v>nebius; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H55" s="44" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I55" s="44" t="str">
+        <x:v>Latest press releases; latest economic news September 8</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3fab472898a49ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e31c788e88e4500"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research IREN AI compute economics
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0c4b3283f05541f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R1f4545370fcc4234"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rd25de35d7b094d53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R49cdfcf44e0c4109"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R5b90e5cf421848c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R78b23928c7c64a87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rba4c0d29382543ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8f42fe57f81947f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R2ba5da2a4ac34032"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R51e1fac7f19d431e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R4390ca48ac6f4f9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R531b80c559bc46e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R62536adaff7845a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R960d766efd57444e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -938,7 +938,7 @@
       </x:c>
       <x:c r="D20" s="19" t="str">
         <x:f>'Company Models'!N12</x:f>
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E20" s="58" t="str">
         <x:f>IF('Company Models'!S12="","",'Company Models'!S12)</x:f>
@@ -1631,11 +1631,17 @@
         <x:v>MERCHANT-IREN</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D12" s="27"/>
-      <x:c r="E12" s="29"/>
-      <x:c r="F12" s="31"/>
+        <x:v>Q4 FY2026</x:v>
+      </x:c>
+      <x:c r="D12" s="27" t="n">
+        <x:v>70515000</x:v>
+      </x:c>
+      <x:c r="E12" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F12" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="G12" s="33"/>
       <x:c r="H12" s="23"/>
       <x:c r="I12" s="35"/>
@@ -1643,16 +1649,17 @@
       <x:c r="K12" s="35"/>
       <x:c r="L12" s="35"/>
       <x:c r="M12" s="19" t="str">
-        <x:v>SRC-CHAT-001</x:v>
+        <x:v>SRC-IREN-10K-FY26</x:v>
       </x:c>
       <x:c r="N12" s="19" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O12" s="43" t="str">
-        <x:v>Exclude mining revenue and mining MW</x:v>
-      </x:c>
-      <x:c r="P12" s="37" t="str">
+        <x:v>AI Cloud revenue only derived from FY less nine months; Q4 average active IT MW, utilization and fleet PUE missing. The 40MW June 30 exit capacity is excluded.</x:v>
+      </x:c>
+      <x:c r="P12" s="37" t="n">
         <x:f>IF(OR(D12="",E12="",F12=""),"",D12*E12*F12)</x:f>
+        <x:v>282060000</x:v>
       </x:c>
       <x:c r="Q12" s="39" t="str">
         <x:f>IF(G12="","",IF(H12="IT load",G12,IF(H12="Facility power",IF(I12="","",G12/I12),IF(H12="Generation",IF(OR(I12="",J12="",K12=""),"",G12*J12*K12/I12),IF(H12="Effective utilized IT",G12,"")))))</x:f>
@@ -2294,13 +2301,13 @@
         <x:v>Annualized AI cloud and services revenue only</x:v>
       </x:c>
       <x:c r="E12" s="43" t="str">
-        <x:v>Average active AI IT MW times utilization</x:v>
+        <x:v>Average active AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F12" s="43" t="str">
         <x:v>Exclude Bitcoin mining revenue and mining power</x:v>
       </x:c>
       <x:c r="G12" s="43" t="str">
-        <x:v>Configured; inputs open</x:v>
+        <x:v>Q4 FY2026 numerator established; average active IT MW utilization and matched PUE open</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2467,7 +2474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53b70c1f9e394b1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41b81da4bb84839"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3091,7 +3098,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0536ca08fe794681"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78a2f8136cb24bc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5008,38 +5015,531 @@
       </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="20" t="str">
+      <x:c r="A55" s="19" t="str">
         <x:v>SRC-NBIS-NEWSROOM-20260915</x:v>
       </x:c>
-      <x:c r="B55" s="46" t="n">
+      <x:c r="B55" s="45" t="n">
         <x:v>46280</x:v>
       </x:c>
-      <x:c r="C55" s="20" t="str">
+      <x:c r="C55" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
       </x:c>
-      <x:c r="D55" s="44" t="str">
+      <x:c r="D55" s="43" t="str">
         <x:v>Issuer news index checked September 15</x:v>
       </x:c>
-      <x:c r="E55" s="44" t="str">
+      <x:c r="E55" s="43" t="str">
         <x:v>issuer_index</x:v>
       </x:c>
-      <x:c r="F55" s="44" t="str">
+      <x:c r="F55" s="43" t="str">
         <x:v>https://nebius.com/newsroom</x:v>
       </x:c>
-      <x:c r="G55" s="44" t="str">
+      <x:c r="G55" s="43" t="str">
         <x:v>nebius; revenue_per_mw; contract_economics</x:v>
       </x:c>
-      <x:c r="H55" s="44" t="str">
+      <x:c r="H55" s="43" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="I55" s="44" t="str">
+      <x:c r="I55" s="43" t="str">
         <x:v>Latest press releases; latest economic news September 8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="19" t="str">
+        <x:v>SRC-IREN-10K-FY26</x:v>
+      </x:c>
+      <x:c r="B56" s="45" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="C56" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D56" s="43" t="str">
+        <x:v>FY2026 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E56" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F56" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000052/iren-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G56" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H56" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I56" s="43" t="str">
+        <x:v>Item 1 pp.12-15; Item 7 pp.115-124; Notes 4 20 23 and 26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="19" t="str">
+        <x:v>SRC-IREN-10Q-Q3FY26</x:v>
+      </x:c>
+      <x:c r="B57" s="45" t="n">
+        <x:v>46150</x:v>
+      </x:c>
+      <x:c r="C57" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D57" s="43" t="str">
+        <x:v>Q3 FY2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E57" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F57" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000026/iren-20260331.htm</x:v>
+      </x:c>
+      <x:c r="G57" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H57" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I57" s="43" t="str">
+        <x:v>Note 2 segment policy; Note 4 revenue; Microsoft agreement; MD&amp;A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="19" t="str">
+        <x:v>SRC-IREN-Q3FY26-ER</x:v>
+      </x:c>
+      <x:c r="B58" s="45" t="n">
+        <x:v>46150</x:v>
+      </x:c>
+      <x:c r="C58" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D58" s="43" t="str">
+        <x:v>Q3 FY2026 results</x:v>
+      </x:c>
+      <x:c r="E58" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F58" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000025/irenreportsq3fy26results.htm</x:v>
+      </x:c>
+      <x:c r="G58" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H58" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I58" s="43" t="str">
+        <x:v>pp.1-4 operating and contract update; p.9 revenue table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="19" t="str">
+        <x:v>SRC-IREN-FY26-ER</x:v>
+      </x:c>
+      <x:c r="B59" s="45" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="C59" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D59" s="43" t="str">
+        <x:v>FY2026 results</x:v>
+      </x:c>
+      <x:c r="E59" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F59" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000051/irenreportsfy26results.htm</x:v>
+      </x:c>
+      <x:c r="G59" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H59" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I59" s="43" t="str">
+        <x:v>pp.1-3 pricing delivery and financing; pp.9-13 financial tables</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="19" t="str">
+        <x:v>SRC-IREN-FY26-PRESENTATION</x:v>
+      </x:c>
+      <x:c r="B60" s="45" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="C60" s="19" t="str">
+        <x:v>IREN Limited</x:v>
+      </x:c>
+      <x:c r="D60" s="43" t="str">
+        <x:v>FY2026 results presentation</x:v>
+      </x:c>
+      <x:c r="E60" s="43" t="str">
+        <x:v>earnings_presentation</x:v>
+      </x:c>
+      <x:c r="F60" s="43" t="str">
+        <x:v>https://iren.gcs-web.com/static-files/1ca5b6f0-4b4d-4710-a7e2-69435e112b60</x:v>
+      </x:c>
+      <x:c r="G60" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H60" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I60" s="43" t="str">
+        <x:v>pp.5 9 11-15 20 22-24 and 26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="19" t="str">
+        <x:v>SRC-IREN-MSFT-8K-20251103</x:v>
+      </x:c>
+      <x:c r="B61" s="45" t="n">
+        <x:v>45964</x:v>
+      </x:c>
+      <x:c r="C61" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D61" s="43" t="str">
+        <x:v>Microsoft and Dell agreements</x:v>
+      </x:c>
+      <x:c r="E61" s="43" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="F61" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000114036125040072/ef20058139_8k.htm</x:v>
+      </x:c>
+      <x:c r="G61" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H61" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I61" s="43" t="str">
+        <x:v>Items 1.01 and 7.01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="19" t="str">
+        <x:v>SRC-IREN-MSFT-CONTRACT</x:v>
+      </x:c>
+      <x:c r="B62" s="45" t="n">
+        <x:v>46058</x:v>
+      </x:c>
+      <x:c r="C62" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D62" s="43" t="str">
+        <x:v>Microsoft partner statement of work</x:v>
+      </x:c>
+      <x:c r="E62" s="43" t="str">
+        <x:v>contract_exhibit</x:v>
+      </x:c>
+      <x:c r="F62" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000015/exhibit103-partnerstatem.htm</x:v>
+      </x:c>
+      <x:c r="G62" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H62" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I62" s="43" t="str">
+        <x:v>pp.3-5 acceptance; pp.6-8 fees tranches and prepayment; pp.9-13 delay and termination</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="19" t="str">
+        <x:v>SRC-IREN-GPUFIN-8K-20260529</x:v>
+      </x:c>
+      <x:c r="B63" s="45" t="n">
+        <x:v>46171</x:v>
+      </x:c>
+      <x:c r="C63" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D63" s="43" t="str">
+        <x:v>Microsoft GPU financing</x:v>
+      </x:c>
+      <x:c r="E63" s="43" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="F63" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000114036126023427/ef20075181_8k.htm</x:v>
+      </x:c>
+      <x:c r="G63" s="43" t="str">
+        <x:v>iren; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H63" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I63" s="43" t="str">
+        <x:v>Item 1.01 financing collateral covenants 1.05x ongoing DSCR and guarantees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="19" t="str">
+        <x:v>SRC-IREN-GPUFIN-NPA</x:v>
+      </x:c>
+      <x:c r="B64" s="45" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="C64" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D64" s="43" t="str">
+        <x:v>5.96% note purchase agreement</x:v>
+      </x:c>
+      <x:c r="E64" s="43" t="str">
+        <x:v>financing_exhibit</x:v>
+      </x:c>
+      <x:c r="F64" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000052/a1036notepurchaseagreeme.htm</x:v>
+      </x:c>
+      <x:c r="G64" s="43" t="str">
+        <x:v>iren; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H64" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I64" s="43" t="str">
+        <x:v>Sections 1 3 8-9 and Schedule B</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="19" t="str">
+        <x:v>SRC-IREN-GPUFIN-CTA</x:v>
+      </x:c>
+      <x:c r="B65" s="45" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="C65" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D65" s="43" t="str">
+        <x:v>GPU financing common terms agreement</x:v>
+      </x:c>
+      <x:c r="E65" s="43" t="str">
+        <x:v>financing_exhibit</x:v>
+      </x:c>
+      <x:c r="F65" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000052/a1037commontermsagreemen.htm</x:v>
+      </x:c>
+      <x:c r="G65" s="43" t="str">
+        <x:v>iren; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H65" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I65" s="43" t="str">
+        <x:v>Sections 3 5 and 6; Schedule 1.1(a)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="19" t="str">
+        <x:v>SRC-IREN-GPUFIN-REMARKETING-GUARANTEE</x:v>
+      </x:c>
+      <x:c r="B66" s="45" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="C66" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D66" s="43" t="str">
+        <x:v>IREN parent remarketing guarantee</x:v>
+      </x:c>
+      <x:c r="E66" s="43" t="str">
+        <x:v>guarantee_exhibit</x:v>
+      </x:c>
+      <x:c r="F66" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000052/a1038irenlimitedparentguar.htm</x:v>
+      </x:c>
+      <x:c r="G66" s="43" t="str">
+        <x:v>iren; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H66" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I66" s="43" t="str">
+        <x:v>Article II guaranteed obligations; release and termination provisions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="19" t="str">
+        <x:v>SRC-IREN-GPUFIN-PERFORMANCE-GUARANTEE</x:v>
+      </x:c>
+      <x:c r="B67" s="45" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="C67" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D67" s="43" t="str">
+        <x:v>IREN managed-services performance guarantee</x:v>
+      </x:c>
+      <x:c r="E67" s="43" t="str">
+        <x:v>guarantee_exhibit</x:v>
+      </x:c>
+      <x:c r="F67" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000052/a1054irenlimitedparentguar.htm</x:v>
+      </x:c>
+      <x:c r="G67" s="43" t="str">
+        <x:v>iren; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H67" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I67" s="43" t="str">
+        <x:v>Sections 1.1 2.1-2.3 and 5.10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="19" t="str">
+        <x:v>SRC-IREN-HORIZON1-20260813</x:v>
+      </x:c>
+      <x:c r="B68" s="45" t="n">
+        <x:v>46247</x:v>
+      </x:c>
+      <x:c r="C68" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D68" s="43" t="str">
+        <x:v>First Horizon 1 Microsoft tranche accepted</x:v>
+      </x:c>
+      <x:c r="E68" s="43" t="str">
+        <x:v>8-K_exhibit</x:v>
+      </x:c>
+      <x:c r="F68" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000114036126032638/ef20080141_8k.htm</x:v>
+      </x:c>
+      <x:c r="G68" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics</x:v>
+      </x:c>
+      <x:c r="H68" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I68" s="43" t="str">
+        <x:v>Opening three paragraphs; 50 IT MW is subsequent to Q4 FY2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="19" t="str">
+        <x:v>SRC-IREN-NVIDIA-DELL-20260526</x:v>
+      </x:c>
+      <x:c r="B69" s="45" t="n">
+        <x:v>46168</x:v>
+      </x:c>
+      <x:c r="C69" s="19" t="str">
+        <x:v>IREN Limited / SEC</x:v>
+      </x:c>
+      <x:c r="D69" s="43" t="str">
+        <x:v>NVIDIA managed services and Dell purchase agreements</x:v>
+      </x:c>
+      <x:c r="E69" s="43" t="str">
+        <x:v>8-K_and_exhibit</x:v>
+      </x:c>
+      <x:c r="F69" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000030/0001878848-26-000030.txt</x:v>
+      </x:c>
+      <x:c r="G69" s="43" t="str">
+        <x:v>iren; revenue_per_mw; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H69" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I69" s="43" t="str">
+        <x:v>Item 1.01 Dell order and guarantee; Exhibit 99.1 NVIDIA contract</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="19" t="str">
+        <x:v>SRC-IREN-PRINCE-GEORGE-SITE-20260916</x:v>
+      </x:c>
+      <x:c r="B70" s="45" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="C70" s="19" t="str">
+        <x:v>IREN Limited</x:v>
+      </x:c>
+      <x:c r="D70" s="43" t="str">
+        <x:v>Prince George data center specifications</x:v>
+      </x:c>
+      <x:c r="E70" s="43" t="str">
+        <x:v>issuer_site_page</x:v>
+      </x:c>
+      <x:c r="F70" s="43" t="str">
+        <x:v>https://iren.com/data-centers/prince-george</x:v>
+      </x:c>
+      <x:c r="G70" s="43" t="str">
+        <x:v>iren; effective_mw</x:v>
+      </x:c>
+      <x:c r="H70" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I70" s="43" t="str">
+        <x:v>50 MW power capacity; average PUE 1.1; no measurement period or energy totals</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="19" t="str">
+        <x:v>SRC-IREN-MACKENZIE-SITE-20260916</x:v>
+      </x:c>
+      <x:c r="B71" s="45" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="C71" s="19" t="str">
+        <x:v>IREN Limited</x:v>
+      </x:c>
+      <x:c r="D71" s="43" t="str">
+        <x:v>Mackenzie data center specifications</x:v>
+      </x:c>
+      <x:c r="E71" s="43" t="str">
+        <x:v>issuer_site_page</x:v>
+      </x:c>
+      <x:c r="F71" s="43" t="str">
+        <x:v>https://iren.com/data-centers/mackenzie</x:v>
+      </x:c>
+      <x:c r="G71" s="43" t="str">
+        <x:v>iren; effective_mw</x:v>
+      </x:c>
+      <x:c r="H71" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I71" s="43" t="str">
+        <x:v>80 MW power capacity; average PUE 1.1; no measurement period or energy totals</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="20" t="str">
+        <x:v>SRC-IREN-SWEETWATER-20260908</x:v>
+      </x:c>
+      <x:c r="B72" s="46" t="n">
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="C72" s="20" t="str">
+        <x:v>IREN Limited</x:v>
+      </x:c>
+      <x:c r="D72" s="44" t="str">
+        <x:v>Sweetwater conditional ERCOT Batch Zero inclusion</x:v>
+      </x:c>
+      <x:c r="E72" s="44" t="str">
+        <x:v>issuer_press_release</x:v>
+      </x:c>
+      <x:c r="F72" s="44" t="str">
+        <x:v>https://iren.gcs-web.com/static-files/32760df9-d8fc-4118-90b3-6c9d3bb815a7</x:v>
+      </x:c>
+      <x:c r="G72" s="44" t="str">
+        <x:v>iren; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H72" s="44" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I72" s="44" t="str">
+        <x:v>p.1 conditional grid inclusion and 300 MW gross construction target</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e31c788e88e4500"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a268069d5204e9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research Microsoft Azure AI compute economics
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8f42fe57f81947f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R2ba5da2a4ac34032"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R51e1fac7f19d431e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R4390ca48ac6f4f9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R531b80c559bc46e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R62536adaff7845a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R960d766efd57444e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R76bb637026234fd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Ra8ad98f090cb493c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R415180b483ba4a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rad79a6c57b8a471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R27e42596888f4373"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Re24f3fea3b7d46c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rd877d39413264515"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -763,7 +763,7 @@
       </x:c>
       <x:c r="D13" s="19" t="str">
         <x:f>'Company Models'!N5</x:f>
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E13" s="58" t="str">
         <x:f>IF('Company Models'!S5="","",'Company Models'!S5)</x:f>
@@ -1300,10 +1300,14 @@
         <x:v>SEGMENT-AZURE</x:v>
       </x:c>
       <x:c r="C5" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D5" s="27"/>
-      <x:c r="E5" s="29"/>
+        <x:v>Q4 FY2026</x:v>
+      </x:c>
+      <x:c r="D5" s="27" t="n">
+        <x:v>29417000000</x:v>
+      </x:c>
+      <x:c r="E5" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F5" s="31"/>
       <x:c r="G5" s="33"/>
       <x:c r="H5" s="23"/>
@@ -1312,13 +1316,13 @@
       <x:c r="K5" s="35"/>
       <x:c r="L5" s="35"/>
       <x:c r="M5" s="19" t="str">
-        <x:v>SRC-CHAT-001</x:v>
+        <x:v>SRC-MSFT-SEGMENT-EX99-20260902</x:v>
       </x:c>
       <x:c r="N5" s="19" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O5" s="43" t="str">
-        <x:v>Needs matching AI revenue attribution and average AI IT MW</x:v>
+        <x:v>Restated Azure revenue; AI share, period-average active AI IT MW, physical utilization and matched full-fleet PUE missing. FY2025 PUE 1.17 and implied 1.55GW owned-fleet IT load are boundary diagnostics only; Q4 1GW addition excluded.</x:v>
       </x:c>
       <x:c r="P5" s="37" t="str">
         <x:f>IF(OR(D5="",E5="",F5=""),"",D5*E5*F5)</x:f>
@@ -2137,16 +2141,16 @@
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D5" s="43" t="str">
-        <x:v>Annualized Azure or Intelligent Cloud revenue attributable to AI compute</x:v>
+        <x:v>Annualized restated Azure revenue attributable to external AI compute</x:v>
       </x:c>
       <x:c r="E5" s="43" t="str">
-        <x:v>Average effective utilized Azure AI IT MW</x:v>
+        <x:v>Time-weighted average active Azure AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F5" s="43" t="str">
-        <x:v>Isolate AI contribution and non-compute services</x:v>
+        <x:v>Use September 2026 restated Azure perimeter; remove virtual desktop and non-AI consumption; include owned, leased, colocated and purchased capacity; never use quarterly added MW or PPA generation</x:v>
       </x:c>
       <x:c r="G5" s="43" t="str">
-        <x:v>Configured; inputs open</x:v>
+        <x:v>Partial 2026-09-17; exact Azure revenue established; AI attribution and effective-MW denominator open</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2474,7 +2478,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41b81da4bb84839"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c6a903f4b0e4e00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3098,7 +3102,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78a2f8136cb24bc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0714630b43aa4eeb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5508,38 +5512,386 @@
       </x:c>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="20" t="str">
+      <x:c r="A72" s="19" t="str">
         <x:v>SRC-IREN-SWEETWATER-20260908</x:v>
       </x:c>
-      <x:c r="B72" s="46" t="n">
+      <x:c r="B72" s="45" t="n">
         <x:v>46273</x:v>
       </x:c>
-      <x:c r="C72" s="20" t="str">
+      <x:c r="C72" s="19" t="str">
         <x:v>IREN Limited</x:v>
       </x:c>
-      <x:c r="D72" s="44" t="str">
+      <x:c r="D72" s="43" t="str">
         <x:v>Sweetwater conditional ERCOT Batch Zero inclusion</x:v>
       </x:c>
-      <x:c r="E72" s="44" t="str">
+      <x:c r="E72" s="43" t="str">
         <x:v>issuer_press_release</x:v>
       </x:c>
-      <x:c r="F72" s="44" t="str">
+      <x:c r="F72" s="43" t="str">
         <x:v>https://iren.gcs-web.com/static-files/32760df9-d8fc-4118-90b3-6c9d3bb815a7</x:v>
       </x:c>
-      <x:c r="G72" s="44" t="str">
+      <x:c r="G72" s="43" t="str">
         <x:v>iren; contract_economics; capex</x:v>
       </x:c>
-      <x:c r="H72" s="44" t="str">
+      <x:c r="H72" s="43" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="I72" s="44" t="str">
+      <x:c r="I72" s="43" t="str">
         <x:v>p.1 conditional grid inclusion and 300 MW gross construction target</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="19" t="str">
+        <x:v>SRC-MSFT-10K-FY26</x:v>
+      </x:c>
+      <x:c r="B73" s="45" t="n">
+        <x:v>46232</x:v>
+      </x:c>
+      <x:c r="C73" s="19" t="str">
+        <x:v>Microsoft Corporation / SEC</x:v>
+      </x:c>
+      <x:c r="D73" s="43" t="str">
+        <x:v>FY2026 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E73" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F73" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/789019/000119312526323660/msft-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G73" s="43" t="str">
+        <x:v>microsoft_azure; revenue_per_mw; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H73" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I73" s="43" t="str">
+        <x:v>Item 7 pp.33-45; Item 8 pp.52, 68-69, 76-79; obligations p.43; Notes 6, 12 and 13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="19" t="str">
+        <x:v>SRC-MSFT-10Q-Q3FY26</x:v>
+      </x:c>
+      <x:c r="B74" s="45" t="n">
+        <x:v>46141</x:v>
+      </x:c>
+      <x:c r="C74" s="19" t="str">
+        <x:v>Microsoft Corporation / SEC</x:v>
+      </x:c>
+      <x:c r="D74" s="43" t="str">
+        <x:v>Q3 FY2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E74" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F74" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/789019/000119312526191507/msft-20260331.htm</x:v>
+      </x:c>
+      <x:c r="G74" s="43" t="str">
+        <x:v>microsoft_azure; revenue_per_mw; contract_economics; capex</x:v>
+      </x:c>
+      <x:c r="H74" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I74" s="43" t="str">
+        <x:v>Notes 11-12 pp.20-24; Item 2 pp.31-47; uncommenced leases p.23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="19" t="str">
+        <x:v>SRC-MSFT-FY26-ER</x:v>
+      </x:c>
+      <x:c r="B75" s="45" t="n">
+        <x:v>46232</x:v>
+      </x:c>
+      <x:c r="C75" s="19" t="str">
+        <x:v>Microsoft Corporation / SEC</x:v>
+      </x:c>
+      <x:c r="D75" s="43" t="str">
+        <x:v>Q4 and FY2026 results</x:v>
+      </x:c>
+      <x:c r="E75" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F75" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/789019/000119312526323632/msft-ex99_1.htm</x:v>
+      </x:c>
+      <x:c r="G75" s="43" t="str">
+        <x:v>microsoft_azure; revenue_per_mw; capex</x:v>
+      </x:c>
+      <x:c r="H75" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I75" s="43" t="str">
+        <x:v>Business Highlights and financial tables</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="19" t="str">
+        <x:v>SRC-MSFT-FY26-CALL</x:v>
+      </x:c>
+      <x:c r="B76" s="45" t="n">
+        <x:v>46232</x:v>
+      </x:c>
+      <x:c r="C76" s="19" t="str">
+        <x:v>Microsoft Corporation</x:v>
+      </x:c>
+      <x:c r="D76" s="43" t="str">
+        <x:v>Q4 FY2026 earnings call transcript</x:v>
+      </x:c>
+      <x:c r="E76" s="43" t="str">
+        <x:v>earnings_call_transcript</x:v>
+      </x:c>
+      <x:c r="F76" s="43" t="str">
+        <x:v>https://www.microsoft.com/en-us/Investor/events/FY-2026/earnings-fy-2026-q4</x:v>
+      </x:c>
+      <x:c r="G76" s="43" t="str">
+        <x:v>microsoft_azure; revenue_per_mw; token_economics; jevons; capex</x:v>
+      </x:c>
+      <x:c r="H76" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I76" s="43" t="str">
+        <x:v>Capacity, efficiency, capex, leases and outlook</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="19" t="str">
+        <x:v>SRC-MSFT-SEGMENT-8K-20260902</x:v>
+      </x:c>
+      <x:c r="B77" s="45" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="C77" s="19" t="str">
+        <x:v>Microsoft Corporation / SEC</x:v>
+      </x:c>
+      <x:c r="D77" s="43" t="str">
+        <x:v>FY2027 segment reporting change Form 8-K</x:v>
+      </x:c>
+      <x:c r="E77" s="43" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="F77" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/789019/000119312526380280/d291965d8k.htm</x:v>
+      </x:c>
+      <x:c r="G77" s="43" t="str">
+        <x:v>microsoft_azure; revenue_per_mw</x:v>
+      </x:c>
+      <x:c r="H77" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I77" s="43" t="str">
+        <x:v>Item 7.01 and Exhibit 99.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="19" t="str">
+        <x:v>SRC-MSFT-SEGMENT-EX99-20260902</x:v>
+      </x:c>
+      <x:c r="B78" s="45" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="C78" s="19" t="str">
+        <x:v>Microsoft Corporation / SEC</x:v>
+      </x:c>
+      <x:c r="D78" s="43" t="str">
+        <x:v>FY2027 segments and investor metrics</x:v>
+      </x:c>
+      <x:c r="E78" s="43" t="str">
+        <x:v>8-K_exhibit</x:v>
+      </x:c>
+      <x:c r="F78" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/789019/000119312526380280/d291965dex991.htm</x:v>
+      </x:c>
+      <x:c r="G78" s="43" t="str">
+        <x:v>microsoft_azure; revenue_per_mw</x:v>
+      </x:c>
+      <x:c r="H78" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I78" s="43" t="str">
+        <x:v>Slides 4-7, 11-13 and 17-18; exact restated Azure revenue and changed perimeter</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="19" t="str">
+        <x:v>SRC-MSFT-PUE-FY25</x:v>
+      </x:c>
+      <x:c r="B79" s="45" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="C79" s="19" t="str">
+        <x:v>Microsoft Corporation</x:v>
+      </x:c>
+      <x:c r="D79" s="43" t="str">
+        <x:v>Datacenter energy and water efficiency metrics</x:v>
+      </x:c>
+      <x:c r="E79" s="43" t="str">
+        <x:v>issuer_datacenter_efficiency_page</x:v>
+      </x:c>
+      <x:c r="F79" s="43" t="str">
+        <x:v>https://datacenters.microsoft.com/sustainability/efficiency/</x:v>
+      </x:c>
+      <x:c r="G79" s="43" t="str">
+        <x:v>microsoft_azure; effective_mw</x:v>
+      </x:c>
+      <x:c r="H79" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I79" s="43" t="str">
+        <x:v>FY2025 PUE 1.17; fully owned and controlled full-year sites only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="19" t="str">
+        <x:v>SRC-MSFT-ENV-DATA-FY25</x:v>
+      </x:c>
+      <x:c r="B80" s="45" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="C80" s="19" t="str">
+        <x:v>Microsoft Corporation</x:v>
+      </x:c>
+      <x:c r="D80" s="43" t="str">
+        <x:v>2026 Environmental Data Fact Sheet</x:v>
+      </x:c>
+      <x:c r="E80" s="43" t="str">
+        <x:v>environmental_data_fact_sheet</x:v>
+      </x:c>
+      <x:c r="F80" s="43" t="str">
+        <x:v>https://cdn-dynmedia-1.microsoft.com/is/content/microsoftcorp/microsoft/msc/documents/presentations/CSR/2026-Microsoft-Environmental-Data-Fact-Sheet-PDF.pdf</x:v>
+      </x:c>
+      <x:c r="G80" s="43" t="str">
+        <x:v>microsoft_azure; effective_mw</x:v>
+      </x:c>
+      <x:c r="H80" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I80" s="43" t="str">
+        <x:v>PDF pp.25-26 Table 15; 15,931,489 MWh listed facility electricity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="19" t="str">
+        <x:v>SRC-MSFT-OPENAI-20251028</x:v>
+      </x:c>
+      <x:c r="B81" s="45" t="n">
+        <x:v>45958</x:v>
+      </x:c>
+      <x:c r="C81" s="19" t="str">
+        <x:v>Microsoft Corporation</x:v>
+      </x:c>
+      <x:c r="D81" s="43" t="str">
+        <x:v>The next chapter of the Microsoft-OpenAI partnership</x:v>
+      </x:c>
+      <x:c r="E81" s="43" t="str">
+        <x:v>issuer_partnership_announcement</x:v>
+      </x:c>
+      <x:c r="F81" s="43" t="str">
+        <x:v>https://blogs.microsoft.com/blog/2025/10/28/the-next-chapter-of-the-microsoft-openai-partnership/</x:v>
+      </x:c>
+      <x:c r="G81" s="43" t="str">
+        <x:v>microsoft_azure; contract_economics; open_vs_proprietary</x:v>
+      </x:c>
+      <x:c r="H81" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I81" s="43" t="str">
+        <x:v>$250B incremental Azure commitment and partnership terms</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="19" t="str">
+        <x:v>SRC-MSFT-OPENAI-20260427</x:v>
+      </x:c>
+      <x:c r="B82" s="45" t="n">
+        <x:v>46139</x:v>
+      </x:c>
+      <x:c r="C82" s="19" t="str">
+        <x:v>Microsoft Corporation</x:v>
+      </x:c>
+      <x:c r="D82" s="43" t="str">
+        <x:v>The next phase of the Microsoft-OpenAI partnership</x:v>
+      </x:c>
+      <x:c r="E82" s="43" t="str">
+        <x:v>issuer_partnership_amendment</x:v>
+      </x:c>
+      <x:c r="F82" s="43" t="str">
+        <x:v>https://blogs.microsoft.com/blog/2026/04/27/the-next-phase-of-the-microsoft-openai-partnership/</x:v>
+      </x:c>
+      <x:c r="G82" s="43" t="str">
+        <x:v>microsoft_azure; contract_economics; open_vs_proprietary</x:v>
+      </x:c>
+      <x:c r="H82" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I82" s="43" t="str">
+        <x:v>Primary cloud multi-cloud revenue-share and IP terms amended</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="19" t="str">
+        <x:v>SRC-MSFT-POWER-20240920</x:v>
+      </x:c>
+      <x:c r="B83" s="45" t="n">
+        <x:v>45555</x:v>
+      </x:c>
+      <x:c r="C83" s="19" t="str">
+        <x:v>Microsoft Corporation</x:v>
+      </x:c>
+      <x:c r="D83" s="43" t="str">
+        <x:v>Accelerating the addition of carbon-free energy</x:v>
+      </x:c>
+      <x:c r="E83" s="43" t="str">
+        <x:v>issuer_power_procurement_update</x:v>
+      </x:c>
+      <x:c r="F83" s="43" t="str">
+        <x:v>https://www.microsoft.com/en-us/microsoft-cloud/blog/2024/09/20/accelerating-the-addition-of-carbon-free-energy-an-update-on-progress/</x:v>
+      </x:c>
+      <x:c r="G83" s="43" t="str">
+        <x:v>microsoft_azure; contract_economics; power_to_silicon</x:v>
+      </x:c>
+      <x:c r="H83" s="43" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I83" s="43" t="str">
+        <x:v>Constellation, Brookfield and Powerex arrangements; generation MW kept separate from IT MW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="20" t="str">
+        <x:v>SRC-CEG-MSFT-PPA-20240920</x:v>
+      </x:c>
+      <x:c r="B84" s="46" t="n">
+        <x:v>45555</x:v>
+      </x:c>
+      <x:c r="C84" s="20" t="str">
+        <x:v>Constellation Energy</x:v>
+      </x:c>
+      <x:c r="D84" s="44" t="str">
+        <x:v>Constellation to launch Crane Clean Energy Center</x:v>
+      </x:c>
+      <x:c r="E84" s="44" t="str">
+        <x:v>counterparty_PPA_announcement</x:v>
+      </x:c>
+      <x:c r="F84" s="44" t="str">
+        <x:v>https://www.constellationenergy.com/news/2024/Constellation-to-Launch-Crane-Clean-Energy-Center-Restoring-Jobs-and-Carbon-Free-Power-to-The-Grid.html</x:v>
+      </x:c>
+      <x:c r="G84" s="44" t="str">
+        <x:v>microsoft_azure; contract_economics; power_to_silicon</x:v>
+      </x:c>
+      <x:c r="H84" s="44" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="I84" s="44" t="str">
+        <x:v>20-year PPA; approximately 835 MW to grid; expected online 2028; price undisclosed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a268069d5204e9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbde42e9552cf4c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research AWS AI compute economics and delivery-conditioned funding
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R76bb637026234fd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Ra8ad98f090cb493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R415180b483ba4a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rad79a6c57b8a471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R27e42596888f4373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Re24f3fea3b7d46c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rd877d39413264515"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2c3d27ddadb247e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rdac7c49ef1e24c14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R3f7a032154684d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Ra2df288a6c7f4c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Rec5a298ddf6444d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R2d534c5bbce24b0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rc5bbbbbdad4e448c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -788,7 +788,7 @@
       </x:c>
       <x:c r="D14" s="19" t="str">
         <x:f>'Company Models'!N6</x:f>
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E14" s="58" t="str">
         <x:f>IF('Company Models'!S6="","",'Company Models'!S6)</x:f>
@@ -1349,10 +1349,14 @@
         <x:v>SEGMENT-AWS</x:v>
       </x:c>
       <x:c r="C6" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D6" s="27"/>
-      <x:c r="E6" s="29"/>
+        <x:v>Q2 2026</x:v>
+      </x:c>
+      <x:c r="D6" s="27" t="n">
+        <x:v>42232000000</x:v>
+      </x:c>
+      <x:c r="E6" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F6" s="31"/>
       <x:c r="G6" s="33"/>
       <x:c r="H6" s="23"/>
@@ -1361,13 +1365,13 @@
       <x:c r="K6" s="35"/>
       <x:c r="L6" s="35"/>
       <x:c r="M6" s="19" t="str">
-        <x:v>SRC-CHAT-001</x:v>
+        <x:v>SRC-AMZN-10Q-Q2FY26</x:v>
       </x:c>
       <x:c r="N6" s="19" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O6" s="43" t="str">
-        <x:v>Needs matching AI revenue attribution and average AI IT MW</x:v>
+        <x:v>AWS all services; AI/chips run rates overlap and are not Q2 AI revenue. Active AI IT MW and utilization missing. 2025 PUE 1.14 is historical only.</x:v>
       </x:c>
       <x:c r="P6" s="37" t="str">
         <x:f>IF(OR(D6="",E6="",F6=""),"",D6*E6*F6)</x:f>
@@ -2164,16 +2168,16 @@
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D6" s="43" t="str">
-        <x:v>Annualized AWS revenue attributable to AI compute</x:v>
+        <x:v>Annualized recognized external AWS AI compute revenue</x:v>
       </x:c>
       <x:c r="E6" s="43" t="str">
-        <x:v>Average effective utilized AWS AI IT MW</x:v>
+        <x:v>Time-weighted active AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F6" s="43" t="str">
-        <x:v>Separate Trainium Inferentia and third-party GPU workloads</x:v>
+        <x:v>Separate Trainium Inferentia and NVIDIA; exclude internal/noncompute revenue and run-rate overlap; PUE only for matched facility-power conversion</x:v>
       </x:c>
       <x:c r="G6" s="43" t="str">
-        <x:v>Configured; inputs open</x:v>
+        <x:v>Partial 2026-09-19; matched numerator and denominator open</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2478,7 +2482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c6a903f4b0e4e00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0aa8876f84bd4484"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3102,7 +3106,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0714630b43aa4eeb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R875f3743166b4772"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5860,38 +5864,465 @@
       </x:c>
     </x:row>
     <x:row r="84">
-      <x:c r="A84" s="20" t="str">
+      <x:c r="A84" s="19" t="str">
         <x:v>SRC-CEG-MSFT-PPA-20240920</x:v>
       </x:c>
-      <x:c r="B84" s="46" t="n">
+      <x:c r="B84" s="45" t="n">
         <x:v>45555</x:v>
       </x:c>
-      <x:c r="C84" s="20" t="str">
+      <x:c r="C84" s="19" t="str">
         <x:v>Constellation Energy</x:v>
       </x:c>
-      <x:c r="D84" s="44" t="str">
+      <x:c r="D84" s="43" t="str">
         <x:v>Constellation to launch Crane Clean Energy Center</x:v>
       </x:c>
-      <x:c r="E84" s="44" t="str">
+      <x:c r="E84" s="43" t="str">
         <x:v>counterparty_PPA_announcement</x:v>
       </x:c>
-      <x:c r="F84" s="44" t="str">
+      <x:c r="F84" s="43" t="str">
         <x:v>https://www.constellationenergy.com/news/2024/Constellation-to-Launch-Crane-Clean-Energy-Center-Restoring-Jobs-and-Carbon-Free-Power-to-The-Grid.html</x:v>
       </x:c>
-      <x:c r="G84" s="44" t="str">
+      <x:c r="G84" s="43" t="str">
         <x:v>microsoft_azure; contract_economics; power_to_silicon</x:v>
       </x:c>
-      <x:c r="H84" s="44" t="str">
+      <x:c r="H84" s="43" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="I84" s="44" t="str">
+      <x:c r="I84" s="43" t="str">
         <x:v>20-year PPA; approximately 835 MW to grid; expected online 2028; price undisclosed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="19" t="str">
+        <x:v>SRC-AMZN-10K-FY25</x:v>
+      </x:c>
+      <x:c r="B85" s="45" t="n">
+        <x:v>46059</x:v>
+      </x:c>
+      <x:c r="C85" s="19" t="str">
+        <x:v>Amazon / SEC</x:v>
+      </x:c>
+      <x:c r="D85" s="43" t="str">
+        <x:v>FY2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E85" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F85" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1018724/000101872426000004/amzn-20251231.htm</x:v>
+      </x:c>
+      <x:c r="G85" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H85" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I85" s="43" t="str">
+        <x:v>Note 1 pp.41,47: estimates and property/equipment lives; Note 2 investments; Note 10 segment tables. Period: 2025-01-01/2025-12-31. Publication: 2026-02-06.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="19" t="str">
+        <x:v>SRC-AMZN-10Q-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B86" s="45" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="C86" s="19" t="str">
+        <x:v>Amazon / SEC</x:v>
+      </x:c>
+      <x:c r="D86" s="43" t="str">
+        <x:v>Q2 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E86" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F86" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1018724/000101872426000026/amzn-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G86" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H86" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I86" s="43" t="str">
+        <x:v>Note 1 pp.8-10 energy derivatives/unearned revenue; Note 2 pp.11-13 investments/VIE; Note 3 pp.13-14; Note 4 p.15 commitments; Note 5 pp.17-18 debt; Note 8 p.23 segment results; MD&amp;A p.30 pricing; Item 6 p.51 exhibits. Period: 2026-04-01/2026-06-30; H1 and subsequent events. Publication: 2026-07-31.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="19" t="str">
+        <x:v>SRC-AMZN-Q2FY26-ER</x:v>
+      </x:c>
+      <x:c r="B87" s="45" t="n">
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="C87" s="19" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="D87" s="43" t="str">
+        <x:v>Q2 2026 earnings release</x:v>
+      </x:c>
+      <x:c r="E87" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F87" s="43" t="str">
+        <x:v>https://ir.aboutamazon.com/news-release/news-release-details/2026/Amazon-com-Announces-Second-Quarter-Results/default.aspx</x:v>
+      </x:c>
+      <x:c r="G87" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H87" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I87" s="43" t="str">
+        <x:v>Opening results; Jassy quotation; AI/chips highlights; cash-flow tables. Period: Q2 2026. Publication: 2026-07-30.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="19" t="str">
+        <x:v>SRC-AMZN-Q2FY26-REMARKS</x:v>
+      </x:c>
+      <x:c r="B88" s="45"/>
+      <x:c r="C88" s="19" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="D88" s="43" t="str">
+        <x:v>CEO Q2 earnings remarks excerpt</x:v>
+      </x:c>
+      <x:c r="E88" s="43" t="str">
+        <x:v>issuer_earnings_remarks</x:v>
+      </x:c>
+      <x:c r="F88" s="43" t="str">
+        <x:v>https://www.aboutamazon.com/news/company-news/amazon-ceo-andy-jassy-aws-revenue-growth-q2-2026-earnings</x:v>
+      </x:c>
+      <x:c r="G88" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H88" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I88" s="43" t="str">
+        <x:v>Opening AWS, Chips and AI run-rate paragraphs; core-services and model-training discussion. Period: Q2 2026. Publication: not verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="19" t="str">
+        <x:v>SRC-AWS-PUE-FY25</x:v>
+      </x:c>
+      <x:c r="B89" s="45"/>
+      <x:c r="C89" s="19" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="D89" s="43" t="str">
+        <x:v>AWS 2025 Sustainability Summary</x:v>
+      </x:c>
+      <x:c r="E89" s="43" t="str">
+        <x:v>sustainability_report</x:v>
+      </x:c>
+      <x:c r="F89" s="43" t="str">
+        <x:v>https://sustainability.aboutamazon.com/2025-aws-summary.pdf</x:v>
+      </x:c>
+      <x:c r="G89" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H89" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I89" s="43" t="str">
+        <x:v>p.6 Climate and Energy PUE; p.15 endnote 2. Period: 2025-01-01/2025-12-31. Publication: not verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="19" t="str">
+        <x:v>SRC-AWS-PUE-REGIONS</x:v>
+      </x:c>
+      <x:c r="B90" s="45"/>
+      <x:c r="C90" s="19" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="D90" s="43" t="str">
+        <x:v>AWS regional PUE and WUE table</x:v>
+      </x:c>
+      <x:c r="E90" s="43" t="str">
+        <x:v>issuer_energy_disclosure</x:v>
+      </x:c>
+      <x:c r="F90" s="43" t="str">
+        <x:v>https://sustainability.aboutamazon.com/products-services/aws-cloud</x:v>
+      </x:c>
+      <x:c r="G90" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H90" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I90" s="43" t="str">
+        <x:v>Power usage effectiveness; coverage paragraph; AWS PUE and WUE and AWS Region PUE and WUE tables. Period: Calendar 2025 and historical comparisons. Publication: not verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="19" t="str">
+        <x:v>SRC-AWS-PUE-METHOD</x:v>
+      </x:c>
+      <x:c r="B91" s="45" t="n">
+        <x:v>45629</x:v>
+      </x:c>
+      <x:c r="C91" s="19" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="D91" s="43" t="str">
+        <x:v>AWS PUE methodology</x:v>
+      </x:c>
+      <x:c r="E91" s="43" t="str">
+        <x:v>methodology</x:v>
+      </x:c>
+      <x:c r="F91" s="43" t="str">
+        <x:v>https://sustainability.aboutamazon.com/pue-methodology.pdf</x:v>
+      </x:c>
+      <x:c r="G91" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H91" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I91" s="43" t="str">
+        <x:v>p.2 ratio definition, intermediate metering, one-minute measurement and trailing-twelve-month reporting. Period: Methodology updated 2024-12-03. Publication: 2024-12-03.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="19" t="str">
+        <x:v>SRC-AMZN-ANTHROPIC-20260420</x:v>
+      </x:c>
+      <x:c r="B92" s="45" t="n">
+        <x:v>46132</x:v>
+      </x:c>
+      <x:c r="C92" s="19" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="D92" s="43" t="str">
+        <x:v>Expanded Anthropic strategic collaboration</x:v>
+      </x:c>
+      <x:c r="E92" s="43" t="str">
+        <x:v>issuer_deal_announcement</x:v>
+      </x:c>
+      <x:c r="F92" s="43" t="str">
+        <x:v>https://www.aboutamazon.com/news/company-news/amazon-invests-additional-5-billion-anthropic-ai</x:v>
+      </x:c>
+      <x:c r="G92" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H92" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I92" s="43" t="str">
+        <x:v>Opening commitment/capacity paragraphs; investment milestone paragraph; Trainium2/3/4 and Graviton scope. Period: Agreement announced 2026-04-20. Publication: 2026-04-20.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="19" t="str">
+        <x:v>SRC-ANTHROPIC-AWS-20260420</x:v>
+      </x:c>
+      <x:c r="B93" s="45" t="n">
+        <x:v>46132</x:v>
+      </x:c>
+      <x:c r="C93" s="19" t="str">
+        <x:v>Anthropic</x:v>
+      </x:c>
+      <x:c r="D93" s="43" t="str">
+        <x:v>Up to 5 GW expanded Amazon collaboration</x:v>
+      </x:c>
+      <x:c r="E93" s="43" t="str">
+        <x:v>counterparty_deal_announcement</x:v>
+      </x:c>
+      <x:c r="F93" s="43" t="str">
+        <x:v>https://www.anthropic.com/news/anthropic-amazon-compute</x:v>
+      </x:c>
+      <x:c r="G93" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H93" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I93" s="43" t="str">
+        <x:v>Opening capacity paragraph; Infrastructure at scale; Meeting record demand; timing to year-end 2026. Period: Announced 2026-04-20; clarified 2026-04-21. Publication: 2026-04-20.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="19" t="str">
+        <x:v>SRC-AMZN-OPENAI-20260227</x:v>
+      </x:c>
+      <x:c r="B94" s="45" t="n">
+        <x:v>46080</x:v>
+      </x:c>
+      <x:c r="C94" s="19" t="str">
+        <x:v>Amazon / OpenAI</x:v>
+      </x:c>
+      <x:c r="D94" s="43" t="str">
+        <x:v>OpenAI and Amazon strategic partnership</x:v>
+      </x:c>
+      <x:c r="E94" s="43" t="str">
+        <x:v>issuer_deal_announcement</x:v>
+      </x:c>
+      <x:c r="F94" s="43" t="str">
+        <x:v>https://press.aboutamazon.com/2026/2/openai-and-amazon-announce-strategic-partnership</x:v>
+      </x:c>
+      <x:c r="G94" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H94" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I94" s="43" t="str">
+        <x:v>Opening investment paragraph; OpenAI to use Trainium compute section. Period: 8-year expansion; Trainium4 expected 2027. Publication: 2026-02-27.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="19" t="str">
+        <x:v>SRC-AMZN-TERMLOAN-20260610</x:v>
+      </x:c>
+      <x:c r="B95" s="45" t="n">
+        <x:v>46183</x:v>
+      </x:c>
+      <x:c r="C95" s="19" t="str">
+        <x:v>Amazon / SEC</x:v>
+      </x:c>
+      <x:c r="D95" s="43" t="str">
+        <x:v>June 8 term loan agreement</x:v>
+      </x:c>
+      <x:c r="E95" s="43" t="str">
+        <x:v>8-K_Exhibit_10.1</x:v>
+      </x:c>
+      <x:c r="F95" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1018724/000110465926072140/tm2613616d4_ex10-1.htm</x:v>
+      </x:c>
+      <x:c r="G95" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H95" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I95" s="43" t="str">
+        <x:v>Section 1.01 Applicable Rate p.2 and Commitment Termination Date p.7; Article II loans. Period: Agreement 2026-06-08; draw deadline 2026-09-30. Publication: 2026-06-10.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="19" t="str">
+        <x:v>SRC-AMZN-REVOLVER364-20260731</x:v>
+      </x:c>
+      <x:c r="B96" s="45" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="C96" s="19" t="str">
+        <x:v>Amazon / SEC</x:v>
+      </x:c>
+      <x:c r="D96" s="43" t="str">
+        <x:v>364-day credit agreement amendment</x:v>
+      </x:c>
+      <x:c r="E96" s="43" t="str">
+        <x:v>10-Q_Exhibit_10.2</x:v>
+      </x:c>
+      <x:c r="F96" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1018724/000101872426000026/amzn-20260630xex102.htm</x:v>
+      </x:c>
+      <x:c r="G96" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H96" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I96" s="43" t="str">
+        <x:v>First Amendment sections 1-3 and Exhibit A. Period: Amendment 2026-06-08. Publication: 2026-07-31.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="19" t="str">
+        <x:v>SRC-AMZN-REVOLVER5Y-20260731</x:v>
+      </x:c>
+      <x:c r="B97" s="45" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="C97" s="19" t="str">
+        <x:v>Amazon / SEC</x:v>
+      </x:c>
+      <x:c r="D97" s="43" t="str">
+        <x:v>Five-year credit agreement amendment</x:v>
+      </x:c>
+      <x:c r="E97" s="43" t="str">
+        <x:v>10-Q_Exhibit_10.3</x:v>
+      </x:c>
+      <x:c r="F97" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1018724/000101872426000026/amzn-20260630xex103.htm</x:v>
+      </x:c>
+      <x:c r="G97" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H97" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I97" s="43" t="str">
+        <x:v>First Amendment sections 1-3 and Exhibit A. Period: Amendment 2026-06-08. Publication: 2026-07-31.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="19" t="str">
+        <x:v>SRC-TALEN-AWS-PPA-20250611</x:v>
+      </x:c>
+      <x:c r="B98" s="45" t="n">
+        <x:v>45819</x:v>
+      </x:c>
+      <x:c r="C98" s="19" t="str">
+        <x:v>Talen / SEC</x:v>
+      </x:c>
+      <x:c r="D98" s="43" t="str">
+        <x:v>Expanded Susquehanna AWS PPA</x:v>
+      </x:c>
+      <x:c r="E98" s="43" t="str">
+        <x:v>8-K_Exhibit_99.1</x:v>
+      </x:c>
+      <x:c r="F98" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1622536/000162828025030559/a20250611pressreleasebusin.htm</x:v>
+      </x:c>
+      <x:c r="G98" s="43" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H98" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I98" s="43" t="str">
+        <x:v>Opening capacity/term/ramp paragraphs; front-of-meter transition paragraph. Period: Announced 2025-06-11; through 2042. Publication: 2025-06-11.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="20" t="str">
+        <x:v>SRC-AMZN-FILING-INDEX-20260919</x:v>
+      </x:c>
+      <x:c r="B99" s="46"/>
+      <x:c r="C99" s="20" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D99" s="44" t="str">
+        <x:v>Amazon filing index freshness check</x:v>
+      </x:c>
+      <x:c r="E99" s="44" t="str">
+        <x:v>filing_index</x:v>
+      </x:c>
+      <x:c r="F99" s="44" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=1018724</x:v>
+      </x:c>
+      <x:c r="G99" s="44" t="str">
+        <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H99" s="44" t="str">
+        <x:v>index_checked</x:v>
+      </x:c>
+      <x:c r="I99" s="44" t="str">
+        <x:v>Search-index rendered selected filings: latest annual February 6; quarterly July 31; September 9 items. Period: As checked 2026-09-19. Publication: not verified.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbde42e9552cf4c93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56a667ec19964cd9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research Google Cloud AI compute economics
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2c3d27ddadb247e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rdac7c49ef1e24c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R3f7a032154684d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Ra2df288a6c7f4c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Rec5a298ddf6444d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R2d534c5bbce24b0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rc5bbbbbdad4e448c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c5332af934946a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rda03f4208688419f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R632c3c6ea1ae455b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rd65145f55fdb46b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R765b40eacb144943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R124371ed8b514f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R9a18a82c5182495b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +362,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I109" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -813,7 +813,7 @@
       </x:c>
       <x:c r="D15" s="19" t="str">
         <x:f>'Company Models'!N7</x:f>
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E15" s="58" t="str">
         <x:f>IF('Company Models'!S7="","",'Company Models'!S7)</x:f>
@@ -1398,10 +1398,14 @@
         <x:v>SEGMENT-GCP</x:v>
       </x:c>
       <x:c r="C7" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D7" s="27"/>
-      <x:c r="E7" s="29"/>
+        <x:v>Q2 2026</x:v>
+      </x:c>
+      <x:c r="D7" s="27" t="n">
+        <x:v>24768000000</x:v>
+      </x:c>
+      <x:c r="E7" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F7" s="31"/>
       <x:c r="G7" s="33"/>
       <x:c r="H7" s="23"/>
@@ -1410,13 +1414,13 @@
       <x:c r="K7" s="35"/>
       <x:c r="L7" s="35"/>
       <x:c r="M7" s="19" t="str">
-        <x:v>SRC-CHAT-001</x:v>
+        <x:v>SRC-GOOG-10Q-Q2FY26</x:v>
       </x:c>
       <x:c r="N7" s="19" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O7" s="43" t="str">
-        <x:v>Needs external GCP AI numerator separate from internal TPU use</x:v>
+        <x:v>Google Cloud includes GCP, Workspace, security/data services and newly recognized TPU system sales. External AI-compute attribution, period-average active external AI IT MW, physical utilization and matched GCP-only PUE remain missing. Fleet TTM PUE 1.09 is a proxy only.</x:v>
       </x:c>
       <x:c r="P7" s="37" t="str">
         <x:f>IF(OR(D7="",E7="",F7=""),"",D7*E7*F7)</x:f>
@@ -2191,16 +2195,16 @@
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D7" s="43" t="str">
-        <x:v>Annualized Google Cloud revenue attributable to AI compute</x:v>
+        <x:v>Annualized recognized external GCP AI compute service revenue</x:v>
       </x:c>
       <x:c r="E7" s="43" t="str">
-        <x:v>Average effective utilized GCP AI IT MW</x:v>
+        <x:v>Time-weighted active external GCP AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F7" s="43" t="str">
-        <x:v>Separate internal Search and YouTube from external GCP; TPU ownership</x:v>
+        <x:v>Exclude Workspace, security/data/non-AI services, internal Search/YouTube/Gemini, TPU system sales and backlog; separate TPU/GPU/third-party capacity cohorts; PUE only for matched facility-power conversion</x:v>
       </x:c>
       <x:c r="G7" s="43" t="str">
-        <x:v>Configured; inputs open</x:v>
+        <x:v>Partial 2026-09-20; exact Cloud revenue and fleet PUE established; AI attribution and effective-MW denominator open</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2482,7 +2486,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0aa8876f84bd4484"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd758a829b4344474"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3106,7 +3110,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R875f3743166b4772"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb62e90fc3bce4a3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6293,36 +6297,320 @@
       </x:c>
     </x:row>
     <x:row r="99">
-      <x:c r="A99" s="20" t="str">
+      <x:c r="A99" s="19" t="str">
         <x:v>SRC-AMZN-FILING-INDEX-20260919</x:v>
       </x:c>
-      <x:c r="B99" s="46"/>
-      <x:c r="C99" s="20" t="str">
+      <x:c r="B99" s="45"/>
+      <x:c r="C99" s="19" t="str">
         <x:v>SEC</x:v>
       </x:c>
-      <x:c r="D99" s="44" t="str">
+      <x:c r="D99" s="43" t="str">
         <x:v>Amazon filing index freshness check</x:v>
       </x:c>
-      <x:c r="E99" s="44" t="str">
+      <x:c r="E99" s="43" t="str">
         <x:v>filing_index</x:v>
       </x:c>
-      <x:c r="F99" s="44" t="str">
+      <x:c r="F99" s="43" t="str">
         <x:v>https://www.sec.gov/edgar/browse/?CIK=1018724</x:v>
       </x:c>
-      <x:c r="G99" s="44" t="str">
+      <x:c r="G99" s="43" t="str">
         <x:v>amazon_aws;revenue_per_mw;contract_economics</x:v>
       </x:c>
-      <x:c r="H99" s="44" t="str">
+      <x:c r="H99" s="43" t="str">
         <x:v>index_checked</x:v>
       </x:c>
-      <x:c r="I99" s="44" t="str">
+      <x:c r="I99" s="43" t="str">
         <x:v>Search-index rendered selected filings: latest annual February 6; quarterly July 31; September 9 items. Period: As checked 2026-09-19. Publication: not verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="19" t="str">
+        <x:v>SRC-GOOG-10K-FY25</x:v>
+      </x:c>
+      <x:c r="B100" s="45" t="n">
+        <x:v>46058</x:v>
+      </x:c>
+      <x:c r="C100" s="19" t="str">
+        <x:v>Alphabet Inc. / SEC</x:v>
+      </x:c>
+      <x:c r="D100" s="43" t="str">
+        <x:v>FY2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E100" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F100" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1652044/000165204426000018/goog-20251231.htm</x:v>
+      </x:c>
+      <x:c r="G100" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H100" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I100" s="43" t="str">
+        <x:v>Item 7 pp.28-40; revenue backlog p.56; commitments pp.37-39; Note 15 pp.86-88. Period FY2025.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="19" t="str">
+        <x:v>SRC-GOOG-10Q-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B101" s="45" t="n">
+        <x:v>46226</x:v>
+      </x:c>
+      <x:c r="C101" s="19" t="str">
+        <x:v>Alphabet Inc. / SEC</x:v>
+      </x:c>
+      <x:c r="D101" s="43" t="str">
+        <x:v>Q2 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E101" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F101" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1652044/000165204426000071/goog-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G101" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H101" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I101" s="43" t="str">
+        <x:v>Notes 2, 4-6, 8, 10 and 15; MD&amp;A pp.43-54. Period Q2/H1 2026.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="19" t="str">
+        <x:v>SRC-GOOG-Q2FY26-ER</x:v>
+      </x:c>
+      <x:c r="B102" s="45" t="n">
+        <x:v>46225</x:v>
+      </x:c>
+      <x:c r="C102" s="19" t="str">
+        <x:v>Alphabet Inc. / SEC</x:v>
+      </x:c>
+      <x:c r="D102" s="43" t="str">
+        <x:v>Alphabet Announces Second Quarter 2026 Results</x:v>
+      </x:c>
+      <x:c r="E102" s="43" t="str">
+        <x:v>8-K_Exhibit_99.1</x:v>
+      </x:c>
+      <x:c r="F102" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1652044/000165204426000066/googexhibit991q22026.htm</x:v>
+      </x:c>
+      <x:c r="G102" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;capex</x:v>
+      </x:c>
+      <x:c r="H102" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I102" s="43" t="str">
+        <x:v>Operating highlights; segment and cash-flow tables</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="19" t="str">
+        <x:v>SRC-GOOG-Q2FY26-CALL</x:v>
+      </x:c>
+      <x:c r="B103" s="45" t="n">
+        <x:v>46225</x:v>
+      </x:c>
+      <x:c r="C103" s="19" t="str">
+        <x:v>Alphabet Inc.</x:v>
+      </x:c>
+      <x:c r="D103" s="43" t="str">
+        <x:v>Q2 2026 earnings call transcript</x:v>
+      </x:c>
+      <x:c r="E103" s="43" t="str">
+        <x:v>issuer_earnings_call_transcript</x:v>
+      </x:c>
+      <x:c r="F103" s="43" t="str">
+        <x:v>https://abc.xyz/investor/events/event-details/2026/2026-Q2-Earnings-Call-2026-GgTAq7Is0z/default.aspx</x:v>
+      </x:c>
+      <x:c r="G103" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H103" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I103" s="43" t="str">
+        <x:v>Cloud, backlog, TPU system sales, third-party capacity, capex, energy and capital structure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="19" t="str">
+        <x:v>SRC-GOOG-PUE-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B104" s="45"/>
+      <x:c r="C104" s="19" t="str">
+        <x:v>Google</x:v>
+      </x:c>
+      <x:c r="D104" s="43" t="str">
+        <x:v>Power usage effectiveness</x:v>
+      </x:c>
+      <x:c r="E104" s="43" t="str">
+        <x:v>issuer_datacenter_efficiency_page</x:v>
+      </x:c>
+      <x:c r="F104" s="43" t="str">
+        <x:v>https://datacenters.google/efficiency/</x:v>
+      </x:c>
+      <x:c r="G104" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;effective_mw</x:v>
+      </x:c>
+      <x:c r="H104" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I104" s="43" t="str">
+        <x:v>Q2 2026 quarterly fleet PUE 1.10 and TTM PUE 1.09; dynamic publication date not shown</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="19" t="str">
+        <x:v>SRC-GOOG-TPU-PRICING-20260920</x:v>
+      </x:c>
+      <x:c r="B105" s="45"/>
+      <x:c r="C105" s="19" t="str">
+        <x:v>Google Cloud</x:v>
+      </x:c>
+      <x:c r="D105" s="43" t="str">
+        <x:v>Cloud TPU pricing</x:v>
+      </x:c>
+      <x:c r="E105" s="43" t="str">
+        <x:v>issuer_pricing_page</x:v>
+      </x:c>
+      <x:c r="F105" s="43" t="str">
+        <x:v>https://cloud.google.com/tpu/pricing</x:v>
+      </x:c>
+      <x:c r="G105" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H105" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I105" s="43" t="str">
+        <x:v>Ironwood and Trillium per-chip-hour list prices as retrieved 2026-09-20; realized price and system power missing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="19" t="str">
+        <x:v>SRC-GOOG-TPU7X-20260920</x:v>
+      </x:c>
+      <x:c r="B106" s="45"/>
+      <x:c r="C106" s="19" t="str">
+        <x:v>Google Cloud</x:v>
+      </x:c>
+      <x:c r="D106" s="43" t="str">
+        <x:v>TPU7x Ironwood architecture</x:v>
+      </x:c>
+      <x:c r="E106" s="43" t="str">
+        <x:v>issuer_technical_documentation</x:v>
+      </x:c>
+      <x:c r="F106" s="43" t="str">
+        <x:v>https://docs.cloud.google.com/tpu/docs/tpu7x</x:v>
+      </x:c>
+      <x:c r="G106" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;power_to_silicon</x:v>
+      </x:c>
+      <x:c r="H106" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I106" s="43" t="str">
+        <x:v>9,216-chip pod and four-chip VM architecture; full-system electrical power not disclosed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="19" t="str">
+        <x:v>SRC-BX-GOOG-TPUJV-20260518</x:v>
+      </x:c>
+      <x:c r="B107" s="45" t="n">
+        <x:v>46160</x:v>
+      </x:c>
+      <x:c r="C107" s="19" t="str">
+        <x:v>Blackstone</x:v>
+      </x:c>
+      <x:c r="D107" s="43" t="str">
+        <x:v>Blackstone Announces Joint Venture with Google to Create New TPU Cloud</x:v>
+      </x:c>
+      <x:c r="E107" s="43" t="str">
+        <x:v>counterparty_deal_announcement</x:v>
+      </x:c>
+      <x:c r="F107" s="43" t="str">
+        <x:v>https://www.blackstone.com/news/press/blackstone-announces-joint-venture-with-google-to-create-new-tpu-cloud/</x:v>
+      </x:c>
+      <x:c r="G107" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H107" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I107" s="43" t="str">
+        <x:v>$5B initial Blackstone equity commitment; first 500 MW expected 2027; Google supplies TPU hardware/software/services</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="19" t="str">
+        <x:v>SRC-SPX-GOOG-COMPUTE-20260605</x:v>
+      </x:c>
+      <x:c r="B108" s="45" t="n">
+        <x:v>46178</x:v>
+      </x:c>
+      <x:c r="C108" s="19" t="str">
+        <x:v>SpaceX / SEC</x:v>
+      </x:c>
+      <x:c r="D108" s="43" t="str">
+        <x:v>Google Cloud Service Agreement summary</x:v>
+      </x:c>
+      <x:c r="E108" s="43" t="str">
+        <x:v>free_writing_prospectus</x:v>
+      </x:c>
+      <x:c r="F108" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1181412/000162828026041150/spacexagreementfwp.htm</x:v>
+      </x:c>
+      <x:c r="G108" s="43" t="str">
+        <x:v>alphabet_gcp;revenue_per_mw;contract_economics</x:v>
+      </x:c>
+      <x:c r="H108" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I108" s="43" t="str">
+        <x:v>$920M monthly for approximately 110000 GPUs plus systems; delivery and termination terms</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="20" t="str">
+        <x:v>SRC-GOOG-EQUITY-RAISE-20260604</x:v>
+      </x:c>
+      <x:c r="B109" s="46" t="n">
+        <x:v>46177</x:v>
+      </x:c>
+      <x:c r="C109" s="20" t="str">
+        <x:v>Alphabet Inc. / SEC</x:v>
+      </x:c>
+      <x:c r="D109" s="44" t="str">
+        <x:v>AI infrastructure equity capital raise</x:v>
+      </x:c>
+      <x:c r="E109" s="44" t="str">
+        <x:v>8-K_Exhibit_99.1</x:v>
+      </x:c>
+      <x:c r="F109" s="44" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1652044/000119312526257724/d83560dex991.htm</x:v>
+      </x:c>
+      <x:c r="G109" s="44" t="str">
+        <x:v>alphabet_gcp;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H109" s="44" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I109" s="44" t="str">
+        <x:v>Offering composition and AI infrastructure use of proceeds</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56a667ec19964cd9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f35b190f22441b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add Meta MW economics review for 2026-10-04
Record primary-source findings, PUE and revenue attribution gaps, project financing and guarantees. Update atomic records, company projections, rebuilt workbook, and research queue together.
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c5332af934946a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rda03f4208688419f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R632c3c6ea1ae455b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rd65145f55fdb46b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R765b40eacb144943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R124371ed8b514f5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R9a18a82c5182495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R74013eab31504457"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rafd8e37b884d4358"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R5339e32857864bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rff1eec694f974d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Rd482aa08cfe84752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rd37ab03e5c55436e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rf3b1e00ecd2b4b68"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,19 +100,32 @@
     </x:fill>
   </x:fills>
   <x:borders count="6">
-    <x:border/>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FF23415C"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
+      <x:top/>
       <x:bottom style="medium">
         <x:color rgb="FF23415C"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -121,22 +134,31 @@
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
+      <x:top/>
       <x:bottom style="medium">
         <x:color rgb="FF23415C"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:left>
+      <x:right/>
+      <x:top/>
       <x:bottom style="medium">
         <x:color rgb="FF23415C"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9E1E8"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
@@ -345,7 +367,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TokenEconomicsTable" displayName="TokenEconomicsTable" ref="A4:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TokenEconomicsTable" displayName="TokenEconomicsTable" ref="A4:I32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Dataset"/>
@@ -362,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I109" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -838,7 +860,7 @@
       </x:c>
       <x:c r="D16" s="19" t="str">
         <x:f>'Company Models'!N8</x:f>
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E16" s="58" t="str">
         <x:f>IF('Company Models'!S8="","",'Company Models'!S8)</x:f>
@@ -1447,10 +1469,14 @@
         <x:v>INTERNAL-META</x:v>
       </x:c>
       <x:c r="C8" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D8" s="27"/>
-      <x:c r="E8" s="29"/>
+        <x:v>Q2 2026</x:v>
+      </x:c>
+      <x:c r="D8" s="27" t="n">
+        <x:v>60801000000</x:v>
+      </x:c>
+      <x:c r="E8" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F8" s="31"/>
       <x:c r="G8" s="33"/>
       <x:c r="H8" s="23"/>
@@ -1459,13 +1485,13 @@
       <x:c r="K8" s="35"/>
       <x:c r="L8" s="35"/>
       <x:c r="M8" s="19" t="str">
-        <x:v>SRC-CHAT-001</x:v>
+        <x:v>SRC-META-10Q-Q2FY26</x:v>
       </x:c>
       <x:c r="N8" s="19" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O8" s="43" t="str">
-        <x:v>Needs incremental monetization bridge; total ad revenue prohibited</x:v>
+        <x:v>Total revenue is a diagnostic only and excluded from the numerator. Incremental AI-attributed value, recognized external Meta Compute revenue, period-average active AI IT MW, physical utilization and matched AI PUE are missing. FY2024 fleet PUE 1.08 is historical context only.</x:v>
       </x:c>
       <x:c r="P8" s="37" t="str">
         <x:f>IF(OR(D8="",E8="",F8=""),"",D8*E8*F8)</x:f>
@@ -2218,16 +2244,16 @@
         <x:v>Internal compute</x:v>
       </x:c>
       <x:c r="D8" s="43" t="str">
-        <x:v>Incremental ad or engagement revenue plus external Meta Compute revenue attributable to AI</x:v>
+        <x:v>Annualized incremental recognized internal AI value plus recognized external Meta Compute revenue</x:v>
       </x:c>
       <x:c r="E8" s="43" t="str">
-        <x:v>Average effective utilized Meta AI IT MW</x:v>
+        <x:v>Time-weighted average active Meta AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F8" s="43" t="str">
-        <x:v>Never use total advertising revenue; keep internal and external cases separate</x:v>
+        <x:v>Never use total company or advertising revenue; keep internal and external cases separate; use matched PUE only for facility-to-IT conversion</x:v>
       </x:c>
       <x:c r="G8" s="43" t="str">
-        <x:v>Configured; inputs open</x:v>
+        <x:v>Partial 2026-10-04; AI attribution active IT MW utilization and matched PUE open</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2486,7 +2512,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd758a829b4344474"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36ef155607784bbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2586,8 +2612,8 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="45" t="n">
-        <x:v>46234</x:v>
+      <x:c r="A5" s="45" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B5" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -2624,8 +2650,8 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="45" t="n">
-        <x:v>46234</x:v>
+      <x:c r="A6" s="45" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B6" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -2663,8 +2689,8 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="45" t="n">
-        <x:v>46234</x:v>
+      <x:c r="A7" s="45" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B7" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -2701,8 +2727,8 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="45" t="n">
-        <x:v>46234</x:v>
+      <x:c r="A8" s="45" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B8" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -2740,8 +2766,8 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="45" t="n">
-        <x:v>46267</x:v>
+      <x:c r="A9" s="45" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B9" s="19" t="str">
         <x:v>Silicon Data</x:v>
@@ -2779,8 +2805,8 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="45" t="n">
-        <x:v>46267</x:v>
+      <x:c r="A10" s="45" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B10" s="19" t="str">
         <x:v>Silicon Data</x:v>
@@ -2818,8 +2844,8 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="45" t="n">
-        <x:v>46267</x:v>
+      <x:c r="A11" s="45" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B11" s="19" t="str">
         <x:v>Silicon Data</x:v>
@@ -2847,8 +2873,8 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="45" t="n">
-        <x:v>46267</x:v>
+      <x:c r="A12" s="45" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
         <x:v>Silicon Data</x:v>
@@ -2876,8 +2902,8 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="45" t="n">
-        <x:v>46270</x:v>
+      <x:c r="A13" s="45" t="d">
+        <x:v>2026-09-05T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B13" s="19" t="str">
         <x:v>Silicon Data</x:v>
@@ -2905,8 +2931,8 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="45" t="n">
-        <x:v>46271</x:v>
+      <x:c r="A14" s="45" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B14" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -2934,8 +2960,8 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="45" t="n">
-        <x:v>46271</x:v>
+      <x:c r="A15" s="45" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B15" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -2963,8 +2989,8 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="45" t="n">
-        <x:v>46271</x:v>
+      <x:c r="A16" s="45" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B16" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -2992,8 +3018,8 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="45" t="n">
-        <x:v>46271</x:v>
+      <x:c r="A17" s="45" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B17" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -3021,8 +3047,8 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="45" t="n">
-        <x:v>46271</x:v>
+      <x:c r="A18" s="45" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B18" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -3050,8 +3076,8 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="45" t="n">
-        <x:v>46271</x:v>
+      <x:c r="A19" s="45" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B19" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -3079,38 +3105,386 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="46" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-      <x:c r="B20" s="20" t="str">
+      <x:c r="A20" s="45" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="str">
         <x:v>Vercel</x:v>
       </x:c>
-      <x:c r="C20" s="20" t="str">
+      <x:c r="C20" s="19" t="str">
         <x:v>OpenAI spend share</x:v>
       </x:c>
-      <x:c r="D20" s="48" t="n">
+      <x:c r="D20" s="47" t="n">
         <x:v>0.215</x:v>
       </x:c>
-      <x:c r="E20" s="20" t="str">
+      <x:c r="E20" s="19" t="str">
         <x:v>percent</x:v>
       </x:c>
-      <x:c r="F20" s="20" t="str">
+      <x:c r="F20" s="19" t="str">
         <x:v>endpoint</x:v>
       </x:c>
-      <x:c r="G20" s="20" t="str">
+      <x:c r="G20" s="19" t="str">
         <x:v>SRC-TOKEN-WE-SEP06-001</x:v>
       </x:c>
-      <x:c r="H20" s="20" t="str">
+      <x:c r="H20" s="19" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="I20" s="44" t="str">
+      <x:c r="I20" s="43" t="str">
         <x:v>Lab-level share</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="45" t="d">
+        <x:v>2026-09-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B21" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C21" s="19" t="str">
+        <x:v>Effective price per million tokens</x:v>
+      </x:c>
+      <x:c r="D21" s="47" t="n">
+        <x:v>0.68</x:v>
+      </x:c>
+      <x:c r="E21" s="19" t="str">
+        <x:v>USD per million tokens</x:v>
+      </x:c>
+      <x:c r="F21" s="19" t="str">
+        <x:v>publication_week</x:v>
+      </x:c>
+      <x:c r="G21" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-SEP2026</x:v>
+      </x:c>
+      <x:c r="H21" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I21" s="43" t="str">
+        <x:v>Down 41 percent from 2026 peak of 1.15 in March</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B22" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C22" s="19" t="str">
+        <x:v>Total model-attributed spend</x:v>
+      </x:c>
+      <x:c r="D22" s="47" t="n">
+        <x:v>27900000</x:v>
+      </x:c>
+      <x:c r="E22" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F22" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G22" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H22" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I22" s="43" t="str">
+        <x:v>All models in connected business sample</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B23" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C23" s="19" t="str">
+        <x:v>OpenAI provider spend</x:v>
+      </x:c>
+      <x:c r="D23" s="47" t="n">
+        <x:v>13700000</x:v>
+      </x:c>
+      <x:c r="E23" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F23" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G23" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H23" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I23" s="43" t="str">
+        <x:v>Provider total from weekly volume chart</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B24" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C24" s="19" t="str">
+        <x:v>Anthropic provider spend</x:v>
+      </x:c>
+      <x:c r="D24" s="47" t="n">
+        <x:v>13100000</x:v>
+      </x:c>
+      <x:c r="E24" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F24" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G24" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H24" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I24" s="43" t="str">
+        <x:v>Provider total from weekly volume chart</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B25" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C25" s="19" t="str">
+        <x:v>xAI provider spend</x:v>
+      </x:c>
+      <x:c r="D25" s="47" t="n">
+        <x:v>633900</x:v>
+      </x:c>
+      <x:c r="E25" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F25" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G25" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H25" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I25" s="43" t="str">
+        <x:v>Provider total from weekly volume chart</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C26" s="19" t="str">
+        <x:v>Google provider spend</x:v>
+      </x:c>
+      <x:c r="D26" s="47" t="n">
+        <x:v>429500</x:v>
+      </x:c>
+      <x:c r="E26" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F26" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G26" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H26" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I26" s="43" t="str">
+        <x:v>Provider total from weekly volume chart</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B27" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C27" s="19" t="str">
+        <x:v>GPT-6 Astra spend</x:v>
+      </x:c>
+      <x:c r="D27" s="47" t="n">
+        <x:v>5300000</x:v>
+      </x:c>
+      <x:c r="E27" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F27" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G27" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H27" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I27" s="43" t="str">
+        <x:v>Model rank 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B28" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C28" s="19" t="str">
+        <x:v>Claude Opus 5 spend</x:v>
+      </x:c>
+      <x:c r="D28" s="47" t="n">
+        <x:v>4800000</x:v>
+      </x:c>
+      <x:c r="E28" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F28" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G28" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H28" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I28" s="43" t="str">
+        <x:v>Model rank 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B29" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C29" s="19" t="str">
+        <x:v>GPT-5.6 Sol spend</x:v>
+      </x:c>
+      <x:c r="D29" s="47" t="n">
+        <x:v>3200000</x:v>
+      </x:c>
+      <x:c r="E29" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F29" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G29" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H29" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I29" s="43" t="str">
+        <x:v>Model rank 3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C30" s="19" t="str">
+        <x:v>Claude Opus 4.8 spend</x:v>
+      </x:c>
+      <x:c r="D30" s="47" t="n">
+        <x:v>2100000</x:v>
+      </x:c>
+      <x:c r="E30" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F30" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G30" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H30" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I30" s="43" t="str">
+        <x:v>Model rank 4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C31" s="19" t="str">
+        <x:v>Claude Fable 5.1 spend</x:v>
+      </x:c>
+      <x:c r="D31" s="47" t="n">
+        <x:v>1800000</x:v>
+      </x:c>
+      <x:c r="E31" s="19" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F31" s="19" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G31" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H31" s="19" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I31" s="43" t="str">
+        <x:v>Model rank 5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="46" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B32" s="20" t="str">
+        <x:v>Ramp AI Index</x:v>
+      </x:c>
+      <x:c r="C32" s="20" t="str">
+        <x:v>Claude Sonnet 5 spend</x:v>
+      </x:c>
+      <x:c r="D32" s="48" t="n">
+        <x:v>1500000</x:v>
+      </x:c>
+      <x:c r="E32" s="20" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F32" s="20" t="str">
+        <x:v>7D</x:v>
+      </x:c>
+      <x:c r="G32" s="20" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="H32" s="20" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="I32" s="44" t="str">
+        <x:v>Model rank 6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb62e90fc3bce4a3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cb38108a6f34297"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3584,8 +3958,8 @@
       <x:c r="A5" s="19" t="str">
         <x:v>SRC-CHAT-001</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="n">
-        <x:v>46273</x:v>
+      <x:c r="B5" s="45" t="d">
+        <x:v>2026-09-08T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C5" s="19" t="str">
         <x:v>Jake / ChatGPT</x:v>
@@ -3611,8 +3985,8 @@
       <x:c r="A6" s="19" t="str">
         <x:v>SRC-WB-P2S-001</x:v>
       </x:c>
-      <x:c r="B6" s="45" t="n">
-        <x:v>46269</x:v>
+      <x:c r="B6" s="45" t="d">
+        <x:v>2026-09-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C6" s="19" t="str">
         <x:v>Wiki-Brain</x:v>
@@ -3640,8 +4014,8 @@
       <x:c r="A7" s="19" t="str">
         <x:v>SRC-WB-NSCALE-001</x:v>
       </x:c>
-      <x:c r="B7" s="45" t="n">
-        <x:v>46260</x:v>
+      <x:c r="B7" s="45" t="d">
+        <x:v>2026-08-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C7" s="19" t="str">
         <x:v>Wiki-Brain</x:v>
@@ -3669,8 +4043,8 @@
       <x:c r="A8" s="19" t="str">
         <x:v>SRC-WB-CRWV-001</x:v>
       </x:c>
-      <x:c r="B8" s="45" t="n">
-        <x:v>46247</x:v>
+      <x:c r="B8" s="45" t="d">
+        <x:v>2026-08-13T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C8" s="19" t="str">
         <x:v>Wiki-Brain</x:v>
@@ -3698,8 +4072,8 @@
       <x:c r="A9" s="19" t="str">
         <x:v>SRC-VERCEL-JUL26-001</x:v>
       </x:c>
-      <x:c r="B9" s="45" t="n">
-        <x:v>46245</x:v>
+      <x:c r="B9" s="45" t="d">
+        <x:v>2026-08-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C9" s="19" t="str">
         <x:v>Vercel</x:v>
@@ -3727,8 +4101,8 @@
       <x:c r="A10" s="19" t="str">
         <x:v>SRC-SD-SEP02-001</x:v>
       </x:c>
-      <x:c r="B10" s="45" t="n">
-        <x:v>46267</x:v>
+      <x:c r="B10" s="45" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C10" s="19" t="str">
         <x:v>Silicon Data</x:v>
@@ -3756,8 +4130,8 @@
       <x:c r="A11" s="19" t="str">
         <x:v>SRC-TOKEN-WE-SEP06-001</x:v>
       </x:c>
-      <x:c r="B11" s="45" t="n">
-        <x:v>46271</x:v>
+      <x:c r="B11" s="45" t="d">
+        <x:v>2026-09-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
         <x:v>MW/$ prior chat</x:v>
@@ -3785,8 +4159,8 @@
       <x:c r="A12" s="19" t="str">
         <x:v>SRC-TOKEN-AUG19-001</x:v>
       </x:c>
-      <x:c r="B12" s="45" t="n">
-        <x:v>46253</x:v>
+      <x:c r="B12" s="45" t="d">
+        <x:v>2026-08-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
         <x:v>MW/$ prior chat</x:v>
@@ -3814,8 +4188,8 @@
       <x:c r="A13" s="19" t="str">
         <x:v>SRC-NVDA-Q2FY27-001</x:v>
       </x:c>
-      <x:c r="B13" s="45" t="n">
-        <x:v>46260</x:v>
+      <x:c r="B13" s="45" t="d">
+        <x:v>2026-08-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C13" s="19" t="str">
         <x:v>NVIDIA</x:v>
@@ -3843,8 +4217,8 @@
       <x:c r="A14" s="19" t="str">
         <x:v>SRC-XAI-GS-RECAP-20260910</x:v>
       </x:c>
-      <x:c r="B14" s="45" t="n">
-        <x:v>46275</x:v>
+      <x:c r="B14" s="45" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
         <x:v>User-supplied Goldman recap</x:v>
@@ -3870,8 +4244,8 @@
       <x:c r="A15" s="19" t="str">
         <x:v>SRC-XAI-GS-QA-20260910</x:v>
       </x:c>
-      <x:c r="B15" s="45" t="n">
-        <x:v>46275</x:v>
+      <x:c r="B15" s="45" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
         <x:v>Bret Johnsen via Investing.com</x:v>
@@ -3899,8 +4273,8 @@
       <x:c r="A16" s="19" t="str">
         <x:v>SRC-XAI-GS-EVENT-20260910</x:v>
       </x:c>
-      <x:c r="B16" s="45" t="n">
-        <x:v>46275</x:v>
+      <x:c r="B16" s="45" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
         <x:v>SpaceX investor relations</x:v>
@@ -3928,8 +4302,8 @@
       <x:c r="A17" s="19" t="str">
         <x:v>SRC-ORCL-Q1FY27-20260910</x:v>
       </x:c>
-      <x:c r="B17" s="45" t="n">
-        <x:v>46275</x:v>
+      <x:c r="B17" s="45" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
         <x:v>Oracle / SEC</x:v>
@@ -3957,8 +4331,8 @@
       <x:c r="A18" s="19" t="str">
         <x:v>SRC-ORCL-10K-FY26</x:v>
       </x:c>
-      <x:c r="B18" s="45" t="n">
-        <x:v>46195</x:v>
+      <x:c r="B18" s="45" t="d">
+        <x:v>2026-06-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C18" s="19" t="str">
         <x:v>Oracle / SEC</x:v>
@@ -3986,8 +4360,8 @@
       <x:c r="A19" s="19" t="str">
         <x:v>SRC-ORCL-10Q-Q3FY26</x:v>
       </x:c>
-      <x:c r="B19" s="45" t="n">
-        <x:v>46092</x:v>
+      <x:c r="B19" s="45" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C19" s="19" t="str">
         <x:v>Oracle / SEC</x:v>
@@ -4015,8 +4389,8 @@
       <x:c r="A20" s="19" t="str">
         <x:v>SRC-ORCL-CEO-20260612</x:v>
       </x:c>
-      <x:c r="B20" s="45" t="n">
-        <x:v>46185</x:v>
+      <x:c r="B20" s="45" t="d">
+        <x:v>2026-06-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C20" s="19" t="str">
         <x:v>Oracle</x:v>
@@ -4073,8 +4447,8 @@
       <x:c r="A22" s="19" t="str">
         <x:v>SRC-ORCL-CARBON-20250630</x:v>
       </x:c>
-      <x:c r="B22" s="45" t="n">
-        <x:v>45838</x:v>
+      <x:c r="B22" s="45" t="d">
+        <x:v>2025-06-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C22" s="19" t="str">
         <x:v>Oracle</x:v>
@@ -4131,8 +4505,8 @@
       <x:c r="A24" s="19" t="str">
         <x:v>SRC-ORCL-GREEN-CLOUD-20260911</x:v>
       </x:c>
-      <x:c r="B24" s="45" t="n">
-        <x:v>46276</x:v>
+      <x:c r="B24" s="45" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C24" s="19" t="str">
         <x:v>Oracle</x:v>
@@ -4160,8 +4534,8 @@
       <x:c r="A25" s="19" t="str">
         <x:v>SRC-OPENAI-ORACLE-20250722</x:v>
       </x:c>
-      <x:c r="B25" s="45" t="n">
-        <x:v>45860</x:v>
+      <x:c r="B25" s="45" t="d">
+        <x:v>2025-07-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C25" s="19" t="str">
         <x:v>OpenAI</x:v>
@@ -4189,8 +4563,8 @@
       <x:c r="A26" s="19" t="str">
         <x:v>SRC-OPENAI-STARGATE-20250923</x:v>
       </x:c>
-      <x:c r="B26" s="45" t="n">
-        <x:v>45923</x:v>
+      <x:c r="B26" s="45" t="d">
+        <x:v>2025-09-23T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C26" s="19" t="str">
         <x:v>OpenAI</x:v>
@@ -4218,8 +4592,8 @@
       <x:c r="A27" s="19" t="str">
         <x:v>SRC-CRUSOE-ABILENE-20250521</x:v>
       </x:c>
-      <x:c r="B27" s="45" t="n">
-        <x:v>45798</x:v>
+      <x:c r="B27" s="45" t="d">
+        <x:v>2025-05-21T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C27" s="19" t="str">
         <x:v>Crusoe</x:v>
@@ -4247,8 +4621,8 @@
       <x:c r="A28" s="19" t="str">
         <x:v>SRC-ORCL-REVOLVER-20260306</x:v>
       </x:c>
-      <x:c r="B28" s="45" t="n">
-        <x:v>46092</x:v>
+      <x:c r="B28" s="45" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C28" s="19" t="str">
         <x:v>Oracle / SEC</x:v>
@@ -4276,8 +4650,8 @@
       <x:c r="A29" s="19" t="str">
         <x:v>SRC-ORCL-Q1FY27-EVENT</x:v>
       </x:c>
-      <x:c r="B29" s="45" t="n">
-        <x:v>46275</x:v>
+      <x:c r="B29" s="45" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C29" s="19" t="str">
         <x:v>Oracle</x:v>
@@ -4305,8 +4679,8 @@
       <x:c r="A30" s="19" t="str">
         <x:v>SRC-CRWV-10K-FY25</x:v>
       </x:c>
-      <x:c r="B30" s="45" t="n">
-        <x:v>46083</x:v>
+      <x:c r="B30" s="45" t="d">
+        <x:v>2026-03-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C30" s="19" t="str">
         <x:v>CoreWeave / SEC</x:v>
@@ -4334,8 +4708,8 @@
       <x:c r="A31" s="19" t="str">
         <x:v>SRC-CRWV-10Q-Q2FY26</x:v>
       </x:c>
-      <x:c r="B31" s="45" t="n">
-        <x:v>46246</x:v>
+      <x:c r="B31" s="45" t="d">
+        <x:v>2026-08-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C31" s="19" t="str">
         <x:v>CoreWeave / SEC</x:v>
@@ -4363,8 +4737,8 @@
       <x:c r="A32" s="19" t="str">
         <x:v>SRC-CRWV-Q1FY26-ER</x:v>
       </x:c>
-      <x:c r="B32" s="45" t="n">
-        <x:v>46149</x:v>
+      <x:c r="B32" s="45" t="d">
+        <x:v>2026-05-07T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C32" s="19" t="str">
         <x:v>CoreWeave</x:v>
@@ -4392,8 +4766,8 @@
       <x:c r="A33" s="19" t="str">
         <x:v>SRC-CRWV-Q2FY26-ER</x:v>
       </x:c>
-      <x:c r="B33" s="45" t="n">
-        <x:v>46245</x:v>
+      <x:c r="B33" s="45" t="d">
+        <x:v>2026-08-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C33" s="19" t="str">
         <x:v>CoreWeave</x:v>
@@ -4421,8 +4795,8 @@
       <x:c r="A34" s="19" t="str">
         <x:v>SRC-CRWV-DDTL55-8K</x:v>
       </x:c>
-      <x:c r="B34" s="45" t="n">
-        <x:v>46244</x:v>
+      <x:c r="B34" s="45" t="d">
+        <x:v>2026-08-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C34" s="19" t="str">
         <x:v>CoreWeave / SEC</x:v>
@@ -4450,8 +4824,8 @@
       <x:c r="A35" s="19" t="str">
         <x:v>SRC-CRWV-DDTL55-EX10</x:v>
       </x:c>
-      <x:c r="B35" s="45" t="n">
-        <x:v>46241</x:v>
+      <x:c r="B35" s="45" t="d">
+        <x:v>2026-08-07T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C35" s="19" t="str">
         <x:v>CoreWeave / SEC</x:v>
@@ -4479,8 +4853,8 @@
       <x:c r="A36" s="19" t="str">
         <x:v>SRC-CRWV-DDTL55-GUARANTEE</x:v>
       </x:c>
-      <x:c r="B36" s="45" t="n">
-        <x:v>46241</x:v>
+      <x:c r="B36" s="45" t="d">
+        <x:v>2026-08-07T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C36" s="19" t="str">
         <x:v>CoreWeave / SEC</x:v>
@@ -4508,8 +4882,8 @@
       <x:c r="A37" s="19" t="str">
         <x:v>SRC-CRWV-DDTL50-20260518</x:v>
       </x:c>
-      <x:c r="B37" s="45" t="n">
-        <x:v>46160</x:v>
+      <x:c r="B37" s="45" t="d">
+        <x:v>2026-05-18T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C37" s="19" t="str">
         <x:v>CoreWeave</x:v>
@@ -4537,8 +4911,8 @@
       <x:c r="A38" s="19" t="str">
         <x:v>SRC-CRWV-META-20260409</x:v>
       </x:c>
-      <x:c r="B38" s="45" t="n">
-        <x:v>46121</x:v>
+      <x:c r="B38" s="45" t="d">
+        <x:v>2026-04-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C38" s="19" t="str">
         <x:v>CoreWeave</x:v>
@@ -4566,8 +4940,8 @@
       <x:c r="A39" s="19" t="str">
         <x:v>SRC-NBIS-20F-FY25</x:v>
       </x:c>
-      <x:c r="B39" s="45" t="n">
-        <x:v>46142</x:v>
+      <x:c r="B39" s="45" t="d">
+        <x:v>2026-04-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C39" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4595,8 +4969,8 @@
       <x:c r="A40" s="19" t="str">
         <x:v>SRC-NBIS-Q2FY26-FS</x:v>
       </x:c>
-      <x:c r="B40" s="45" t="n">
-        <x:v>46246</x:v>
+      <x:c r="B40" s="45" t="d">
+        <x:v>2026-08-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C40" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4624,8 +4998,8 @@
       <x:c r="A41" s="19" t="str">
         <x:v>SRC-NBIS-Q2FY26-MDNA</x:v>
       </x:c>
-      <x:c r="B41" s="45" t="n">
-        <x:v>46246</x:v>
+      <x:c r="B41" s="45" t="d">
+        <x:v>2026-08-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C41" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4653,8 +5027,8 @@
       <x:c r="A42" s="19" t="str">
         <x:v>SRC-NBIS-Q2FY26-ER</x:v>
       </x:c>
-      <x:c r="B42" s="45" t="n">
-        <x:v>46246</x:v>
+      <x:c r="B42" s="45" t="d">
+        <x:v>2026-08-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C42" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4682,8 +5056,8 @@
       <x:c r="A43" s="19" t="str">
         <x:v>SRC-NBIS-Q2FY26-LETTER</x:v>
       </x:c>
-      <x:c r="B43" s="45" t="n">
-        <x:v>46246</x:v>
+      <x:c r="B43" s="45" t="d">
+        <x:v>2026-08-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C43" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4711,8 +5085,8 @@
       <x:c r="A44" s="19" t="str">
         <x:v>SRC-NBIS-ESG-FY25</x:v>
       </x:c>
-      <x:c r="B44" s="45" t="n">
-        <x:v>46233</x:v>
+      <x:c r="B44" s="45" t="d">
+        <x:v>2026-07-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C44" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4740,8 +5114,8 @@
       <x:c r="A45" s="19" t="str">
         <x:v>SRC-NBIS-MSFT-SOW</x:v>
       </x:c>
-      <x:c r="B45" s="45" t="n">
-        <x:v>46142</x:v>
+      <x:c r="B45" s="45" t="d">
+        <x:v>2026-04-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C45" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4769,8 +5143,8 @@
       <x:c r="A46" s="19" t="str">
         <x:v>SRC-NBIS-MSFT-ADDENDUM</x:v>
       </x:c>
-      <x:c r="B46" s="45" t="n">
-        <x:v>46142</x:v>
+      <x:c r="B46" s="45" t="d">
+        <x:v>2026-04-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C46" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4798,8 +5172,8 @@
       <x:c r="A47" s="19" t="str">
         <x:v>SRC-NBIS-META-CONTRACT</x:v>
       </x:c>
-      <x:c r="B47" s="45" t="n">
-        <x:v>46142</x:v>
+      <x:c r="B47" s="45" t="d">
+        <x:v>2026-04-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C47" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4827,8 +5201,8 @@
       <x:c r="A48" s="19" t="str">
         <x:v>SRC-NBIS-META-20260316</x:v>
       </x:c>
-      <x:c r="B48" s="45" t="n">
-        <x:v>46097</x:v>
+      <x:c r="B48" s="45" t="d">
+        <x:v>2026-03-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C48" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4856,8 +5230,8 @@
       <x:c r="A49" s="19" t="str">
         <x:v>SRC-NBIS-BLOOM-CONTRACT</x:v>
       </x:c>
-      <x:c r="B49" s="45" t="n">
-        <x:v>46162</x:v>
+      <x:c r="B49" s="45" t="d">
+        <x:v>2026-05-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C49" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4885,8 +5259,8 @@
       <x:c r="A50" s="19" t="str">
         <x:v>SRC-NBIS-ABS-20260717</x:v>
       </x:c>
-      <x:c r="B50" s="45" t="n">
-        <x:v>46220</x:v>
+      <x:c r="B50" s="45" t="d">
+        <x:v>2026-07-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C50" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4914,8 +5288,8 @@
       <x:c r="A51" s="19" t="str">
         <x:v>SRC-NBIS-CONVERT-20260824</x:v>
       </x:c>
-      <x:c r="B51" s="45" t="n">
-        <x:v>46258</x:v>
+      <x:c r="B51" s="45" t="d">
+        <x:v>2026-08-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C51" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4943,8 +5317,8 @@
       <x:c r="A52" s="19" t="str">
         <x:v>SRC-NBIS-INDENTURE-2030</x:v>
       </x:c>
-      <x:c r="B52" s="45" t="n">
-        <x:v>46258</x:v>
+      <x:c r="B52" s="45" t="d">
+        <x:v>2026-08-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C52" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -4972,8 +5346,8 @@
       <x:c r="A53" s="19" t="str">
         <x:v>SRC-NBIS-INDENTURE-2034</x:v>
       </x:c>
-      <x:c r="B53" s="45" t="n">
-        <x:v>46258</x:v>
+      <x:c r="B53" s="45" t="d">
+        <x:v>2026-08-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C53" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -5001,8 +5375,8 @@
       <x:c r="A54" s="19" t="str">
         <x:v>SRC-NBIS-PALANTIR-20260908</x:v>
       </x:c>
-      <x:c r="B54" s="45" t="n">
-        <x:v>46273</x:v>
+      <x:c r="B54" s="45" t="d">
+        <x:v>2026-09-08T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C54" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -5030,8 +5404,8 @@
       <x:c r="A55" s="19" t="str">
         <x:v>SRC-NBIS-NEWSROOM-20260915</x:v>
       </x:c>
-      <x:c r="B55" s="45" t="n">
-        <x:v>46280</x:v>
+      <x:c r="B55" s="45" t="d">
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C55" s="19" t="str">
         <x:v>Nebius Group N.V.</x:v>
@@ -5059,8 +5433,8 @@
       <x:c r="A56" s="19" t="str">
         <x:v>SRC-IREN-10K-FY26</x:v>
       </x:c>
-      <x:c r="B56" s="45" t="n">
-        <x:v>46261</x:v>
+      <x:c r="B56" s="45" t="d">
+        <x:v>2026-08-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C56" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5088,8 +5462,8 @@
       <x:c r="A57" s="19" t="str">
         <x:v>SRC-IREN-10Q-Q3FY26</x:v>
       </x:c>
-      <x:c r="B57" s="45" t="n">
-        <x:v>46150</x:v>
+      <x:c r="B57" s="45" t="d">
+        <x:v>2026-05-08T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C57" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5117,8 +5491,8 @@
       <x:c r="A58" s="19" t="str">
         <x:v>SRC-IREN-Q3FY26-ER</x:v>
       </x:c>
-      <x:c r="B58" s="45" t="n">
-        <x:v>46150</x:v>
+      <x:c r="B58" s="45" t="d">
+        <x:v>2026-05-08T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C58" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5146,8 +5520,8 @@
       <x:c r="A59" s="19" t="str">
         <x:v>SRC-IREN-FY26-ER</x:v>
       </x:c>
-      <x:c r="B59" s="45" t="n">
-        <x:v>46261</x:v>
+      <x:c r="B59" s="45" t="d">
+        <x:v>2026-08-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C59" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5175,8 +5549,8 @@
       <x:c r="A60" s="19" t="str">
         <x:v>SRC-IREN-FY26-PRESENTATION</x:v>
       </x:c>
-      <x:c r="B60" s="45" t="n">
-        <x:v>46261</x:v>
+      <x:c r="B60" s="45" t="d">
+        <x:v>2026-08-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C60" s="19" t="str">
         <x:v>IREN Limited</x:v>
@@ -5204,8 +5578,8 @@
       <x:c r="A61" s="19" t="str">
         <x:v>SRC-IREN-MSFT-8K-20251103</x:v>
       </x:c>
-      <x:c r="B61" s="45" t="n">
-        <x:v>45964</x:v>
+      <x:c r="B61" s="45" t="d">
+        <x:v>2025-11-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C61" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5233,8 +5607,8 @@
       <x:c r="A62" s="19" t="str">
         <x:v>SRC-IREN-MSFT-CONTRACT</x:v>
       </x:c>
-      <x:c r="B62" s="45" t="n">
-        <x:v>46058</x:v>
+      <x:c r="B62" s="45" t="d">
+        <x:v>2026-02-05T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C62" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5262,8 +5636,8 @@
       <x:c r="A63" s="19" t="str">
         <x:v>SRC-IREN-GPUFIN-8K-20260529</x:v>
       </x:c>
-      <x:c r="B63" s="45" t="n">
-        <x:v>46171</x:v>
+      <x:c r="B63" s="45" t="d">
+        <x:v>2026-05-29T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C63" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5291,8 +5665,8 @@
       <x:c r="A64" s="19" t="str">
         <x:v>SRC-IREN-GPUFIN-NPA</x:v>
       </x:c>
-      <x:c r="B64" s="45" t="n">
-        <x:v>46261</x:v>
+      <x:c r="B64" s="45" t="d">
+        <x:v>2026-08-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C64" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5320,8 +5694,8 @@
       <x:c r="A65" s="19" t="str">
         <x:v>SRC-IREN-GPUFIN-CTA</x:v>
       </x:c>
-      <x:c r="B65" s="45" t="n">
-        <x:v>46261</x:v>
+      <x:c r="B65" s="45" t="d">
+        <x:v>2026-08-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C65" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5349,8 +5723,8 @@
       <x:c r="A66" s="19" t="str">
         <x:v>SRC-IREN-GPUFIN-REMARKETING-GUARANTEE</x:v>
       </x:c>
-      <x:c r="B66" s="45" t="n">
-        <x:v>46261</x:v>
+      <x:c r="B66" s="45" t="d">
+        <x:v>2026-08-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C66" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5378,8 +5752,8 @@
       <x:c r="A67" s="19" t="str">
         <x:v>SRC-IREN-GPUFIN-PERFORMANCE-GUARANTEE</x:v>
       </x:c>
-      <x:c r="B67" s="45" t="n">
-        <x:v>46261</x:v>
+      <x:c r="B67" s="45" t="d">
+        <x:v>2026-08-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C67" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5407,8 +5781,8 @@
       <x:c r="A68" s="19" t="str">
         <x:v>SRC-IREN-HORIZON1-20260813</x:v>
       </x:c>
-      <x:c r="B68" s="45" t="n">
-        <x:v>46247</x:v>
+      <x:c r="B68" s="45" t="d">
+        <x:v>2026-08-13T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C68" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5436,8 +5810,8 @@
       <x:c r="A69" s="19" t="str">
         <x:v>SRC-IREN-NVIDIA-DELL-20260526</x:v>
       </x:c>
-      <x:c r="B69" s="45" t="n">
-        <x:v>46168</x:v>
+      <x:c r="B69" s="45" t="d">
+        <x:v>2026-05-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C69" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5465,8 +5839,8 @@
       <x:c r="A70" s="19" t="str">
         <x:v>SRC-IREN-PRINCE-GEORGE-SITE-20260916</x:v>
       </x:c>
-      <x:c r="B70" s="45" t="n">
-        <x:v>46281</x:v>
+      <x:c r="B70" s="45" t="d">
+        <x:v>2026-09-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C70" s="19" t="str">
         <x:v>IREN Limited</x:v>
@@ -5494,8 +5868,8 @@
       <x:c r="A71" s="19" t="str">
         <x:v>SRC-IREN-MACKENZIE-SITE-20260916</x:v>
       </x:c>
-      <x:c r="B71" s="45" t="n">
-        <x:v>46281</x:v>
+      <x:c r="B71" s="45" t="d">
+        <x:v>2026-09-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C71" s="19" t="str">
         <x:v>IREN Limited</x:v>
@@ -5523,8 +5897,8 @@
       <x:c r="A72" s="19" t="str">
         <x:v>SRC-IREN-SWEETWATER-20260908</x:v>
       </x:c>
-      <x:c r="B72" s="45" t="n">
-        <x:v>46273</x:v>
+      <x:c r="B72" s="45" t="d">
+        <x:v>2026-09-08T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C72" s="19" t="str">
         <x:v>IREN Limited</x:v>
@@ -5552,8 +5926,8 @@
       <x:c r="A73" s="19" t="str">
         <x:v>SRC-MSFT-10K-FY26</x:v>
       </x:c>
-      <x:c r="B73" s="45" t="n">
-        <x:v>46232</x:v>
+      <x:c r="B73" s="45" t="d">
+        <x:v>2026-07-29T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C73" s="19" t="str">
         <x:v>Microsoft Corporation / SEC</x:v>
@@ -5581,8 +5955,8 @@
       <x:c r="A74" s="19" t="str">
         <x:v>SRC-MSFT-10Q-Q3FY26</x:v>
       </x:c>
-      <x:c r="B74" s="45" t="n">
-        <x:v>46141</x:v>
+      <x:c r="B74" s="45" t="d">
+        <x:v>2026-04-29T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C74" s="19" t="str">
         <x:v>Microsoft Corporation / SEC</x:v>
@@ -5610,8 +5984,8 @@
       <x:c r="A75" s="19" t="str">
         <x:v>SRC-MSFT-FY26-ER</x:v>
       </x:c>
-      <x:c r="B75" s="45" t="n">
-        <x:v>46232</x:v>
+      <x:c r="B75" s="45" t="d">
+        <x:v>2026-07-29T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C75" s="19" t="str">
         <x:v>Microsoft Corporation / SEC</x:v>
@@ -5639,8 +6013,8 @@
       <x:c r="A76" s="19" t="str">
         <x:v>SRC-MSFT-FY26-CALL</x:v>
       </x:c>
-      <x:c r="B76" s="45" t="n">
-        <x:v>46232</x:v>
+      <x:c r="B76" s="45" t="d">
+        <x:v>2026-07-29T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C76" s="19" t="str">
         <x:v>Microsoft Corporation</x:v>
@@ -5668,8 +6042,8 @@
       <x:c r="A77" s="19" t="str">
         <x:v>SRC-MSFT-SEGMENT-8K-20260902</x:v>
       </x:c>
-      <x:c r="B77" s="45" t="n">
-        <x:v>46267</x:v>
+      <x:c r="B77" s="45" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C77" s="19" t="str">
         <x:v>Microsoft Corporation / SEC</x:v>
@@ -5697,8 +6071,8 @@
       <x:c r="A78" s="19" t="str">
         <x:v>SRC-MSFT-SEGMENT-EX99-20260902</x:v>
       </x:c>
-      <x:c r="B78" s="45" t="n">
-        <x:v>46267</x:v>
+      <x:c r="B78" s="45" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C78" s="19" t="str">
         <x:v>Microsoft Corporation / SEC</x:v>
@@ -5726,8 +6100,8 @@
       <x:c r="A79" s="19" t="str">
         <x:v>SRC-MSFT-PUE-FY25</x:v>
       </x:c>
-      <x:c r="B79" s="45" t="n">
-        <x:v>46282</x:v>
+      <x:c r="B79" s="45" t="d">
+        <x:v>2026-09-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C79" s="19" t="str">
         <x:v>Microsoft Corporation</x:v>
@@ -5755,8 +6129,8 @@
       <x:c r="A80" s="19" t="str">
         <x:v>SRC-MSFT-ENV-DATA-FY25</x:v>
       </x:c>
-      <x:c r="B80" s="45" t="n">
-        <x:v>46217</x:v>
+      <x:c r="B80" s="45" t="d">
+        <x:v>2026-07-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C80" s="19" t="str">
         <x:v>Microsoft Corporation</x:v>
@@ -5784,8 +6158,8 @@
       <x:c r="A81" s="19" t="str">
         <x:v>SRC-MSFT-OPENAI-20251028</x:v>
       </x:c>
-      <x:c r="B81" s="45" t="n">
-        <x:v>45958</x:v>
+      <x:c r="B81" s="45" t="d">
+        <x:v>2025-10-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C81" s="19" t="str">
         <x:v>Microsoft Corporation</x:v>
@@ -5813,8 +6187,8 @@
       <x:c r="A82" s="19" t="str">
         <x:v>SRC-MSFT-OPENAI-20260427</x:v>
       </x:c>
-      <x:c r="B82" s="45" t="n">
-        <x:v>46139</x:v>
+      <x:c r="B82" s="45" t="d">
+        <x:v>2026-04-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C82" s="19" t="str">
         <x:v>Microsoft Corporation</x:v>
@@ -5842,8 +6216,8 @@
       <x:c r="A83" s="19" t="str">
         <x:v>SRC-MSFT-POWER-20240920</x:v>
       </x:c>
-      <x:c r="B83" s="45" t="n">
-        <x:v>45555</x:v>
+      <x:c r="B83" s="45" t="d">
+        <x:v>2024-09-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C83" s="19" t="str">
         <x:v>Microsoft Corporation</x:v>
@@ -5871,8 +6245,8 @@
       <x:c r="A84" s="19" t="str">
         <x:v>SRC-CEG-MSFT-PPA-20240920</x:v>
       </x:c>
-      <x:c r="B84" s="45" t="n">
-        <x:v>45555</x:v>
+      <x:c r="B84" s="45" t="d">
+        <x:v>2024-09-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C84" s="19" t="str">
         <x:v>Constellation Energy</x:v>
@@ -5900,8 +6274,8 @@
       <x:c r="A85" s="19" t="str">
         <x:v>SRC-AMZN-10K-FY25</x:v>
       </x:c>
-      <x:c r="B85" s="45" t="n">
-        <x:v>46059</x:v>
+      <x:c r="B85" s="45" t="d">
+        <x:v>2026-02-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C85" s="19" t="str">
         <x:v>Amazon / SEC</x:v>
@@ -5929,8 +6303,8 @@
       <x:c r="A86" s="19" t="str">
         <x:v>SRC-AMZN-10Q-Q2FY26</x:v>
       </x:c>
-      <x:c r="B86" s="45" t="n">
-        <x:v>46234</x:v>
+      <x:c r="B86" s="45" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C86" s="19" t="str">
         <x:v>Amazon / SEC</x:v>
@@ -5958,8 +6332,8 @@
       <x:c r="A87" s="19" t="str">
         <x:v>SRC-AMZN-Q2FY26-ER</x:v>
       </x:c>
-      <x:c r="B87" s="45" t="n">
-        <x:v>46233</x:v>
+      <x:c r="B87" s="45" t="d">
+        <x:v>2026-07-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C87" s="19" t="str">
         <x:v>Amazon</x:v>
@@ -6068,8 +6442,8 @@
       <x:c r="A91" s="19" t="str">
         <x:v>SRC-AWS-PUE-METHOD</x:v>
       </x:c>
-      <x:c r="B91" s="45" t="n">
-        <x:v>45629</x:v>
+      <x:c r="B91" s="45" t="d">
+        <x:v>2024-12-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C91" s="19" t="str">
         <x:v>Amazon</x:v>
@@ -6097,8 +6471,8 @@
       <x:c r="A92" s="19" t="str">
         <x:v>SRC-AMZN-ANTHROPIC-20260420</x:v>
       </x:c>
-      <x:c r="B92" s="45" t="n">
-        <x:v>46132</x:v>
+      <x:c r="B92" s="45" t="d">
+        <x:v>2026-04-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C92" s="19" t="str">
         <x:v>Amazon</x:v>
@@ -6126,8 +6500,8 @@
       <x:c r="A93" s="19" t="str">
         <x:v>SRC-ANTHROPIC-AWS-20260420</x:v>
       </x:c>
-      <x:c r="B93" s="45" t="n">
-        <x:v>46132</x:v>
+      <x:c r="B93" s="45" t="d">
+        <x:v>2026-04-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C93" s="19" t="str">
         <x:v>Anthropic</x:v>
@@ -6155,8 +6529,8 @@
       <x:c r="A94" s="19" t="str">
         <x:v>SRC-AMZN-OPENAI-20260227</x:v>
       </x:c>
-      <x:c r="B94" s="45" t="n">
-        <x:v>46080</x:v>
+      <x:c r="B94" s="45" t="d">
+        <x:v>2026-02-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C94" s="19" t="str">
         <x:v>Amazon / OpenAI</x:v>
@@ -6184,8 +6558,8 @@
       <x:c r="A95" s="19" t="str">
         <x:v>SRC-AMZN-TERMLOAN-20260610</x:v>
       </x:c>
-      <x:c r="B95" s="45" t="n">
-        <x:v>46183</x:v>
+      <x:c r="B95" s="45" t="d">
+        <x:v>2026-06-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C95" s="19" t="str">
         <x:v>Amazon / SEC</x:v>
@@ -6213,8 +6587,8 @@
       <x:c r="A96" s="19" t="str">
         <x:v>SRC-AMZN-REVOLVER364-20260731</x:v>
       </x:c>
-      <x:c r="B96" s="45" t="n">
-        <x:v>46234</x:v>
+      <x:c r="B96" s="45" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C96" s="19" t="str">
         <x:v>Amazon / SEC</x:v>
@@ -6242,8 +6616,8 @@
       <x:c r="A97" s="19" t="str">
         <x:v>SRC-AMZN-REVOLVER5Y-20260731</x:v>
       </x:c>
-      <x:c r="B97" s="45" t="n">
-        <x:v>46234</x:v>
+      <x:c r="B97" s="45" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C97" s="19" t="str">
         <x:v>Amazon / SEC</x:v>
@@ -6271,8 +6645,8 @@
       <x:c r="A98" s="19" t="str">
         <x:v>SRC-TALEN-AWS-PPA-20250611</x:v>
       </x:c>
-      <x:c r="B98" s="45" t="n">
-        <x:v>45819</x:v>
+      <x:c r="B98" s="45" t="d">
+        <x:v>2025-06-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C98" s="19" t="str">
         <x:v>Talen / SEC</x:v>
@@ -6327,8 +6701,8 @@
       <x:c r="A100" s="19" t="str">
         <x:v>SRC-GOOG-10K-FY25</x:v>
       </x:c>
-      <x:c r="B100" s="45" t="n">
-        <x:v>46058</x:v>
+      <x:c r="B100" s="45" t="d">
+        <x:v>2026-02-05T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C100" s="19" t="str">
         <x:v>Alphabet Inc. / SEC</x:v>
@@ -6356,8 +6730,8 @@
       <x:c r="A101" s="19" t="str">
         <x:v>SRC-GOOG-10Q-Q2FY26</x:v>
       </x:c>
-      <x:c r="B101" s="45" t="n">
-        <x:v>46226</x:v>
+      <x:c r="B101" s="45" t="d">
+        <x:v>2026-07-23T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C101" s="19" t="str">
         <x:v>Alphabet Inc. / SEC</x:v>
@@ -6385,8 +6759,8 @@
       <x:c r="A102" s="19" t="str">
         <x:v>SRC-GOOG-Q2FY26-ER</x:v>
       </x:c>
-      <x:c r="B102" s="45" t="n">
-        <x:v>46225</x:v>
+      <x:c r="B102" s="45" t="d">
+        <x:v>2026-07-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C102" s="19" t="str">
         <x:v>Alphabet Inc. / SEC</x:v>
@@ -6414,8 +6788,8 @@
       <x:c r="A103" s="19" t="str">
         <x:v>SRC-GOOG-Q2FY26-CALL</x:v>
       </x:c>
-      <x:c r="B103" s="45" t="n">
-        <x:v>46225</x:v>
+      <x:c r="B103" s="45" t="d">
+        <x:v>2026-07-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C103" s="19" t="str">
         <x:v>Alphabet Inc.</x:v>
@@ -6524,8 +6898,8 @@
       <x:c r="A107" s="19" t="str">
         <x:v>SRC-BX-GOOG-TPUJV-20260518</x:v>
       </x:c>
-      <x:c r="B107" s="45" t="n">
-        <x:v>46160</x:v>
+      <x:c r="B107" s="45" t="d">
+        <x:v>2026-05-18T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C107" s="19" t="str">
         <x:v>Blackstone</x:v>
@@ -6553,8 +6927,8 @@
       <x:c r="A108" s="19" t="str">
         <x:v>SRC-SPX-GOOG-COMPUTE-20260605</x:v>
       </x:c>
-      <x:c r="B108" s="45" t="n">
-        <x:v>46178</x:v>
+      <x:c r="B108" s="45" t="d">
+        <x:v>2026-06-05T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C108" s="19" t="str">
         <x:v>SpaceX / SEC</x:v>
@@ -6579,38 +6953,328 @@
       </x:c>
     </x:row>
     <x:row r="109">
-      <x:c r="A109" s="20" t="str">
+      <x:c r="A109" s="19" t="str">
         <x:v>SRC-GOOG-EQUITY-RAISE-20260604</x:v>
       </x:c>
-      <x:c r="B109" s="46" t="n">
-        <x:v>46177</x:v>
-      </x:c>
-      <x:c r="C109" s="20" t="str">
+      <x:c r="B109" s="45" t="d">
+        <x:v>2026-06-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C109" s="19" t="str">
         <x:v>Alphabet Inc. / SEC</x:v>
       </x:c>
-      <x:c r="D109" s="44" t="str">
+      <x:c r="D109" s="43" t="str">
         <x:v>AI infrastructure equity capital raise</x:v>
       </x:c>
-      <x:c r="E109" s="44" t="str">
+      <x:c r="E109" s="43" t="str">
         <x:v>8-K_Exhibit_99.1</x:v>
       </x:c>
-      <x:c r="F109" s="44" t="str">
+      <x:c r="F109" s="43" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1652044/000119312526257724/d83560dex991.htm</x:v>
       </x:c>
-      <x:c r="G109" s="44" t="str">
+      <x:c r="G109" s="43" t="str">
         <x:v>alphabet_gcp;contract_economics;capex</x:v>
       </x:c>
-      <x:c r="H109" s="44" t="str">
+      <x:c r="H109" s="43" t="str">
         <x:v>primary_read</x:v>
       </x:c>
-      <x:c r="I109" s="44" t="str">
+      <x:c r="I109" s="43" t="str">
         <x:v>Offering composition and AI infrastructure use of proceeds</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-WE20260920</x:v>
+      </x:c>
+      <x:c r="B110" s="45" t="d">
+        <x:v>2026-09-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C110" s="19" t="str">
+        <x:v>Ramp Economics Lab</x:v>
+      </x:c>
+      <x:c r="D110" s="43" t="str">
+        <x:v>Ramp AI Index weekly token and spend volumes week ending September 20 2026</x:v>
+      </x:c>
+      <x:c r="E110" s="43" t="str">
+        <x:v>Interactive dashboard capture</x:v>
+      </x:c>
+      <x:c r="F110" s="43" t="str">
+        <x:v>https://ramp.com/data/ai-index</x:v>
+      </x:c>
+      <x:c r="G110" s="43" t="str">
+        <x:v>Weekly model attributed spend provider spend model spend and token volume series availability</x:v>
+      </x:c>
+      <x:c r="H110" s="43" t="str">
+        <x:v>Primary capture</x:v>
+      </x:c>
+      <x:c r="I110" s="43" t="str">
+        <x:v>Exact selected week values captured from Ramp UI screenshot supplied by user on 2026-09-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="19" t="str">
+        <x:v>SRC-RAMP-AIINDEX-SEP2026</x:v>
+      </x:c>
+      <x:c r="B111" s="45" t="d">
+        <x:v>2026-09-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C111" s="19" t="str">
+        <x:v>Ramp Economics Lab</x:v>
+      </x:c>
+      <x:c r="D111" s="43" t="str">
+        <x:v>Cracks in the AI Thesis Part 2</x:v>
+      </x:c>
+      <x:c r="E111" s="43" t="str">
+        <x:v>Web</x:v>
+      </x:c>
+      <x:c r="F111" s="43" t="str">
+        <x:v>https://ramp.com/data/ai-index-sept-2026</x:v>
+      </x:c>
+      <x:c r="G111" s="43" t="str">
+        <x:v>Effective token price price decline business mix and methodology</x:v>
+      </x:c>
+      <x:c r="H111" s="43" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="I111" s="43" t="str">
+        <x:v>Ramp reported 0.68 USD per million tokens and a 41 percent decline from the 2026 peak</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="19" t="str">
+        <x:v>SRC-META-10K-FY25</x:v>
+      </x:c>
+      <x:c r="B112" s="45" t="d">
+        <x:v>2026-01-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C112" s="19" t="str">
+        <x:v>Meta Platforms Inc. / SEC</x:v>
+      </x:c>
+      <x:c r="D112" s="43" t="str">
+        <x:v>FY2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E112" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F112" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1326801/000162828026003942/meta-20251231.htm</x:v>
+      </x:c>
+      <x:c r="G112" s="43" t="str">
+        <x:v>meta;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H112" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I112" s="43" t="str">
+        <x:v>Filing index; MD&amp;A; revenue; leases and contractual commitments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="19" t="str">
+        <x:v>SRC-META-10Q-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B113" s="45" t="d">
+        <x:v>2026-07-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C113" s="19" t="str">
+        <x:v>Meta Platforms Inc. / SEC</x:v>
+      </x:c>
+      <x:c r="D113" s="43" t="str">
+        <x:v>Q2 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E113" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F113" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1326801/000162828026050705/meta-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G113" s="43" t="str">
+        <x:v>meta;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H113" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I113" s="43" t="str">
+        <x:v>Revenue, VIEs, property, debt, commitments, subsequent event and MD&amp;A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="19" t="str">
+        <x:v>SRC-META-Q2FY26-ER</x:v>
+      </x:c>
+      <x:c r="B114" s="45" t="d">
+        <x:v>2026-07-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C114" s="19" t="str">
+        <x:v>Meta Platforms Inc.</x:v>
+      </x:c>
+      <x:c r="D114" s="43" t="str">
+        <x:v>Meta Reports Second Quarter 2026 Results</x:v>
+      </x:c>
+      <x:c r="E114" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F114" s="43" t="str">
+        <x:v>https://investor.atmeta.com/investor-news/press-release-details/2026/Meta-Reports-Second-Quarter-2026-Results/default.aspx</x:v>
+      </x:c>
+      <x:c r="G114" s="43" t="str">
+        <x:v>meta;revenue_per_mw;capex</x:v>
+      </x:c>
+      <x:c r="H114" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I114" s="43" t="str">
+        <x:v>Financial highlights capex cash flow and 2026 capex outlook</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="19" t="str">
+        <x:v>SRC-META-Q2FY26-CALL</x:v>
+      </x:c>
+      <x:c r="B115" s="45" t="d">
+        <x:v>2026-07-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C115" s="19" t="str">
+        <x:v>Meta Platforms Inc.</x:v>
+      </x:c>
+      <x:c r="D115" s="43" t="str">
+        <x:v>Q2 2026 earnings call transcript</x:v>
+      </x:c>
+      <x:c r="E115" s="43" t="str">
+        <x:v>issuer_earnings_call_transcript</x:v>
+      </x:c>
+      <x:c r="F115" s="43" t="str">
+        <x:v>https://s21.q4cdn.com/399680738/files/doc_financials/2026/q2/META-Q2-2026-Earnings-Call-Transcript.pdf</x:v>
+      </x:c>
+      <x:c r="G115" s="43" t="str">
+        <x:v>meta;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H115" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I115" s="43" t="str">
+        <x:v>AI monetization claims capacity strategy capex and direct-compute Q&amp;A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="19" t="str">
+        <x:v>SRC-META-Q2FY26-FOLLOWUP</x:v>
+      </x:c>
+      <x:c r="B116" s="45" t="d">
+        <x:v>2026-07-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C116" s="19" t="str">
+        <x:v>Meta Platforms Inc.</x:v>
+      </x:c>
+      <x:c r="D116" s="43" t="str">
+        <x:v>Q2 2026 follow-up call transcript</x:v>
+      </x:c>
+      <x:c r="E116" s="43" t="str">
+        <x:v>issuer_follow_up_call_transcript</x:v>
+      </x:c>
+      <x:c r="F116" s="43" t="str">
+        <x:v>https://s21.q4cdn.com/399680738/files/doc_financials/2026/q2/META-Q2-2026-Follow-Up-Call-Transcript.pdf</x:v>
+      </x:c>
+      <x:c r="G116" s="43" t="str">
+        <x:v>meta;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H116" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I116" s="43" t="str">
+        <x:v>Capacity partnership financing third-party cloud and enterprise monetization</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="19" t="str">
+        <x:v>SRC-META-PUE-FY24</x:v>
+      </x:c>
+      <x:c r="B117" s="45" t="d">
+        <x:v>2025-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C117" s="19" t="str">
+        <x:v>Meta Platforms Inc.</x:v>
+      </x:c>
+      <x:c r="D117" s="43" t="str">
+        <x:v>Meta 2025 Environmental Data Index</x:v>
+      </x:c>
+      <x:c r="E117" s="43" t="str">
+        <x:v>environmental_data_index</x:v>
+      </x:c>
+      <x:c r="F117" s="43" t="str">
+        <x:v>https://sustainability.atmeta.com/wp-content/uploads/2025/10/Meta_2025-Environmental-Data-Index.pdf</x:v>
+      </x:c>
+      <x:c r="G117" s="43" t="str">
+        <x:v>meta;revenue_per_mw;effective_mw</x:v>
+      </x:c>
+      <x:c r="H117" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I117" s="43" t="str">
+        <x:v>FY2024 annual fleet PUE 1.08; not a Q2 2026 AI-specific boundary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="19" t="str">
+        <x:v>SRC-META-HYPERION-20251021</x:v>
+      </x:c>
+      <x:c r="B118" s="45" t="d">
+        <x:v>2025-10-21T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C118" s="19" t="str">
+        <x:v>Meta Platforms Inc.</x:v>
+      </x:c>
+      <x:c r="D118" s="43" t="str">
+        <x:v>Meta Announces Joint Venture with Funds Managed by Blue Owl Capital to Develop Hyperion Data Center</x:v>
+      </x:c>
+      <x:c r="E118" s="43" t="str">
+        <x:v>issuer_joint_venture_announcement</x:v>
+      </x:c>
+      <x:c r="F118" s="43" t="str">
+        <x:v>https://investor.atmeta.com/investor-news/press-release-details/2025/Meta-Announces-Joint-Venture-with-Funds-Managed-by-Blue-Owl-Capital-to-Develop-Hyperion-Data-Center/default.aspx</x:v>
+      </x:c>
+      <x:c r="G118" s="43" t="str">
+        <x:v>meta;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H118" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I118" s="43" t="str">
+        <x:v>Ownership development funding contribution distribution lease and residual-value guarantee</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="20" t="str">
+        <x:v>SRC-META-ELPASO-20260728</x:v>
+      </x:c>
+      <x:c r="B119" s="46" t="d">
+        <x:v>2026-07-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C119" s="20" t="str">
+        <x:v>Meta Platforms Inc. and BlackRock</x:v>
+      </x:c>
+      <x:c r="D119" s="44" t="str">
+        <x:v>Meta Announces New Strategic Venture with BlackRock to Develop Data Center in El Paso</x:v>
+      </x:c>
+      <x:c r="E119" s="44" t="str">
+        <x:v>issuer_joint_venture_announcement</x:v>
+      </x:c>
+      <x:c r="F119" s="44" t="str">
+        <x:v>https://investor.atmeta.com/investor-news/press-release-details/2026/Meta-Announces-New-Strategic-Venture-with-BlackRock-to-Develop-Data-Center-in-El-Paso/default.aspx</x:v>
+      </x:c>
+      <x:c r="G119" s="44" t="str">
+        <x:v>meta;revenue_per_mw;contract_economics;capex</x:v>
+      </x:c>
+      <x:c r="H119" s="44" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I119" s="44" t="str">
+        <x:v>1 GW stated compute capacity expected 2028 with venture financing lease and residual-value guarantee</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f35b190f22441b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re83df2093adf4590"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research Nscale financing and acceptance economics; add compute futures time analysis
Read September S-1 annual/interim statements and contract exhibits. Replace rounded Anthropic value with conditional $44.6B; retain unsupported rate and capex estimates as historical references. Persist October 5 partial review and advance only Nscale in the queue.

Complete authorized FT/CME intake and time-aware current read. Rebuild workbook, remove stale dashboard anchor, and validate schemas, provenance, arithmetic and infrastructure/time projections.
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R74013eab31504457"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rafd8e37b884d4358"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R5339e32857864bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rff1eec694f974d95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Rd482aa08cfe84752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rd37ab03e5c55436e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rf3b1e00ecd2b4b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R67462a04965e4e37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R3d09ef5a820e42b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rbe3dc5fb3a904f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R8cb0fd8943ba44ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Ra52dbec6e8f543c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Re4b308c2d7d44753"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R828b41ab2b774c2d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I134" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -684,7 +684,7 @@
       </x:c>
       <x:c r="B7" s="19" t="n">
         <x:f>COUNT('Company Models'!S5:S19)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="19" t="str">
         <x:v>Acceptability line</x:v>
@@ -704,26 +704,21 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="19" t="str">
-        <x:v>Nscale contracted revenue ($M / effective MW-year)</x:v>
-      </x:c>
-      <x:c r="B8" s="58" t="n">
+        <x:v>Nscale recognized revenue ($M / effective MW-year)</x:v>
+      </x:c>
+      <x:c r="B8" s="58" t="str">
         <x:f>'Company Models'!S13</x:f>
-        <x:v>16.304347826086957</x:v>
       </x:c>
       <x:c r="D8" s="19" t="str">
         <x:v>Nscale / Anthropic</x:v>
       </x:c>
-      <x:c r="E8" s="54" t="n">
-        <x:v>16.3</x:v>
-      </x:c>
-      <x:c r="F8" s="54" t="n">
-        <x:v>16.3</x:v>
-      </x:c>
+      <x:c r="E8" s="54"/>
+      <x:c r="F8" s="54"/>
       <x:c r="G8" s="19" t="str">
-        <x:v>Contracted</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="H8" s="19" t="str">
-        <x:v>Does the offtake premium persist?</x:v>
+        <x:v>Capacity, term and rate redacted; see primary review</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -985,15 +980,14 @@
       </x:c>
       <x:c r="D21" s="19" t="str">
         <x:f>'Company Models'!N13</x:f>
-        <x:v>DERIVED</x:v>
-      </x:c>
-      <x:c r="E21" s="58" t="n">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="E21" s="58" t="str">
         <x:f>IF('Company Models'!S13="","",'Company Models'!S13)</x:f>
-        <x:v>16.304347826086957</x:v>
       </x:c>
       <x:c r="F21" s="19" t="str">
         <x:f>'Company Models'!T13</x:f>
-        <x:v>Calculated</x:v>
+        <x:v>Missing numerator or denominator</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1721,63 +1715,43 @@
         <x:v>CONTRACT-NSCALE</x:v>
       </x:c>
       <x:c r="C13" s="19" t="str">
-        <x:v>2026 contract</x:v>
-      </x:c>
-      <x:c r="D13" s="27" t="n">
-        <x:v>7500000000</x:v>
-      </x:c>
-      <x:c r="E13" s="29" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F13" s="31" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G13" s="33" t="n">
-        <x:v>460</x:v>
-      </x:c>
+        <x:v>H1 2026 / future tranches</x:v>
+      </x:c>
+      <x:c r="D13" s="27"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="31"/>
+      <x:c r="G13" s="33"/>
       <x:c r="H13" s="23" t="str">
-        <x:v>IT load</x:v>
-      </x:c>
-      <x:c r="I13" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J13" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K13" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L13" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I13" s="35"/>
+      <x:c r="J13" s="35"/>
+      <x:c r="K13" s="35"/>
+      <x:c r="L13" s="35"/>
       <x:c r="M13" s="19" t="str">
-        <x:v>SRC-WB-NSCALE-001</x:v>
+        <x:v>SRC-NSCALE-S1-20260918</x:v>
       </x:c>
       <x:c r="N13" s="19" t="str">
-        <x:v>DERIVED</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O13" s="43" t="str">
-        <x:v>$45B over six years divided by 460 MW contracted IT load</x:v>
-      </x:c>
-      <x:c r="P13" s="37" t="n">
+        <x:v>Up to $44.6B future payments. Public Anthropic order redacts capacity/rate/term. H1 $136.7M service+lease is a bundled diagnostic; matched AI revenue, average active IT MW, utilization and PUE missing. Old $16.30M rate is reference only.</x:v>
+      </x:c>
+      <x:c r="P13" s="37" t="str">
         <x:f>IF(OR(D13="",E13="",F13=""),"",D13*E13*F13)</x:f>
-        <x:v>7500000000</x:v>
-      </x:c>
-      <x:c r="Q13" s="39" t="n">
+      </x:c>
+      <x:c r="Q13" s="39" t="str">
         <x:f>IF(G13="","",IF(H13="IT load",G13,IF(H13="Facility power",IF(I13="","",G13/I13),IF(H13="Generation",IF(OR(I13="",J13="",K13=""),"",G13*J13*K13/I13),IF(H13="Effective utilized IT",G13,"")))))</x:f>
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="R13" s="39" t="n">
+      </x:c>
+      <x:c r="R13" s="39" t="str">
         <x:f>IF(Q13="","",IF(H13="Effective utilized IT",Q13,IF(L13="","",Q13*L13)))</x:f>
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="S13" s="41" t="n">
+      </x:c>
+      <x:c r="S13" s="41" t="str">
         <x:f>IF(OR(P13="",R13="",R13=0),"",P13/R13/1000000)</x:f>
-        <x:v>16.304347826086957</x:v>
       </x:c>
       <x:c r="T13" s="25" t="str">
         <x:f>IF(S13&lt;&gt;"","Calculated",IF(OR(N13="VENDOR ONLY",N13="CAPEX ONLY"),"Not an operator output","Missing numerator or denominator"))</x:f>
-        <x:v>Calculated</x:v>
+        <x:v>Missing numerator or denominator</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2359,16 +2333,16 @@
         <x:v>Contracted compute</x:v>
       </x:c>
       <x:c r="D13" s="43" t="str">
-        <x:v>Annual contract value</x:v>
+        <x:v>Recognized attributable compute revenue</x:v>
       </x:c>
       <x:c r="E13" s="43" t="str">
-        <x:v>Contracted IT-load MW</x:v>
+        <x:v>Period-average effective utilized IT MW</x:v>
       </x:c>
       <x:c r="F13" s="43" t="str">
-        <x:v>Keep contract rate separate from physical utilization</x:v>
+        <x:v>Keep future contract rate separate; acceptance and financing gates</x:v>
       </x:c>
       <x:c r="G13" s="43" t="str">
-        <x:v>Active anchor</x:v>
+        <x:v>Partial; public terms redacted</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2512,7 +2486,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36ef155607784bbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801260d1ca5f402d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3484,7 +3458,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cb38108a6f34297"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bac0a80a0cf4884"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3661,37 +3635,25 @@
       <x:c r="B7" s="19" t="str">
         <x:v>Vera Rubin greenfield islanded</x:v>
       </x:c>
-      <x:c r="C7" s="54" t="n">
-        <x:v>34.8</x:v>
-      </x:c>
-      <x:c r="D7" s="54" t="n">
-        <x:v>17.9</x:v>
-      </x:c>
-      <x:c r="E7" s="54" t="n">
-        <x:v>52.7</x:v>
-      </x:c>
-      <x:c r="F7" s="54" t="n">
-        <x:v>16.3</x:v>
-      </x:c>
-      <x:c r="G7" s="54" t="n">
-        <x:v>16.3</x:v>
-      </x:c>
+      <x:c r="C7" s="54"/>
+      <x:c r="D7" s="54"/>
+      <x:c r="E7" s="54"/>
+      <x:c r="F7" s="54"/>
+      <x:c r="G7" s="54"/>
       <x:c r="H7" s="19" t="str">
-        <x:v>SRC-WB-NSCALE-001</x:v>
+        <x:v>SRC-NSCALE-S1-20260918</x:v>
       </x:c>
       <x:c r="I7" s="19" t="str">
-        <x:v>Derived</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="J7" s="43" t="str">
-        <x:v>Contracted rate; 2 GW onsite gas plus batteries for 1.35 GW IT</x:v>
-      </x:c>
-      <x:c r="K7" s="56" t="n">
+        <x:v>Inherited capex/rate estimates retained as reference_only atomic history. Current primary contract capacity/term/rate are redacted; no verified project payback.</x:v>
+      </x:c>
+      <x:c r="K7" s="56" t="str">
         <x:f>IF(OR(E7="",G7="",G7=0),"",E7/G7)</x:f>
-        <x:v>3.233128834355828</x:v>
-      </x:c>
-      <x:c r="L7" s="56" t="n">
+      </x:c>
+      <x:c r="L7" s="56" t="str">
         <x:f>IF(OR(E7="",F7="",F7=0),"",E7/F7)</x:f>
-        <x:v>3.233128834355828</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -7243,38 +7205,465 @@
       </x:c>
     </x:row>
     <x:row r="119">
-      <x:c r="A119" s="20" t="str">
+      <x:c r="A119" s="19" t="str">
         <x:v>SRC-META-ELPASO-20260728</x:v>
       </x:c>
-      <x:c r="B119" s="46" t="d">
+      <x:c r="B119" s="45" t="d">
         <x:v>2026-07-28T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C119" s="20" t="str">
+      <x:c r="C119" s="19" t="str">
         <x:v>Meta Platforms Inc. and BlackRock</x:v>
       </x:c>
-      <x:c r="D119" s="44" t="str">
+      <x:c r="D119" s="43" t="str">
         <x:v>Meta Announces New Strategic Venture with BlackRock to Develop Data Center in El Paso</x:v>
       </x:c>
-      <x:c r="E119" s="44" t="str">
+      <x:c r="E119" s="43" t="str">
         <x:v>issuer_joint_venture_announcement</x:v>
       </x:c>
-      <x:c r="F119" s="44" t="str">
+      <x:c r="F119" s="43" t="str">
         <x:v>https://investor.atmeta.com/investor-news/press-release-details/2026/Meta-Announces-New-Strategic-Venture-with-BlackRock-to-Develop-Data-Center-in-El-Paso/default.aspx</x:v>
       </x:c>
-      <x:c r="G119" s="44" t="str">
+      <x:c r="G119" s="43" t="str">
         <x:v>meta;revenue_per_mw;contract_economics;capex</x:v>
       </x:c>
-      <x:c r="H119" s="44" t="str">
+      <x:c r="H119" s="43" t="str">
         <x:v>primary_read</x:v>
       </x:c>
-      <x:c r="I119" s="44" t="str">
+      <x:c r="I119" s="43" t="str">
         <x:v>1 GW stated compute capacity expected 2028 with venture financing lease and residual-value guarantee</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="19" t="str">
+        <x:v>SRC-FT-COMPUTE-FUTURES-20261003</x:v>
+      </x:c>
+      <x:c r="B120" s="45" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C120" s="19" t="str">
+        <x:v>Financial Times</x:v>
+      </x:c>
+      <x:c r="D120" s="43" t="str">
+        <x:v>The coming futures market in AI compute</x:v>
+      </x:c>
+      <x:c r="E120" s="43" t="str">
+        <x:v>commentary</x:v>
+      </x:c>
+      <x:c r="F120" s="43" t="str">
+        <x:v>https://www.ft.com/content/a1815bc5-b5d5-47ff-bbbc-e1a689929321</x:v>
+      </x:c>
+      <x:c r="G120" s="43" t="str">
+        <x:v>compute_futures;time_to_mw</x:v>
+      </x:c>
+      <x:c r="H120" s="43" t="str">
+        <x:v>secondary_read</x:v>
+      </x:c>
+      <x:c r="I120" s="43" t="str">
+        <x:v>Text retrieved through search; direct page unavailable. Commentary, not proof of a live market or project-default prediction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="19" t="str">
+        <x:v>SRC-CME-COMPUTE-SPECS-20261004</x:v>
+      </x:c>
+      <x:c r="B121" s="45"/>
+      <x:c r="C121" s="19" t="str">
+        <x:v>CME Group</x:v>
+      </x:c>
+      <x:c r="D121" s="43" t="str">
+        <x:v>Compute futures product specifications</x:v>
+      </x:c>
+      <x:c r="E121" s="43" t="str">
+        <x:v>exchange_product_page</x:v>
+      </x:c>
+      <x:c r="F121" s="43" t="str">
+        <x:v>https://www.cmegroup.com/markets/energy/power/compute-futures.html</x:v>
+      </x:c>
+      <x:c r="G121" s="43" t="str">
+        <x:v>compute_futures;contract_economics</x:v>
+      </x:c>
+      <x:c r="H121" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I121" s="43" t="str">
+        <x:v>Undated live page observed October 4; planned H100/B200 non-hyperscaler rental benchmarks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="19" t="str">
+        <x:v>SRC-CME-COMPUTE-REVISED-20261004</x:v>
+      </x:c>
+      <x:c r="B122" s="45"/>
+      <x:c r="C122" s="19" t="str">
+        <x:v>CME Group</x:v>
+      </x:c>
+      <x:c r="D122" s="43" t="str">
+        <x:v>Revised clearing advisory 26-274: effective date to be announced</x:v>
+      </x:c>
+      <x:c r="E122" s="43" t="str">
+        <x:v>exchange_clearing_notice</x:v>
+      </x:c>
+      <x:c r="F122" s="43" t="str">
+        <x:v>https://www.cmegroup.com/notices/clearing/2026/08/26-274.html</x:v>
+      </x:c>
+      <x:c r="G122" s="43" t="str">
+        <x:v>compute_futures</x:v>
+      </x:c>
+      <x:c r="H122" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I122" s="43" t="str">
+        <x:v>Exact revision publication date unavailable. Page title says effective date to be announced; full advisory attachment not exposed in retrieved page.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="19" t="str">
+        <x:v>SRC-CME-COMPUTE-ANNOUNCE-20260811</x:v>
+      </x:c>
+      <x:c r="B123" s="45" t="d">
+        <x:v>2026-08-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C123" s="19" t="str">
+        <x:v>CME Group</x:v>
+      </x:c>
+      <x:c r="D123" s="43" t="str">
+        <x:v>CME Group and Silicon Data to Launch Compute Futures on October 5</x:v>
+      </x:c>
+      <x:c r="E123" s="43" t="str">
+        <x:v>exchange_press_release</x:v>
+      </x:c>
+      <x:c r="F123" s="43" t="str">
+        <x:v>https://cmegroupinc.gcs-web.com/node/55686</x:v>
+      </x:c>
+      <x:c r="G123" s="43" t="str">
+        <x:v>compute_futures</x:v>
+      </x:c>
+      <x:c r="H123" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I123" s="43" t="str">
+        <x:v>Original target only; later revised notice prevents treating October 5 as a confirmed live-trading date.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="19" t="str">
+        <x:v>SRC-MW-TIME-METHOD-20261002</x:v>
+      </x:c>
+      <x:c r="B124" s="45" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C124" s="19" t="str">
+        <x:v>MW/$ research</x:v>
+      </x:c>
+      <x:c r="D124" s="43" t="str">
+        <x:v>Project time and depreciation method and seeded dashboard</x:v>
+      </x:c>
+      <x:c r="E124" s="43" t="str">
+        <x:v>internal_method</x:v>
+      </x:c>
+      <x:c r="F124" s="43" t="str">
+        <x:v>https://github.com/smsyt4sjvc-crypto/MW-/blob/3172e3699ebbe47c46b8e8d8cdd734e849624342/ops/project-time-depreciation.md</x:v>
+      </x:c>
+      <x:c r="G124" s="43" t="str">
+        <x:v>time_to_mw;economic_depreciation</x:v>
+      </x:c>
+      <x:c r="H124" s="43" t="str">
+        <x:v>internal_model</x:v>
+      </x:c>
+      <x:c r="I124" s="43" t="str">
+        <x:v>Reference scenarios and three-observation seed, not an industry estimate; underlying primary milestone sources remain in infrastructure source ledger.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="19" t="str">
+        <x:v>SRC-NSCALE-S1-20260918</x:v>
+      </x:c>
+      <x:c r="B125" s="45" t="d">
+        <x:v>2026-09-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C125" s="19" t="str">
+        <x:v>Nscale / SEC</x:v>
+      </x:c>
+      <x:c r="D125" s="43" t="str">
+        <x:v>Nscale S-1: annual FY2025 and interim H1 2026 financials</x:v>
+      </x:c>
+      <x:c r="E125" s="43" t="str">
+        <x:v>S-1</x:v>
+      </x:c>
+      <x:c r="F125" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2110365/000119312526395475/ck0002110365-20260918.htm</x:v>
+      </x:c>
+      <x:c r="G125" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H125" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I125" s="43" t="str">
+        <x:v>pp. 13,27,84-86,99-100,114-115,118-119; F-4,F-6,F-10,F-17-18,F-45,F-47,F-49-50,F-52-55,F-63-65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="19" t="str">
+        <x:v>SRC-NSCALE-ANTHROPIC-EX1025</x:v>
+      </x:c>
+      <x:c r="B126" s="45" t="d">
+        <x:v>2026-09-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C126" s="19" t="str">
+        <x:v>Nscale / SEC</x:v>
+      </x:c>
+      <x:c r="D126" s="43" t="str">
+        <x:v>Form of Anthropic GPU services order</x:v>
+      </x:c>
+      <x:c r="E126" s="43" t="str">
+        <x:v>S-1 Exhibit 10.25</x:v>
+      </x:c>
+      <x:c r="F126" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2110365/000119312526395475/ck0002110365-ex10_25.htm</x:v>
+      </x:c>
+      <x:c r="G126" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H126" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I126" s="43" t="str">
+        <x:v>Order sections 1(c),4-9; pricing and capacity tables; terms of service and redacted schedules</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="19" t="str">
+        <x:v>SRC-NSCALE-MSFT-EX1019</x:v>
+      </x:c>
+      <x:c r="B127" s="45" t="d">
+        <x:v>2026-09-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C127" s="19" t="str">
+        <x:v>Nscale / SEC</x:v>
+      </x:c>
+      <x:c r="D127" s="43" t="str">
+        <x:v>Form of Microsoft partner statement of work</x:v>
+      </x:c>
+      <x:c r="E127" s="43" t="str">
+        <x:v>S-1 Exhibit 10.19</x:v>
+      </x:c>
+      <x:c r="F127" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2110365/000119312526395475/ck0002110365-ex10_19.htm</x:v>
+      </x:c>
+      <x:c r="G127" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H127" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I127" s="43" t="str">
+        <x:v>Sections 1.3,3.1-3.4,6.10: customer-supplied equipment, acceptance, delay credits and prepayment refund</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="19" t="str">
+        <x:v>SRC-NSCALE-DFS-EX1020</x:v>
+      </x:c>
+      <x:c r="B128" s="45" t="d">
+        <x:v>2026-09-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C128" s="19" t="str">
+        <x:v>Nscale / SEC</x:v>
+      </x:c>
+      <x:c r="D128" s="43" t="str">
+        <x:v>Dell Financial Services global framework agreement</x:v>
+      </x:c>
+      <x:c r="E128" s="43" t="str">
+        <x:v>S-1 Exhibit 10.20</x:v>
+      </x:c>
+      <x:c r="F128" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2110365/000119312526395475/ck0002110365-ex10_20.htm</x:v>
+      </x:c>
+      <x:c r="G128" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H128" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I128" s="43" t="str">
+        <x:v>Sections 2-8: title, unconditional payments, return, loss and acceleration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="19" t="str">
+        <x:v>SRC-NSCALE-WARD-EX1023</x:v>
+      </x:c>
+      <x:c r="B129" s="45" t="d">
+        <x:v>2026-09-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C129" s="19" t="str">
+        <x:v>Nscale / SEC</x:v>
+      </x:c>
+      <x:c r="D129" s="43" t="str">
+        <x:v>Ward County SPV credit agreement</x:v>
+      </x:c>
+      <x:c r="E129" s="43" t="str">
+        <x:v>S-1 Exhibit 10.23</x:v>
+      </x:c>
+      <x:c r="F129" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2110365/000119312526395475/ck0002110365-ex10_23.htm</x:v>
+      </x:c>
+      <x:c r="G129" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H129" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I129" s="43" t="str">
+        <x:v>Section 1.01 Term Maturity Date; sections 2.20 cash waterfall and 4.02 credit-event conditions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="19" t="str">
+        <x:v>SRC-NSCALE-NC-EX1024</x:v>
+      </x:c>
+      <x:c r="B130" s="45" t="d">
+        <x:v>2026-09-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C130" s="19" t="str">
+        <x:v>Nscale / SEC</x:v>
+      </x:c>
+      <x:c r="D130" s="43" t="str">
+        <x:v>North Carolina SPV credit agreement</x:v>
+      </x:c>
+      <x:c r="E130" s="43" t="str">
+        <x:v>S-1 Exhibit 10.24</x:v>
+      </x:c>
+      <x:c r="F130" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2110365/000119312526395475/ck0002110365-ex10_24.htm</x:v>
+      </x:c>
+      <x:c r="G130" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H130" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I130" s="43" t="str">
+        <x:v>Section 1.01 Advance Rate and Term Maturity Date; sections 2.20 and 4.02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="19" t="str">
+        <x:v>SRC-NSCALE-CONVERT-20260925</x:v>
+      </x:c>
+      <x:c r="B131" s="45" t="d">
+        <x:v>2026-09-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C131" s="19" t="str">
+        <x:v>Nscale</x:v>
+      </x:c>
+      <x:c r="D131" s="43" t="str">
+        <x:v>Nscale raises $3.36B pre-IPO convertible financing</x:v>
+      </x:c>
+      <x:c r="E131" s="43" t="str">
+        <x:v>issuer_release</x:v>
+      </x:c>
+      <x:c r="F131" s="43" t="str">
+        <x:v>https://www.nscale.com/press-releases/pre-ipo-convertible-financing</x:v>
+      </x:c>
+      <x:c r="G131" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H131" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I131" s="43" t="str">
+        <x:v>Opening paragraph and financing/tranche/conversion paragraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="19" t="str">
+        <x:v>SRC-NSCALE-DEPLOY-20261001</x:v>
+      </x:c>
+      <x:c r="B132" s="45" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C132" s="19" t="str">
+        <x:v>Nscale</x:v>
+      </x:c>
+      <x:c r="D132" s="43" t="str">
+        <x:v>Execution at scale: doubling deployments</x:v>
+      </x:c>
+      <x:c r="E132" s="43" t="str">
+        <x:v>issuer_operational_update</x:v>
+      </x:c>
+      <x:c r="F132" s="43" t="str">
+        <x:v>https://www.nscale.com/press-releases/execution-at-scale</x:v>
+      </x:c>
+      <x:c r="G132" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H132" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I132" s="43" t="str">
+        <x:v>Opening two paragraphs: 24000 additional GPUs and over 50000 across six active sites</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="19" t="str">
+        <x:v>SRC-NSCALE-SITES-20261005</x:v>
+      </x:c>
+      <x:c r="B133" s="45"/>
+      <x:c r="C133" s="19" t="str">
+        <x:v>Nscale</x:v>
+      </x:c>
+      <x:c r="D133" s="43" t="str">
+        <x:v>Nscale AI infrastructure site descriptions</x:v>
+      </x:c>
+      <x:c r="E133" s="43" t="str">
+        <x:v>issuer_site_page</x:v>
+      </x:c>
+      <x:c r="F133" s="43" t="str">
+        <x:v>https://www.nscale.com/ai-infrastructure</x:v>
+      </x:c>
+      <x:c r="G133" s="43" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H133" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I133" s="43" t="str">
+        <x:v>Glomfjord; Monarch Compute Campus; Ward County; North Carolina</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="20" t="str">
+        <x:v>SRC-NSCALE-SEC-INDEX-20261005</x:v>
+      </x:c>
+      <x:c r="B134" s="46"/>
+      <x:c r="C134" s="20" t="str">
+        <x:v>Nscale / SEC</x:v>
+      </x:c>
+      <x:c r="D134" s="44" t="str">
+        <x:v>Nscale SEC submissions index</x:v>
+      </x:c>
+      <x:c r="E134" s="44" t="str">
+        <x:v>regulator_index</x:v>
+      </x:c>
+      <x:c r="F134" s="44" t="str">
+        <x:v>https://data.sec.gov/submissions/CIK0002110365.json</x:v>
+      </x:c>
+      <x:c r="G134" s="44" t="str">
+        <x:v>Nscale review 2026-10-05</x:v>
+      </x:c>
+      <x:c r="H134" s="44" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I134" s="44" t="str">
+        <x:v>filings.recent: latest public S-1 September 18, 2026; prior DRS amendments</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re83df2093adf4590"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69ff014de7454947"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research xAI SpaceX cloud MW economics
Read the final prospectus, Q2 10-Q, earnings materials and primary deal/financing sources. Add a recognized-cloud/nameplate diagnostic while keeping PUE and canonical effective-MW economics blank. Persist the capital-stack findings, queue advance, workbook rebuild and compact 9PM handoff. Repair the missing Nscale question priority.
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R67462a04965e4e37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R3d09ef5a820e42b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rbe3dc5fb3a904f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R8cb0fd8943ba44ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Ra52dbec6e8f543c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Re4b308c2d7d44753"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R828b41ab2b774c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R651c7caa3f694ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rab522096438f4b8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Reb1a3bb99ead44e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Ra632b9d3fb434ced"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Ra123386f96d64be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rd3a8f9e138e54077"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rd39e3ee210d84731"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I134" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1001,11 +1001,11 @@
       </x:c>
       <x:c r="C22" s="19" t="str">
         <x:f>IFERROR(INDEX(Methods!$C$5:$C$19,MATCH(B22,Methods!$A$5:$A$19,0)),"")</x:f>
-        <x:v>Reference operator</x:v>
+        <x:v>Operator segment</x:v>
       </x:c>
       <x:c r="D22" s="19" t="str">
         <x:f>'Company Models'!N14</x:f>
-        <x:v>GUIDANCE ONLY</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E22" s="58" t="str">
         <x:f>IF('Company Models'!S14="","",'Company Models'!S14)</x:f>
@@ -1762,42 +1762,40 @@
         <x:v>PROJECT-XAI</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="D14" s="27"/>
-      <x:c r="E14" s="29"/>
+        <x:v>Q2 2026</x:v>
+      </x:c>
+      <x:c r="D14" s="27" t="n">
+        <x:v>1600000000</x:v>
+      </x:c>
+      <x:c r="E14" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="F14" s="31"/>
       <x:c r="G14" s="33" t="n">
-        <x:v>1400</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="H14" s="23" t="str">
         <x:v>IT load</x:v>
       </x:c>
-      <x:c r="I14" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J14" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K14" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="I14" s="35"/>
+      <x:c r="J14" s="35"/>
+      <x:c r="K14" s="35"/>
       <x:c r="L14" s="35"/>
       <x:c r="M14" s="19" t="str">
-        <x:v>SRC-WB-P2S-001</x:v>
+        <x:v>SRC-SPX-10Q-Q2FY26</x:v>
       </x:c>
       <x:c r="N14" s="19" t="str">
-        <x:v>GUIDANCE ONLY</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O14" s="43" t="str">
-        <x:v>Capex power anchor only; Sep 10 guidance is $30-50B per stated GW-year; effective denominator unresolved</x:v>
+        <x:v>Recognized incremental cloud-services revenue; modeled average nameplate draw 1.0-1.4 GW (1.2 base) from Q1/Q2 exits. Diagnostic $4.57-$6.40M per total nameplate MW-year only; external capacity allocation physical utilization and PUE are undisclosed so canonical effective-MW output stays blank.</x:v>
       </x:c>
       <x:c r="P14" s="37" t="str">
         <x:f>IF(OR(D14="",E14="",F14=""),"",D14*E14*F14)</x:f>
       </x:c>
       <x:c r="Q14" s="39" t="n">
         <x:f>IF(G14="","",IF(H14="IT load",G14,IF(H14="Facility power",IF(I14="","",G14/I14),IF(H14="Generation",IF(OR(I14="",J14="",K14=""),"",G14*J14*K14/I14),IF(H14="Effective utilized IT",G14,"")))))</x:f>
-        <x:v>1400</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="R14" s="39" t="str">
         <x:f>IF(Q14="","",IF(H14="Effective utilized IT",Q14,IF(L14="","",Q14*L14)))</x:f>
@@ -2353,19 +2351,19 @@
         <x:v>xAI / SpaceX</x:v>
       </x:c>
       <x:c r="C14" s="43" t="str">
-        <x:v>Reference operator</x:v>
+        <x:v>Operator segment</x:v>
       </x:c>
       <x:c r="D14" s="43" t="str">
-        <x:v>Recognized external compute revenue when reconciled</x:v>
+        <x:v>Annualized recognized external cloud-services revenue</x:v>
       </x:c>
       <x:c r="E14" s="43" t="str">
-        <x:v>Average effective Colossus IT MW</x:v>
+        <x:v>Time-weighted external allocated IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F14" s="43" t="str">
-        <x:v>Retain capex benchmark; separate Sep 10 monetization guidance until power scope reconciled</x:v>
+        <x:v>Use reported nameplate compute draw only as an IT-load exit metric; exclude internal Grok and non-cloud AI revenue; keep PUE guidance contracted sales and realized revenue separate</x:v>
       </x:c>
       <x:c r="G14" s="43" t="str">
-        <x:v>Capex anchor plus management guidance</x:v>
+        <x:v>Partial 2026-10-06; recognized new-cloud revenue and nameplate bounds established; external allocation and utilization open</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2486,7 +2484,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801260d1ca5f402d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42a328a283d04c53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3458,7 +3456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bac0a80a0cf4884"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra85cbefac5a044e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7634,36 +7632,237 @@
       </x:c>
     </x:row>
     <x:row r="134">
-      <x:c r="A134" s="20" t="str">
+      <x:c r="A134" s="19" t="str">
         <x:v>SRC-NSCALE-SEC-INDEX-20261005</x:v>
       </x:c>
-      <x:c r="B134" s="46"/>
-      <x:c r="C134" s="20" t="str">
+      <x:c r="B134" s="45"/>
+      <x:c r="C134" s="19" t="str">
         <x:v>Nscale / SEC</x:v>
       </x:c>
-      <x:c r="D134" s="44" t="str">
+      <x:c r="D134" s="43" t="str">
         <x:v>Nscale SEC submissions index</x:v>
       </x:c>
-      <x:c r="E134" s="44" t="str">
+      <x:c r="E134" s="43" t="str">
         <x:v>regulator_index</x:v>
       </x:c>
-      <x:c r="F134" s="44" t="str">
+      <x:c r="F134" s="43" t="str">
         <x:v>https://data.sec.gov/submissions/CIK0002110365.json</x:v>
       </x:c>
-      <x:c r="G134" s="44" t="str">
+      <x:c r="G134" s="43" t="str">
         <x:v>Nscale review 2026-10-05</x:v>
       </x:c>
-      <x:c r="H134" s="44" t="str">
+      <x:c r="H134" s="43" t="str">
         <x:v>Primary read</x:v>
       </x:c>
-      <x:c r="I134" s="44" t="str">
+      <x:c r="I134" s="43" t="str">
         <x:v>filings.recent: latest public S-1 September 18, 2026; prior DRS amendments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="19" t="str">
+        <x:v>SRC-SPX-424B4-20260612</x:v>
+      </x:c>
+      <x:c r="B135" s="45" t="d">
+        <x:v>2026-06-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C135" s="19" t="str">
+        <x:v>Space Exploration Technologies Corp. / SEC</x:v>
+      </x:c>
+      <x:c r="D135" s="43" t="str">
+        <x:v>Final prospectus with FY2025 audited financial statements</x:v>
+      </x:c>
+      <x:c r="E135" s="43" t="str">
+        <x:v>424B4</x:v>
+      </x:c>
+      <x:c r="F135" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1181412/000162828026042639/spaceexplorationtechnologi.htm</x:v>
+      </x:c>
+      <x:c r="G135" s="43" t="str">
+        <x:v>xAI / SpaceX review 2026-10-06</x:v>
+      </x:c>
+      <x:c r="H135" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I135" s="43" t="str">
+        <x:v>pp. 90,124; F-5; F-63; Note 17 and subsequent-event deal disclosures</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="19" t="str">
+        <x:v>SRC-SPX-10Q-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B136" s="45" t="d">
+        <x:v>2026-08-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C136" s="19" t="str">
+        <x:v>Space Exploration Technologies Corp. / SEC</x:v>
+      </x:c>
+      <x:c r="D136" s="43" t="str">
+        <x:v>Q2 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E136" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F136" s="43" t="str">
+        <x:v>https://s21.q4cdn.com/184289198/files/doc_financials/2026/q2/dc41a8f3-2234-40ec-95e3-3867336ae181.pdf</x:v>
+      </x:c>
+      <x:c r="G136" s="43" t="str">
+        <x:v>xAI / SpaceX review 2026-10-06</x:v>
+      </x:c>
+      <x:c r="H136" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I136" s="43" t="str">
+        <x:v>pp. 12-14,17-21,27,29-31,36,38,44-45 and 51-52</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="19" t="str">
+        <x:v>SRC-SPX-Q2FY26-ER</x:v>
+      </x:c>
+      <x:c r="B137" s="45" t="d">
+        <x:v>2026-08-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C137" s="19" t="str">
+        <x:v>Space Exploration Technologies Corp.</x:v>
+      </x:c>
+      <x:c r="D137" s="43" t="str">
+        <x:v>SpaceX reports second quarter 2026 results</x:v>
+      </x:c>
+      <x:c r="E137" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F137" s="43" t="str">
+        <x:v>https://s21.q4cdn.com/184289198/files/doc_financials/2026/q2/SpaceX-Reports-Second-Quarter-2026-Results.pdf</x:v>
+      </x:c>
+      <x:c r="G137" s="43" t="str">
+        <x:v>xAI / SpaceX review 2026-10-06</x:v>
+      </x:c>
+      <x:c r="H137" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I137" s="43" t="str">
+        <x:v>AI segment results nameplate compute capex cash debt and contracted-sales definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="19" t="str">
+        <x:v>SRC-SPX-Q2FY26-CALL</x:v>
+      </x:c>
+      <x:c r="B138" s="45" t="d">
+        <x:v>2026-08-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C138" s="19" t="str">
+        <x:v>Space Exploration Technologies Corp.</x:v>
+      </x:c>
+      <x:c r="D138" s="43" t="str">
+        <x:v>Q2 2026 earnings call transcript</x:v>
+      </x:c>
+      <x:c r="E138" s="43" t="str">
+        <x:v>earnings_call_transcript</x:v>
+      </x:c>
+      <x:c r="F138" s="43" t="str">
+        <x:v>https://s21.q4cdn.com/184289198/files/doc_financials/2026/q2/SpaceX-Q2-2026-Earnings_Transcript-FINAL.pdf</x:v>
+      </x:c>
+      <x:c r="G138" s="43" t="str">
+        <x:v>xAI / SpaceX review 2026-10-06</x:v>
+      </x:c>
+      <x:c r="H138" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I138" s="43" t="str">
+        <x:v>pp. 5-6 and 9-10: cloud ramp nameplate capex financing payback and guidance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="19" t="str">
+        <x:v>SRC-SPX-BOND-20260623</x:v>
+      </x:c>
+      <x:c r="B139" s="45" t="d">
+        <x:v>2026-06-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C139" s="19" t="str">
+        <x:v>Space Exploration Technologies Corp.</x:v>
+      </x:c>
+      <x:c r="D139" s="43" t="str">
+        <x:v>SpaceX announces pricing of $25 billion inaugural bond issuance</x:v>
+      </x:c>
+      <x:c r="E139" s="43" t="str">
+        <x:v>issuer_financing_release</x:v>
+      </x:c>
+      <x:c r="F139" s="43" t="str">
+        <x:v>https://ir.spacex.com/updates/releases-details/2026/SpaceX-Announces-Pricing-of-25-Billion-Inaugural-Bond-Issuance-2026-33VwNgsx3O/default.aspx</x:v>
+      </x:c>
+      <x:c r="G139" s="43" t="str">
+        <x:v>xAI / SpaceX review 2026-10-06</x:v>
+      </x:c>
+      <x:c r="H139" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I139" s="43" t="str">
+        <x:v>Five tranches coupons and maturities</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="19" t="str">
+        <x:v>SRC-XAI-ANTHROPIC-20260506</x:v>
+      </x:c>
+      <x:c r="B140" s="45" t="d">
+        <x:v>2026-05-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C140" s="19" t="str">
+        <x:v>SpaceXAI</x:v>
+      </x:c>
+      <x:c r="D140" s="43" t="str">
+        <x:v>New compute partnership with Anthropic</x:v>
+      </x:c>
+      <x:c r="E140" s="43" t="str">
+        <x:v>issuer_customer_announcement</x:v>
+      </x:c>
+      <x:c r="F140" s="43" t="str">
+        <x:v>https://x.ai/news/anthropic-compute-partnership</x:v>
+      </x:c>
+      <x:c r="G140" s="43" t="str">
+        <x:v>xAI / SpaceX review 2026-10-06</x:v>
+      </x:c>
+      <x:c r="H140" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I140" s="43" t="str">
+        <x:v>Colossus 1 access for training fine-tuning inference and HPC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="20" t="str">
+        <x:v>SRC-XAI-MEMPHIS-20261006</x:v>
+      </x:c>
+      <x:c r="B141" s="46"/>
+      <x:c r="C141" s="20" t="str">
+        <x:v>SpaceXAI</x:v>
+      </x:c>
+      <x:c r="D141" s="44" t="str">
+        <x:v>Memphis information center and fact-versus-fiction pages</x:v>
+      </x:c>
+      <x:c r="E141" s="44" t="str">
+        <x:v>issuer_site_pages</x:v>
+      </x:c>
+      <x:c r="F141" s="44" t="str">
+        <x:v>https://x.ai/memphis/info</x:v>
+      </x:c>
+      <x:c r="G141" s="44" t="str">
+        <x:v>xAI / SpaceX review 2026-10-06</x:v>
+      </x:c>
+      <x:c r="H141" s="44" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I141" s="44" t="str">
+        <x:v>No measured matched facility energy IT energy utilization or PUE</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69ff014de7454947"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R323905e13aba432e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research OpenAI Stargate MW economics
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R651c7caa3f694ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rab522096438f4b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Reb1a3bb99ead44e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Ra632b9d3fb434ced"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="Ra123386f96d64be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rd3a8f9e138e54077"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rd39e3ee210d84731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8ed2ba7de43a4fc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R71eae90b20f349ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Reafb317659514057"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R96fc4fe1b32e4ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R281b877273e045db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R8c2edcf155df4fb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rbd80d087fdec42db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I155" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1030,14 +1030,14 @@
       </x:c>
       <x:c r="D23" s="19" t="str">
         <x:f>'Company Models'!N15</x:f>
-        <x:v>CAPEX ONLY</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="E23" s="58" t="str">
         <x:f>IF('Company Models'!S15="","",'Company Models'!S15)</x:f>
       </x:c>
       <x:c r="F23" s="19" t="str">
         <x:f>'Company Models'!T15</x:f>
-        <x:v>Not an operator output</x:v>
+        <x:v>Missing numerator or denominator</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1816,52 +1816,51 @@
         <x:v>PROJECT-STARGATE</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
-        <x:v>2026</x:v>
+        <x:v>Abilene full build / evidence through 2026-10-07</x:v>
       </x:c>
       <x:c r="D15" s="27"/>
       <x:c r="E15" s="29"/>
       <x:c r="F15" s="31"/>
       <x:c r="G15" s="33" t="n">
-        <x:v>1000</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="H15" s="23" t="str">
-        <x:v>IT load</x:v>
+        <x:v>Facility power</x:v>
       </x:c>
       <x:c r="I15" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J15" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K15" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L15" s="35"/>
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="J15" s="35"/>
+      <x:c r="K15" s="35"/>
+      <x:c r="L15" s="35" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
       <x:c r="M15" s="19" t="str">
-        <x:v>SRC-WB-P2S-001</x:v>
+        <x:v>SRC-CRUSOE-IMPACT-20260528</x:v>
       </x:c>
       <x:c r="N15" s="19" t="str">
-        <x:v>CAPEX ONLY</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O15" s="43" t="str">
-        <x:v>Revenue numerator not disclosed; power used for capex benchmark only</x:v>
+        <x:v>Full-build design sensitivity only: 1.2GW facility / 1.2-1.4 design PUE = 857-1,000 IT MW. Utilization 80% is an explicit scenario, not measured. Revenue, period-average active IT MW and external allocation remain missing; canonical revenue/effective-MW stays blank.</x:v>
       </x:c>
       <x:c r="P15" s="37" t="str">
         <x:f>IF(OR(D15="",E15="",F15=""),"",D15*E15*F15)</x:f>
       </x:c>
       <x:c r="Q15" s="39" t="n">
         <x:f>IF(G15="","",IF(H15="IT load",G15,IF(H15="Facility power",IF(I15="","",G15/I15),IF(H15="Generation",IF(OR(I15="",J15="",K15=""),"",G15*J15*K15/I15),IF(H15="Effective utilized IT",G15,"")))))</x:f>
-        <x:v>1000</x:v>
-      </x:c>
-      <x:c r="R15" s="39" t="str">
+        <x:v>923.0769230769231</x:v>
+      </x:c>
+      <x:c r="R15" s="39" t="n">
         <x:f>IF(Q15="","",IF(H15="Effective utilized IT",Q15,IF(L15="","",Q15*L15)))</x:f>
+        <x:v>738.4615384615386</x:v>
       </x:c>
       <x:c r="S15" s="41" t="str">
         <x:f>IF(OR(P15="",R15="",R15=0),"",P15/R15/1000000)</x:f>
       </x:c>
       <x:c r="T15" s="25" t="str">
         <x:f>IF(S15&lt;&gt;"","Calculated",IF(OR(N15="VENDOR ONLY",N15="CAPEX ONLY"),"Not an operator output","Missing numerator or denominator"))</x:f>
-        <x:v>Not an operator output</x:v>
+        <x:v>Missing numerator or denominator</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2377,16 +2376,16 @@
         <x:v>Reference project</x:v>
       </x:c>
       <x:c r="D15" s="43" t="str">
-        <x:v>Recognized or contracted compute revenue</x:v>
+        <x:v>Annualized site-attributable recognized or contracted compute revenue</x:v>
       </x:c>
       <x:c r="E15" s="43" t="str">
-        <x:v>Contracted or active IT-load MW</x:v>
+        <x:v>Time-weighted active IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F15" s="43" t="str">
-        <x:v>Separate financing and total campus spend from revenue</x:v>
+        <x:v>Keep secured/exit MW, financing, RPO, prepayments, internal workloads and pass-through hardware separate; report project-capital sensitivities only when revenue is unavailable</x:v>
       </x:c>
       <x:c r="G15" s="43" t="str">
-        <x:v>Capex anchor only</x:v>
+        <x:v>Partial 2026-10-07; Abilene primary capital/PUE sensitivity established; revenue and effective-MW denominator open</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2484,7 +2483,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42a328a283d04c53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d6db8cc5a3d4855"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3456,7 +3455,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra85cbefac5a044e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R034de1b3870942ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3749,23 +3748,25 @@
         <x:v>OpenAI / Stargate</x:v>
       </x:c>
       <x:c r="B11" s="19" t="str">
-        <x:v>Unspecified</x:v>
-      </x:c>
-      <x:c r="C11" s="54" t="n">
-        <x:v>24.7</x:v>
-      </x:c>
-      <x:c r="D11" s="54"/>
-      <x:c r="E11" s="54"/>
+        <x:v>Abilene full-build facility/JV</x:v>
+      </x:c>
+      <x:c r="C11" s="54"/>
+      <x:c r="D11" s="54" t="n">
+        <x:v>16.25</x:v>
+      </x:c>
+      <x:c r="E11" s="54" t="n">
+        <x:v>16.25</x:v>
+      </x:c>
       <x:c r="F11" s="54"/>
       <x:c r="G11" s="54"/>
       <x:c r="H11" s="19" t="str">
-        <x:v>SRC-WB-P2S-001</x:v>
+        <x:v>SRC-CRUSOE-ABILENE-20250521</x:v>
       </x:c>
       <x:c r="I11" s="19" t="str">
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="J11" s="43" t="str">
-        <x:v>Per GW IT load</x:v>
+        <x:v>$15B / (1.2GW facility / 1.3 design PUE). Range $15.0B-$17.5B per IT GW at 1.2-1.4 design PUE. Project/facility capital, not compute-content spend or revenue.</x:v>
       </x:c>
       <x:c r="K11" s="56" t="str">
         <x:f>IF(OR(E11="",G11="",G11=0),"",E11/G11)</x:f>
@@ -7833,36 +7834,440 @@
       </x:c>
     </x:row>
     <x:row r="141">
-      <x:c r="A141" s="20" t="str">
+      <x:c r="A141" s="19" t="str">
         <x:v>SRC-XAI-MEMPHIS-20261006</x:v>
       </x:c>
-      <x:c r="B141" s="46"/>
-      <x:c r="C141" s="20" t="str">
+      <x:c r="B141" s="45"/>
+      <x:c r="C141" s="19" t="str">
         <x:v>SpaceXAI</x:v>
       </x:c>
-      <x:c r="D141" s="44" t="str">
+      <x:c r="D141" s="43" t="str">
         <x:v>Memphis information center and fact-versus-fiction pages</x:v>
       </x:c>
-      <x:c r="E141" s="44" t="str">
+      <x:c r="E141" s="43" t="str">
         <x:v>issuer_site_pages</x:v>
       </x:c>
-      <x:c r="F141" s="44" t="str">
+      <x:c r="F141" s="43" t="str">
         <x:v>https://x.ai/memphis/info</x:v>
       </x:c>
-      <x:c r="G141" s="44" t="str">
+      <x:c r="G141" s="43" t="str">
         <x:v>xAI / SpaceX review 2026-10-06</x:v>
       </x:c>
-      <x:c r="H141" s="44" t="str">
+      <x:c r="H141" s="43" t="str">
         <x:v>Primary read</x:v>
       </x:c>
-      <x:c r="I141" s="44" t="str">
+      <x:c r="I141" s="43" t="str">
         <x:v>No measured matched facility energy IT energy utilization or PUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="19" t="str">
+        <x:v>SRC-OPENAI-COMPUTE-INFRA-20260429</x:v>
+      </x:c>
+      <x:c r="B142" s="45" t="d">
+        <x:v>2026-04-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C142" s="19" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="D142" s="43" t="str">
+        <x:v>Building the compute infrastructure for the Intelligence Age</x:v>
+      </x:c>
+      <x:c r="E142" s="43" t="str">
+        <x:v>issuer_infrastructure_update</x:v>
+      </x:c>
+      <x:c r="F142" s="43" t="str">
+        <x:v>https://openai.com/index/building-the-compute-infrastructure-for-the-intelligence-age/</x:v>
+      </x:c>
+      <x:c r="G142" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H142" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I142" s="43" t="str">
+        <x:v>10 GW commitment and recent additions; Abilene operations and cooling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="19" t="str">
+        <x:v>SRC-CRUSOE-IMPACT-20260528</x:v>
+      </x:c>
+      <x:c r="B143" s="45" t="d">
+        <x:v>2026-05-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C143" s="19" t="str">
+        <x:v>Crusoe</x:v>
+      </x:c>
+      <x:c r="D143" s="43" t="str">
+        <x:v>Crusoe's 2025 Impact Report</x:v>
+      </x:c>
+      <x:c r="E143" s="43" t="str">
+        <x:v>developer_sustainability_report</x:v>
+      </x:c>
+      <x:c r="F143" s="43" t="str">
+        <x:v>https://www.crusoe.ai/resources/blog/crusoes-2025-impact-report</x:v>
+      </x:c>
+      <x:c r="G143" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H143" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I143" s="43" t="str">
+        <x:v>Abilene annualized design PUE 1.2-1.4; not measured operational PUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="19" t="str">
+        <x:v>SRC-CRUSOE-CAPACITY-20260609</x:v>
+      </x:c>
+      <x:c r="B144" s="45" t="d">
+        <x:v>2026-06-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C144" s="19" t="str">
+        <x:v>Crusoe</x:v>
+      </x:c>
+      <x:c r="D144" s="43" t="str">
+        <x:v>Crusoe's contracted AI infrastructure capacity approaches 5 gigawatts</x:v>
+      </x:c>
+      <x:c r="E144" s="43" t="str">
+        <x:v>developer_operational_update</x:v>
+      </x:c>
+      <x:c r="F144" s="43" t="str">
+        <x:v>https://www.crusoe.ai/resources/newsroom/crusoes-contracted-ai-infrastructure-capacity-approaches-5-gigawatts-across-data-centers-and-cloud</x:v>
+      </x:c>
+      <x:c r="G144" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H144" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I144" s="43" t="str">
+        <x:v>Abilene 1.2GW for Oracle; first two buildings operational and six under construction</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="19" t="str">
+        <x:v>SRC-OPENAI-FUNDING-20260227</x:v>
+      </x:c>
+      <x:c r="B145" s="45" t="d">
+        <x:v>2026-02-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C145" s="19" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="D145" s="43" t="str">
+        <x:v>Scaling AI for everyone</x:v>
+      </x:c>
+      <x:c r="E145" s="43" t="str">
+        <x:v>issuer_financing_announcement</x:v>
+      </x:c>
+      <x:c r="F145" s="43" t="str">
+        <x:v>https://openai.com/index/scaling-ai-for-everyone/</x:v>
+      </x:c>
+      <x:c r="G145" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H145" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I145" s="43" t="str">
+        <x:v>$110B investment at $730B pre-money valuation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="19" t="str">
+        <x:v>SRC-SBG-AR-FY26-20260727</x:v>
+      </x:c>
+      <x:c r="B146" s="45" t="d">
+        <x:v>2026-07-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C146" s="19" t="str">
+        <x:v>SoftBank Group Corp.</x:v>
+      </x:c>
+      <x:c r="D146" s="43" t="str">
+        <x:v>Annual Report FY2026</x:v>
+      </x:c>
+      <x:c r="E146" s="43" t="str">
+        <x:v>annual_report</x:v>
+      </x:c>
+      <x:c r="F146" s="43" t="str">
+        <x:v>https://group.softbank/media/Project/sbg/sbg/pdf/ir/financials/annual_reports/annual-report_fy2026_en.pdf</x:v>
+      </x:c>
+      <x:c r="G146" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H146" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I146" s="43" t="str">
+        <x:v>PDF pp.25,74,103: OpenAI investment bridge financing and Stargate exposure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="19" t="str">
+        <x:v>SRC-SBG-Q1FY26-20260806</x:v>
+      </x:c>
+      <x:c r="B147" s="45" t="d">
+        <x:v>2026-08-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C147" s="19" t="str">
+        <x:v>SoftBank Group Corp.</x:v>
+      </x:c>
+      <x:c r="D147" s="43" t="str">
+        <x:v>Consolidated Financial Report for the Three-Month Period Ended June 30 2026</x:v>
+      </x:c>
+      <x:c r="E147" s="43" t="str">
+        <x:v>quarterly_financial_report</x:v>
+      </x:c>
+      <x:c r="F147" s="43" t="str">
+        <x:v>https://group.softbank/media/Project/sbg/sbg/pdf/ir/financials/financial_reports/financial-report_q1fy2026_01_en.pdf</x:v>
+      </x:c>
+      <x:c r="G147" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H147" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I147" s="43" t="str">
+        <x:v>PDF pp.69-70: tranche schedule bridge and mandatory-prepayment linkage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="19" t="str">
+        <x:v>SRC-SBG-OPENAI-20261001</x:v>
+      </x:c>
+      <x:c r="B148" s="45" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C148" s="19" t="str">
+        <x:v>SoftBank Group Corp.</x:v>
+      </x:c>
+      <x:c r="D148" s="43" t="str">
+        <x:v>Third closing of additional investment in OpenAI</x:v>
+      </x:c>
+      <x:c r="E148" s="43" t="str">
+        <x:v>issuer_financing_update</x:v>
+      </x:c>
+      <x:c r="F148" s="43" t="str">
+        <x:v>https://group.softbank/en/news/press/20261001</x:v>
+      </x:c>
+      <x:c r="G148" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H148" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I148" s="43" t="str">
+        <x:v>$64.6B cumulative investment; bridge repaid and cancelled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="19" t="str">
+        <x:v>SRC-ORCL-10Q-Q1FY27</x:v>
+      </x:c>
+      <x:c r="B149" s="45" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C149" s="19" t="str">
+        <x:v>Oracle Corporation / SEC</x:v>
+      </x:c>
+      <x:c r="D149" s="43" t="str">
+        <x:v>Oracle Q1 FY2027 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E149" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F149" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="G149" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H149" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I149" s="43" t="str">
+        <x:v>Commitments prepayments cash flows and RPO; consolidated not wholly Stargate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="19" t="str">
+        <x:v>SRC-BLUEOWL-10Q-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B150" s="45" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C150" s="19" t="str">
+        <x:v>Blue Owl Capital Inc. / SEC</x:v>
+      </x:c>
+      <x:c r="D150" s="43" t="str">
+        <x:v>Blue Owl Q2 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E150" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F150" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1823945/000182394526000040/owl-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G150" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H150" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I150" s="43" t="str">
+        <x:v>No Abilene project-level economics identified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="19" t="str">
+        <x:v>SRC-DAC-JUPITER-IRB</x:v>
+      </x:c>
+      <x:c r="B151" s="45"/>
+      <x:c r="C151" s="19" t="str">
+        <x:v>Dona Ana County New Mexico</x:v>
+      </x:c>
+      <x:c r="D151" s="43" t="str">
+        <x:v>Project Jupiter IRB Series 2025A executed and recorded ordinance</x:v>
+      </x:c>
+      <x:c r="E151" s="43" t="str">
+        <x:v>county_irb_ordinance</x:v>
+      </x:c>
+      <x:c r="F151" s="43" t="str">
+        <x:v>https://cms2.revize.com/revize/donaanacounty/Documents/About%20Us/Economic%20Development%20Projects/IRB%20Series%202025A%20-%20Executed%20%26%20Recorded.pdf?t=202606101848290</x:v>
+      </x:c>
+      <x:c r="G151" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H151" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I151" s="43" t="str">
+        <x:v>$165B authorization ceiling; not proof of funded cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="19" t="str">
+        <x:v>SRC-ORCL-JUPITER-20260728</x:v>
+      </x:c>
+      <x:c r="B152" s="45" t="d">
+        <x:v>2026-07-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C152" s="19" t="str">
+        <x:v>Oracle Corporation</x:v>
+      </x:c>
+      <x:c r="D152" s="43" t="str">
+        <x:v>Project Jupiter brings AI infrastructure investment to New Mexico</x:v>
+      </x:c>
+      <x:c r="E152" s="43" t="str">
+        <x:v>issuer_project_announcement</x:v>
+      </x:c>
+      <x:c r="F152" s="43" t="str">
+        <x:v>https://www.oracle.com/news/announcement/project-jupiter-2026-07-28/</x:v>
+      </x:c>
+      <x:c r="G152" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H152" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I152" s="43" t="str">
+        <x:v>Project projections conditional on air permit and pipeline approval</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="19" t="str">
+        <x:v>SRC-NMED-JUPITER-20261007</x:v>
+      </x:c>
+      <x:c r="B153" s="45" t="d">
+        <x:v>2026-10-07T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C153" s="19" t="str">
+        <x:v>New Mexico Environment Department</x:v>
+      </x:c>
+      <x:c r="D153" s="43" t="str">
+        <x:v>Project Jupiter YGI Microgrid air-permit public notice status</x:v>
+      </x:c>
+      <x:c r="E153" s="43" t="str">
+        <x:v>regulator_status_notice</x:v>
+      </x:c>
+      <x:c r="F153" s="43" t="str">
+        <x:v>https://www.env.nm.gov/</x:v>
+      </x:c>
+      <x:c r="G153" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H153" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I153" s="43" t="str">
+        <x:v>Public-comment item marked stayed by New Mexico Supreme Court</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="19" t="str">
+        <x:v>SRC-NMED-JUPITER-DOCKET-20261007</x:v>
+      </x:c>
+      <x:c r="B154" s="45" t="d">
+        <x:v>2026-10-07T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C154" s="19" t="str">
+        <x:v>New Mexico Environment Department</x:v>
+      </x:c>
+      <x:c r="D154" s="43" t="str">
+        <x:v>Yucca Growth Infrastructure LLC microgrid permit docket</x:v>
+      </x:c>
+      <x:c r="E154" s="43" t="str">
+        <x:v>regulator_permit_docket</x:v>
+      </x:c>
+      <x:c r="F154" s="43" t="str">
+        <x:v>https://www.env.nm.gov/public-notices/yucca-growth-infrastructure-llc-ygi-microgrid/</x:v>
+      </x:c>
+      <x:c r="G154" s="43" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H154" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I154" s="43" t="str">
+        <x:v>Application revisions draft permit and hearing notices</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="20" t="str">
+        <x:v>SRC-FT-JUPITER-20260924</x:v>
+      </x:c>
+      <x:c r="B155" s="46" t="d">
+        <x:v>2026-09-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C155" s="20" t="str">
+        <x:v>Financial Times Alphaville</x:v>
+      </x:c>
+      <x:c r="D155" s="44" t="str">
+        <x:v>Oracle's New Mexico data-centre financing comes under pressure</x:v>
+      </x:c>
+      <x:c r="E155" s="44" t="str">
+        <x:v>secondary_financing_report</x:v>
+      </x:c>
+      <x:c r="F155" s="44" t="str">
+        <x:v>https://www.ft.com/content/82dbd39c-f8dd-4ef1-8a80-d430a22579bd</x:v>
+      </x:c>
+      <x:c r="G155" s="44" t="str">
+        <x:v>OpenAI / Stargate review 2026-10-07</x:v>
+      </x:c>
+      <x:c r="H155" s="44" t="str">
+        <x:v>Secondary read</x:v>
+      </x:c>
+      <x:c r="I155" s="44" t="str">
+        <x:v>Approx. $18B loans reported at 89-91; not independently verified</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R323905e13aba432e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb07595c58fbf4fff"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research NVIDIA supplier economics and customer financing (2026-10-08)
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8ed2ba7de43a4fc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R71eae90b20f349ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Reafb317659514057"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R96fc4fe1b32e4ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R281b877273e045db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R8c2edcf155df4fb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rbd80d087fdec42db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a5fc38919d04b4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R8c6a88a63ad249ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rfa99c586a67e400a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R1ea7ed8cf6a149cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R1ee6f0d044034f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R6a4a9e9f8b9d4856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R2688a68d01b24c6f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I155" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I164" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1152,9 +1152,9 @@
       <x:c r="G28" s="61"/>
       <x:c r="H28" s="61"/>
     </x:row>
-    <x:row r="29" ht="68" customHeight="1">
+    <x:row r="29" ht="110" customHeight="1">
       <x:c r="A29" s="62" t="str">
-        <x:v>Rubin raises NVIDIA content per IT-load GW from $25B to $40B, about 60%. Operator revenue/GW must rise comparably to preserve gross-revenue payback. If revenue/GW stays flat again, vendor economics strengthen while operator replacement economics deteriorate.</x:v>
+        <x:v>NVIDIA claims $25B Blackwell / $40B Rubin per stated GW; the IT boundary is unverified. The 60% increase concerns supplier content only. Matching component capital/revenue requires comparable growth; whole-project cash payback also needs opex, financing, utilization and replacement life.</x:v>
       </x:c>
       <x:c r="B29" s="62"/>
       <x:c r="C29" s="62"/>
@@ -1871,26 +1871,18 @@
         <x:v>VENDOR-NVDA</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
-        <x:v>Generation anchors</x:v>
+        <x:v>Generation guidance 2026-08-26; review 2026-10-08</x:v>
       </x:c>
       <x:c r="D16" s="27"/>
       <x:c r="E16" s="29"/>
       <x:c r="F16" s="31"/>
-      <x:c r="G16" s="33" t="n">
-        <x:v>1000</x:v>
-      </x:c>
+      <x:c r="G16" s="33"/>
       <x:c r="H16" s="23" t="str">
-        <x:v>IT load</x:v>
-      </x:c>
-      <x:c r="I16" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J16" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K16" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="I16" s="35"/>
+      <x:c r="J16" s="35"/>
+      <x:c r="K16" s="35"/>
       <x:c r="L16" s="35"/>
       <x:c r="M16" s="19" t="str">
         <x:v>SRC-NVDA-Q2FY27-001</x:v>
@@ -1899,14 +1891,13 @@
         <x:v>VENDOR ONLY</x:v>
       </x:c>
       <x:c r="O16" s="43" t="str">
-        <x:v>Use silicon content per GW; not operator revenue per MW</x:v>
+        <x:v>Supplier PUE not_applicable; 18/25/40B per stated GW opportunities are not verified IT-GW or annual operator revenue; PORTS guarantee density separate</x:v>
       </x:c>
       <x:c r="P16" s="37" t="str">
         <x:f>IF(OR(D16="",E16="",F16=""),"",D16*E16*F16)</x:f>
       </x:c>
-      <x:c r="Q16" s="39" t="n">
+      <x:c r="Q16" s="39" t="str">
         <x:f>IF(G16="","",IF(H16="IT load",G16,IF(H16="Facility power",IF(I16="","",G16/I16),IF(H16="Generation",IF(OR(I16="",J16="",K16=""),"",G16*J16*K16/I16),IF(H16="Effective utilized IT",G16,"")))))</x:f>
-        <x:v>1000</x:v>
       </x:c>
       <x:c r="R16" s="39" t="str">
         <x:f>IF(Q16="","",IF(H16="Effective utilized IT",Q16,IF(L16="","",Q16*L16)))</x:f>
@@ -2402,13 +2393,13 @@
         <x:v>Accelerator networking and systems content</x:v>
       </x:c>
       <x:c r="E16" s="43" t="str">
-        <x:v>Deployed IT-load GW</x:v>
+        <x:v>Verified deployed IT GW; otherwise stated GW separately</x:v>
       </x:c>
       <x:c r="F16" s="43" t="str">
-        <x:v>Generation-specific content ladder is not operator revenue</x:v>
+        <x:v>PUE not_applicable; isolate supplier content from recurring revenue and contingent guarantees</x:v>
       </x:c>
       <x:c r="G16" s="43" t="str">
-        <x:v>Vendor anchor</x:v>
+        <x:v>Partial2026-10-08; generation power scope open</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2483,7 +2474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d6db8cc5a3d4855"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad73596e28a640d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3455,7 +3446,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R034de1b3870942ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3ffda1859764b9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3499,7 +3490,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>All figures are per IT-load GW. Facility cost remains project-specific.</x:v>
+        <x:v>Numeric columns require verified IT-load GW; scope-unresolved supplier claims remain in notes.</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -3660,9 +3651,7 @@
       <x:c r="B8" s="19" t="str">
         <x:v>Hopper</x:v>
       </x:c>
-      <x:c r="C8" s="54" t="n">
-        <x:v>18</x:v>
-      </x:c>
+      <x:c r="C8" s="54"/>
       <x:c r="D8" s="54"/>
       <x:c r="E8" s="54"/>
       <x:c r="F8" s="54"/>
@@ -3671,10 +3660,10 @@
         <x:v>SRC-NVDA-Q2FY27-001</x:v>
       </x:c>
       <x:c r="I8" s="19" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Company claim</x:v>
       </x:c>
       <x:c r="J8" s="43" t="str">
-        <x:v>VENDOR content only</x:v>
+        <x:v>$18B per stated GW supplier opportunity; IT/facility boundary unstated. IT-normalized numeric cell intentionally blank; not annual revenue.</x:v>
       </x:c>
       <x:c r="K8" s="56" t="str">
         <x:f>IF(OR(E8="",G8="",G8=0),"",E8/G8)</x:f>
@@ -3690,9 +3679,7 @@
       <x:c r="B9" s="19" t="str">
         <x:v>Blackwell</x:v>
       </x:c>
-      <x:c r="C9" s="54" t="n">
-        <x:v>25</x:v>
-      </x:c>
+      <x:c r="C9" s="54"/>
       <x:c r="D9" s="54"/>
       <x:c r="E9" s="54"/>
       <x:c r="F9" s="54"/>
@@ -3701,10 +3688,10 @@
         <x:v>SRC-NVDA-Q2FY27-001</x:v>
       </x:c>
       <x:c r="I9" s="19" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Company claim</x:v>
       </x:c>
       <x:c r="J9" s="43" t="str">
-        <x:v>VENDOR content only</x:v>
+        <x:v>$25B per stated GW supplier opportunity; IT/facility boundary unstated. IT-normalized numeric cell intentionally blank; not annual revenue.</x:v>
       </x:c>
       <x:c r="K9" s="56" t="str">
         <x:f>IF(OR(E9="",G9="",G9=0),"",E9/G9)</x:f>
@@ -3720,9 +3707,7 @@
       <x:c r="B10" s="19" t="str">
         <x:v>Vera Rubin</x:v>
       </x:c>
-      <x:c r="C10" s="54" t="n">
-        <x:v>40</x:v>
-      </x:c>
+      <x:c r="C10" s="54"/>
       <x:c r="D10" s="54"/>
       <x:c r="E10" s="54"/>
       <x:c r="F10" s="54"/>
@@ -3731,10 +3716,10 @@
         <x:v>SRC-NVDA-Q2FY27-001</x:v>
       </x:c>
       <x:c r="I10" s="19" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Company claim</x:v>
       </x:c>
       <x:c r="J10" s="43" t="str">
-        <x:v>VENDOR content only</x:v>
+        <x:v>$40B per stated GW supplier opportunity; IT/facility boundary unstated. IT-normalized numeric cell intentionally blank; not annual revenue.</x:v>
       </x:c>
       <x:c r="K10" s="56" t="str">
         <x:f>IF(OR(E10="",G10="",G10=0),"",E10/G10)</x:f>
@@ -4162,16 +4147,16 @@
         <x:v>Transcript</x:v>
       </x:c>
       <x:c r="F13" s="43" t="str">
-        <x:v>https://investor.nvidia.com/</x:v>
+        <x:v>https://investor.nvidia.com/files/content_files/TRANSCRIPT_-NVIDIA-Corp-NVDA-US-Q2-2027-Earnings-Call-26-August-2026-5_00-PM-ET.pdf</x:v>
       </x:c>
       <x:c r="G13" s="43" t="str">
         <x:v>Hopper Blackwell and Rubin content per GW</x:v>
       </x:c>
       <x:c r="H13" s="43" t="str">
-        <x:v>Primary</x:v>
+        <x:v>Primary read; scope qualified</x:v>
       </x:c>
       <x:c r="I13" s="43" t="str">
-        <x:v>Exact transcript URL to pin on refresh</x:v>
+        <x:v>Exact original pinned October 8. Management revenue opportunity per stated GW; call does not explicitly define IT versus facility boundary for ladder. Not realized annual cloud revenue.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -5793,7 +5778,7 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="I69" s="43" t="str">
-        <x:v>Item 1.01 Dell order and guarantee; Exhibit 99.1 NVIDIA contract</x:v>
+        <x:v>Re-read 8-K Item1.01 and Ex99.1: guarantee is IREN parent for its subsidiary, not NVIDIA. This exhibit describes an unnamed $3.4B customer contract and does not identify 60MW or NVIDIA as the customer; prior locator/title alone cannot establish those claims. See SRC-IREN-DELL-EX991-20260526.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -8236,38 +8221,299 @@
       </x:c>
     </x:row>
     <x:row r="155">
-      <x:c r="A155" s="20" t="str">
+      <x:c r="A155" s="19" t="str">
         <x:v>SRC-FT-JUPITER-20260924</x:v>
       </x:c>
-      <x:c r="B155" s="46" t="d">
+      <x:c r="B155" s="45" t="d">
         <x:v>2026-09-24T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C155" s="20" t="str">
+      <x:c r="C155" s="19" t="str">
         <x:v>Financial Times Alphaville</x:v>
       </x:c>
-      <x:c r="D155" s="44" t="str">
+      <x:c r="D155" s="43" t="str">
         <x:v>Oracle's New Mexico data-centre financing comes under pressure</x:v>
       </x:c>
-      <x:c r="E155" s="44" t="str">
+      <x:c r="E155" s="43" t="str">
         <x:v>secondary_financing_report</x:v>
       </x:c>
-      <x:c r="F155" s="44" t="str">
+      <x:c r="F155" s="43" t="str">
         <x:v>https://www.ft.com/content/82dbd39c-f8dd-4ef1-8a80-d430a22579bd</x:v>
       </x:c>
-      <x:c r="G155" s="44" t="str">
+      <x:c r="G155" s="43" t="str">
         <x:v>OpenAI / Stargate review 2026-10-07</x:v>
       </x:c>
-      <x:c r="H155" s="44" t="str">
+      <x:c r="H155" s="43" t="str">
         <x:v>Secondary read</x:v>
       </x:c>
-      <x:c r="I155" s="44" t="str">
+      <x:c r="I155" s="43" t="str">
         <x:v>Approx. $18B loans reported at 89-91; not independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="19" t="str">
+        <x:v>SRC-NVDA-10K-FY26</x:v>
+      </x:c>
+      <x:c r="B156" s="45" t="d">
+        <x:v>2026-02-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C156" s="19" t="str">
+        <x:v>NVIDIA / SEC</x:v>
+      </x:c>
+      <x:c r="D156" s="43" t="str">
+        <x:v>FY2026 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E156" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F156" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1045810/000104581026000021/nvda-20260125.htm</x:v>
+      </x:c>
+      <x:c r="G156" s="43" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H156" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I156" s="43" t="str">
+        <x:v>Note 10 p69 facility guarantees; Note 12 p70 commitments; Item 8 financial statements</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" s="19" t="str">
+        <x:v>SRC-NVDA-10Q-Q2FY27</x:v>
+      </x:c>
+      <x:c r="B157" s="45" t="d">
+        <x:v>2026-08-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C157" s="19" t="str">
+        <x:v>NVIDIA / SEC</x:v>
+      </x:c>
+      <x:c r="D157" s="43" t="str">
+        <x:v>Q2 FY2027 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E157" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F157" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1045810/000104581026000075/nvda-20260726.htm</x:v>
+      </x:c>
+      <x:c r="G157" s="43" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H157" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I157" s="43" t="str">
+        <x:v>Notes 6-10 pp13-19; MD&amp;A pp25-27; Item 6 p42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" s="19" t="str">
+        <x:v>SRC-NVDA-CFO-Q2FY27</x:v>
+      </x:c>
+      <x:c r="B158" s="45" t="d">
+        <x:v>2026-08-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C158" s="19" t="str">
+        <x:v>NVIDIA / SEC</x:v>
+      </x:c>
+      <x:c r="D158" s="43" t="str">
+        <x:v>Q2 FY2027 CFO commentary</x:v>
+      </x:c>
+      <x:c r="E158" s="43" t="str">
+        <x:v>8-K exhibit</x:v>
+      </x:c>
+      <x:c r="F158" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1045810/000104581026000073/q2fy27cfocommentary.htm</x:v>
+      </x:c>
+      <x:c r="G158" s="43" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H158" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I158" s="43" t="str">
+        <x:v>Revenue by Market Platform; Commitments; Additional Commitments; Guarantees; Balance Sheet and Cash Flow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" s="19" t="str">
+        <x:v>SRC-NVDA-PORTS-20260817</x:v>
+      </x:c>
+      <x:c r="B159" s="45" t="d">
+        <x:v>2026-08-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C159" s="19" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="D159" s="43" t="str">
+        <x:v>PORTS-Pike credit support announcement</x:v>
+      </x:c>
+      <x:c r="E159" s="43" t="str">
+        <x:v>issuer_release</x:v>
+      </x:c>
+      <x:c r="F159" s="43" t="str">
+        <x:v>https://investor.nvidia.com/news/press-release-details/2026/NVIDIA-Guarantees-SB-Energys-PORTS-Pike-Technology-Campus-in-Ohio-to-Exclusively-Host-NVIDIA-AI-Compute/default.aspx</x:v>
+      </x:c>
+      <x:c r="G159" s="43" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H159" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I159" s="43" t="str">
+        <x:v>News Summary and opening paragraphs; initial 4.25 IT-GW and optional 3.75 IT-GW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" s="19" t="str">
+        <x:v>SRC-NVDA-FINANCE-MOU-20260810</x:v>
+      </x:c>
+      <x:c r="B160" s="45" t="d">
+        <x:v>2026-08-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C160" s="19" t="str">
+        <x:v>Blackstone / NVIDIA</x:v>
+      </x:c>
+      <x:c r="D160" s="43" t="str">
+        <x:v>Independent AI compute financing platform MOUs</x:v>
+      </x:c>
+      <x:c r="E160" s="43" t="str">
+        <x:v>counterparty_release</x:v>
+      </x:c>
+      <x:c r="F160" s="43" t="str">
+        <x:v>https://www.blackstone.com/news/press/nvidia-partners-with-apollo-blackrock-blackstone-brookfield-goldman-sachs-and-kkr-to-establish-ai-compute-infrastructure-financing-platforms-to-mobilize-over-500-billion-of-third-party-capital/</x:v>
+      </x:c>
+      <x:c r="G160" s="43" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H160" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I160" s="43" t="str">
+        <x:v>Opening three paragraphs; Forward-Looking Statements</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" s="19" t="str">
+        <x:v>SRC-NVDA-NOTES-20260618</x:v>
+      </x:c>
+      <x:c r="B161" s="45" t="d">
+        <x:v>2026-06-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C161" s="19" t="str">
+        <x:v>NVIDIA / SEC</x:v>
+      </x:c>
+      <x:c r="D161" s="43" t="str">
+        <x:v>Officers certificate and seven note forms</x:v>
+      </x:c>
+      <x:c r="E161" s="43" t="str">
+        <x:v>8-K exhibit 4.2</x:v>
+      </x:c>
+      <x:c r="F161" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1045810/000119312526275783/d48176dex42.htm</x:v>
+      </x:c>
+      <x:c r="G161" s="43" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H161" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I161" s="43" t="str">
+        <x:v>Sections establishing each series: Initial Aggregate Principal Amount, Maturity, Rate of Interest; Annexes A-G</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="19" t="str">
+        <x:v>SRC-NVDA-EARNINGS-Q2FY27</x:v>
+      </x:c>
+      <x:c r="B162" s="45" t="d">
+        <x:v>2026-08-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C162" s="19" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="D162" s="43" t="str">
+        <x:v>Q2 FY2027 financial results</x:v>
+      </x:c>
+      <x:c r="E162" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F162" s="43" t="str">
+        <x:v>https://investor.nvidia.com/news/press-release-details/2026/NVIDIA-Announces-Financial-Results-for-Second-Quarter-Fiscal-2027/default.aspx</x:v>
+      </x:c>
+      <x:c r="G162" s="43" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H162" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I162" s="43" t="str">
+        <x:v>Opening results; Q2 summary; cash-flow statement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="19" t="str">
+        <x:v>SRC-NVDA-EARNINGS-FY26</x:v>
+      </x:c>
+      <x:c r="B163" s="45" t="d">
+        <x:v>2026-02-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C163" s="19" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="D163" s="43" t="str">
+        <x:v>Q4 and FY2026 financial results</x:v>
+      </x:c>
+      <x:c r="E163" s="43" t="str">
+        <x:v>earnings_release</x:v>
+      </x:c>
+      <x:c r="F163" s="43" t="str">
+        <x:v>https://investor.nvidia.com/news/press-release-details/2026/NVIDIA-Announces-Financial-Results-for-Fourth-Quarter-and-Fiscal-2026/</x:v>
+      </x:c>
+      <x:c r="G163" s="43" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H163" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I163" s="43" t="str">
+        <x:v>Fiscal 2026 Summary; Data Center highlights</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" s="20" t="str">
+        <x:v>SRC-IREN-DELL-EX991-20260526</x:v>
+      </x:c>
+      <x:c r="B164" s="46" t="d">
+        <x:v>2026-05-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C164" s="20" t="str">
+        <x:v>IREN / SEC</x:v>
+      </x:c>
+      <x:c r="D164" s="44" t="str">
+        <x:v>Dell Blackwell deployment at Childress</x:v>
+      </x:c>
+      <x:c r="E164" s="44" t="str">
+        <x:v>8-K exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="F164" s="44" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000030/irentrgts44bninarrwithbl.htm</x:v>
+      </x:c>
+      <x:c r="G164" s="44" t="str">
+        <x:v>NVIDIA supplier economics and financing</x:v>
+      </x:c>
+      <x:c r="H164" s="44" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I164" s="44" t="str">
+        <x:v>Ex99.1 pp1-2; related 8-K Item1.01: IREN parent guarantees subsidiary Dell obligations</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb07595c58fbf4fff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R070ca4829cd643e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research Palantir cloud commitments and software MW boundaries
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a5fc38919d04b4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R8c6a88a63ad249ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rfa99c586a67e400a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R1ea7ed8cf6a149cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R1ee6f0d044034f2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R6a4a9e9f8b9d4856"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R2688a68d01b24c6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R622505dd11384eaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rf1824ba6b2534017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R44b3f18795ec405d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rd8f3833de5a24437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R743bdc6f50cf47f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rf56c81c5f7584230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rd03a833525ae40d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I164" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I189" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -704,10 +704,11 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="19" t="str">
-        <x:v>Nscale recognized revenue ($M / effective MW-year)</x:v>
-      </x:c>
-      <x:c r="B8" s="58" t="str">
-        <x:f>'Company Models'!S13</x:f>
+        <x:v>Bloom Q2 revenue ($B)</x:v>
+      </x:c>
+      <x:c r="B8" s="54" t="n">
+        <x:f>1.065365</x:f>
+        <x:v>1.065365</x:v>
       </x:c>
       <x:c r="D8" s="19" t="str">
         <x:v>Nscale / Anthropic</x:v>
@@ -1154,7 +1155,7 @@
     </x:row>
     <x:row r="29" ht="110" customHeight="1">
       <x:c r="A29" s="62" t="str">
-        <x:v>NVIDIA claims $25B Blackwell / $40B Rubin per stated GW; the IT boundary is unverified. The 60% increase concerns supplier content only. Matching component capital/revenue requires comparable growth; whole-project cash payback also needs opex, financing, utilization and replacement life.</x:v>
+        <x:v>Bloom's Nebius agreement implies an aggregate upper bound of $1.04M per guaranteed generation MW-year ($0.793M per installed generation MW-year), not operator revenue per IT MW. Q2 revenue was $1.065B and 73% came from one non-related contractual customer, which can be a project-finance affiliate. Keep the $25B Brookfield framework, project financing, recognized revenue and generation capacity separate; supplier PUE is not applicable.</x:v>
       </x:c>
       <x:c r="B29" s="62"/>
       <x:c r="C29" s="62"/>
@@ -1918,42 +1919,35 @@
         <x:v>VENDOR-AVGO</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="D17" s="27"/>
+        <x:v>Q3 FY2026</x:v>
+      </x:c>
+      <x:c r="D17" s="27" t="n">
+        <x:v>16700000000</x:v>
+      </x:c>
       <x:c r="E17" s="29"/>
-      <x:c r="F17" s="31"/>
-      <x:c r="G17" s="33" t="n">
-        <x:v>1000</x:v>
-      </x:c>
-      <x:c r="H17" s="23" t="str">
-        <x:v>IT load</x:v>
-      </x:c>
-      <x:c r="I17" s="35" t="n">
+      <x:c r="F17" s="31" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J17" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K17" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="G17" s="33"/>
+      <x:c r="H17" s="23"/>
+      <x:c r="I17" s="35"/>
+      <x:c r="J17" s="35"/>
+      <x:c r="K17" s="35"/>
       <x:c r="L17" s="35"/>
       <x:c r="M17" s="19" t="str">
-        <x:v>SRC-WB-P2S-001</x:v>
+        <x:v>SRC-AVGO-EARNINGS-Q3FY26</x:v>
       </x:c>
       <x:c r="N17" s="19" t="str">
         <x:v>VENDOR ONLY</x:v>
       </x:c>
       <x:c r="O17" s="43" t="str">
-        <x:v>Custom silicon only; architecture mix required</x:v>
+        <x:v>Reported AI semiconductor revenue combines custom accelerators and networking. Matched period-average deployed IT-load GW, delivery cohort, architecture split and physical utilization are not disclosed; supplier PUE is not applicable.</x:v>
       </x:c>
       <x:c r="P17" s="37" t="str">
         <x:f>IF(OR(D17="",E17="",F17=""),"",D17*E17*F17)</x:f>
       </x:c>
-      <x:c r="Q17" s="39" t="n">
+      <x:c r="Q17" s="39" t="str">
         <x:f>IF(G17="","",IF(H17="IT load",G17,IF(H17="Facility power",IF(I17="","",G17/I17),IF(H17="Generation",IF(OR(I17="",J17="",K17=""),"",G17*J17*K17/I17),IF(H17="Effective utilized IT",G17,"")))))</x:f>
-        <x:v>1000</x:v>
       </x:c>
       <x:c r="R17" s="39" t="str">
         <x:f>IF(Q17="","",IF(H17="Effective utilized IT",Q17,IF(L17="","",Q17*L17)))</x:f>
@@ -1974,25 +1968,29 @@
         <x:v>SUPPLIER-BLOOM</x:v>
       </x:c>
       <x:c r="C18" s="19" t="str">
-        <x:v>Not reviewed</x:v>
+        <x:v>Nebius Capacity Agreement / review 2026-10-10</x:v>
       </x:c>
       <x:c r="D18" s="27"/>
       <x:c r="E18" s="29"/>
       <x:c r="F18" s="31"/>
-      <x:c r="G18" s="33"/>
-      <x:c r="H18" s="23"/>
+      <x:c r="G18" s="33" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="str">
+        <x:v>Guaranteed generation</x:v>
+      </x:c>
       <x:c r="I18" s="35"/>
       <x:c r="J18" s="35"/>
       <x:c r="K18" s="35"/>
       <x:c r="L18" s="35"/>
       <x:c r="M18" s="19" t="str">
-        <x:v>SRC-NBIS-BLOOM-CONTRACT</x:v>
+        <x:v>SRC-NBIS-BE-CAPACITY-20260520</x:v>
       </x:c>
       <x:c r="N18" s="19" t="str">
         <x:v>VENDOR ONLY</x:v>
       </x:c>
       <x:c r="O18" s="43" t="str">
-        <x:v>Power supplier; PUE not applicable; queued via Nebius agreement.</x:v>
+        <x:v>Upper bound $1.04M per guaranteed generation MW-year and $0.793M per installed generation MW-year over disclosed 10-year terms. This is supplier capacity-service economics, not recognized revenue per IT MW. Supplier PUE not_applicable; customer PUE, IT load, utilization, phase timing and fuel/pass-through terms are not disclosed.</x:v>
       </x:c>
       <x:c r="P18" s="37" t="str">
         <x:f>IF(OR(D18="",E18="",F18=""),"",D18*E18*F18)</x:f>
@@ -2019,7 +2017,7 @@
         <x:v>SOFTWARE-PLTR</x:v>
       </x:c>
       <x:c r="C19" s="20" t="str">
-        <x:v>Not reviewed</x:v>
+        <x:v>Q2 2026; reviewed 2026-10-11</x:v>
       </x:c>
       <x:c r="D19" s="28"/>
       <x:c r="E19" s="30"/>
@@ -2031,13 +2029,13 @@
       <x:c r="K19" s="36"/>
       <x:c r="L19" s="36"/>
       <x:c r="M19" s="20" t="str">
-        <x:v>SRC-NBIS-PALANTIR-20260908</x:v>
+        <x:v>SRC-PLTR-10Q-Q2FY26</x:v>
       </x:c>
       <x:c r="N19" s="20" t="str">
         <x:v>VENDOR ONLY</x:v>
       </x:c>
       <x:c r="O19" s="44" t="str">
-        <x:v>Software attribution; own PUE not applicable; queued via Nebius partnership.</x:v>
+        <x:v>Partial software review. AI revenue and active customer IT MW/utilization missing. Supplier PUE not applicable. $5.6B cloud minimum through Feb 2036 is spend, not MW or revenue.</x:v>
       </x:c>
       <x:c r="P19" s="38" t="str">
         <x:f>IF(OR(D19="",E19="",F19=""),"",D19*E19*F19)</x:f>
@@ -2350,10 +2348,10 @@
         <x:v>Time-weighted external allocated IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F14" s="43" t="str">
-        <x:v>Use reported nameplate compute draw only as an IT-load exit metric; exclude internal Grok and non-cloud AI revenue; keep PUE guidance contracted sales and realized revenue separate</x:v>
+        <x:v>Use reported nameplate compute draw only as an IT-load exit metric; exclude internal Grok and non-cloud AI revenue; keep PUE, guidance, contracted sales, realized revenue, and secondary deal-level $/MW estimates separate; preserve GPU generation, tenor, termination rights, service bundle and power boundary</x:v>
       </x:c>
       <x:c r="G14" s="43" t="str">
-        <x:v>Partial 2026-10-06; recognized new-cloud revenue and nameplate bounds established; external allocation and utilization open</x:v>
+        <x:v>Partial 2026-10-10; Q2 recognized-revenue model unchanged; secondary SpaceX deal/generation curve added; external allocation, utilization and PUE remain open</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2413,16 +2411,16 @@
         <x:v>Silicon vendor</x:v>
       </x:c>
       <x:c r="D17" s="43" t="str">
-        <x:v>Custom accelerator and networking revenue attributable to capacity</x:v>
+        <x:v>Recognized AI semiconductor revenue for the matched delivery cohort</x:v>
       </x:c>
       <x:c r="E17" s="43" t="str">
-        <x:v>Deployed IT-load GW</x:v>
+        <x:v>Matched deployed IT-load GW for the same cohort</x:v>
       </x:c>
       <x:c r="F17" s="43" t="str">
-        <x:v>Preserve custom-only perimeter and architecture mix</x:v>
+        <x:v>Separate custom accelerators and networking where disclosed; exclude non-AI semiconductors and pass-through rack content</x:v>
       </x:c>
       <x:c r="G17" s="43" t="str">
-        <x:v>Configured; inputs partial</x:v>
+        <x:v>Partial 2026-10-09; Q3 AI revenue verified; matched IT-load denominator open</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2436,16 +2434,16 @@
         <x:v>Power supplier</x:v>
       </x:c>
       <x:c r="D18" s="43" t="str">
-        <x:v>Attributable capacity service fees</x:v>
+        <x:v>Aggregate capacity-service fees for the matched service term</x:v>
       </x:c>
       <x:c r="E18" s="43" t="str">
-        <x:v>Guaranteed generation MW service-years</x:v>
+        <x:v>Guaranteed generation MW-service-years</x:v>
       </x:c>
       <x:c r="F18" s="43" t="str">
-        <x:v>Fuel and generation scope; not operator revenue; PUE not applicable</x:v>
+        <x:v>Use phase-specific guaranteed generation MW and service years; keep recognized product revenue, financing frameworks, fuel pass-through, unexercised master volumes and customer IT economics separate; supplier PUE not_applicable; installed/guaranteed ratio is not PUE or utilization</x:v>
       </x:c>
       <x:c r="G18" s="43" t="str">
-        <x:v>Queued; not reviewed</x:v>
+        <x:v>Partial 2026-10-10; Nebius upper bound $1.04M per guaranteed generation MW-year; phase activation, fuel terms and realized revenue open</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2459,22 +2457,22 @@
         <x:v>Software</x:v>
       </x:c>
       <x:c r="D19" s="44" t="str">
-        <x:v>Attributed incremental AI software revenue</x:v>
+        <x:v>Annualized attributable incremental AI software revenue; exclude compute and hardware pass-through</x:v>
       </x:c>
       <x:c r="E19" s="44" t="str">
-        <x:v>Matching associated average IT MW</x:v>
+        <x:v>Period-average associated active customer IT MW; separately model physical utilization</x:v>
       </x:c>
       <x:c r="F19" s="44" t="str">
-        <x:v>No total-company revenue; separate third-party compute</x:v>
+        <x:v>Separate hosted and customer-hosted software; exclude R&amp;D and pilot compute; own PUE not applicable; do not convert minimum cloud spend into MW</x:v>
       </x:c>
       <x:c r="G19" s="44" t="str">
-        <x:v>Queued; not reviewed</x:v>
+        <x:v>Partial 2026-10-11; revenue attribution and active IT-MW cohorts unavailable</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad73596e28a640d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9506ee048adb424a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3446,7 +3444,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3ffda1859764b9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34de0e430cb84fff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3765,25 +3763,21 @@
         <x:v>XPV</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>Unspecified</x:v>
-      </x:c>
-      <x:c r="C12" s="54" t="n">
-        <x:v>35</x:v>
-      </x:c>
+        <x:v>Anthropic / Fluidstack</x:v>
+      </x:c>
+      <x:c r="C12" s="54"/>
       <x:c r="D12" s="54"/>
-      <x:c r="E12" s="54" t="n">
-        <x:v>35</x:v>
-      </x:c>
+      <x:c r="E12" s="54"/>
       <x:c r="F12" s="54"/>
       <x:c r="G12" s="54"/>
       <x:c r="H12" s="19" t="str">
-        <x:v>SRC-WB-P2S-001</x:v>
+        <x:v>SRC-AVGO-XPV-20260609</x:v>
       </x:c>
       <x:c r="I12" s="19" t="str">
-        <x:v>Derived</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="J12" s="43" t="str">
-        <x:v>All-in tranche figure; perimeter needs continuing review</x:v>
+        <x:v>$35B capital solution for more than 1 stated compute GW; financing transaction, not supplier content, facility cost or recognized revenue. Exact power boundary and cost allocation remain open.</x:v>
       </x:c>
       <x:c r="K12" s="56" t="str">
         <x:f>IF(OR(E12="",G12="",G12=0),"",E12/G12)</x:f>
@@ -3797,23 +3791,21 @@
         <x:v>Broadcom</x:v>
       </x:c>
       <x:c r="B13" s="20" t="str">
-        <x:v>Custom silicon</x:v>
-      </x:c>
-      <x:c r="C13" s="55" t="n">
-        <x:v>11.5</x:v>
-      </x:c>
+        <x:v>Custom accelerators and networking</x:v>
+      </x:c>
+      <x:c r="C13" s="55"/>
       <x:c r="D13" s="55"/>
       <x:c r="E13" s="55"/>
       <x:c r="F13" s="55"/>
       <x:c r="G13" s="55"/>
       <x:c r="H13" s="20" t="str">
-        <x:v>SRC-WB-P2S-001</x:v>
+        <x:v>SRC-AVGO-EARNINGS-Q3FY26</x:v>
       </x:c>
       <x:c r="I13" s="20" t="str">
-        <x:v>Derived</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="J13" s="44" t="str">
-        <x:v>Custom silicon only</x:v>
+        <x:v>Q3 AI semiconductor revenue is reported, but matched deployed IT-load GW and architecture mix are not disclosed; prior compiled numeric anchor superseded.</x:v>
       </x:c>
       <x:c r="K13" s="57" t="str">
         <x:f>IF(OR(E13="",G13="",G13=0),"",E13/G13)</x:f>
@@ -8482,38 +8474,761 @@
       </x:c>
     </x:row>
     <x:row r="164">
-      <x:c r="A164" s="20" t="str">
+      <x:c r="A164" s="19" t="str">
         <x:v>SRC-IREN-DELL-EX991-20260526</x:v>
       </x:c>
-      <x:c r="B164" s="46" t="d">
+      <x:c r="B164" s="45" t="d">
         <x:v>2026-05-26T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C164" s="20" t="str">
+      <x:c r="C164" s="19" t="str">
         <x:v>IREN / SEC</x:v>
       </x:c>
-      <x:c r="D164" s="44" t="str">
+      <x:c r="D164" s="43" t="str">
         <x:v>Dell Blackwell deployment at Childress</x:v>
       </x:c>
-      <x:c r="E164" s="44" t="str">
+      <x:c r="E164" s="43" t="str">
         <x:v>8-K exhibit 99.1</x:v>
       </x:c>
-      <x:c r="F164" s="44" t="str">
+      <x:c r="F164" s="43" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000187884826000030/irentrgts44bninarrwithbl.htm</x:v>
       </x:c>
-      <x:c r="G164" s="44" t="str">
+      <x:c r="G164" s="43" t="str">
         <x:v>NVIDIA supplier economics and financing</x:v>
       </x:c>
-      <x:c r="H164" s="44" t="str">
+      <x:c r="H164" s="43" t="str">
         <x:v>Primary read</x:v>
       </x:c>
-      <x:c r="I164" s="44" t="str">
+      <x:c r="I164" s="43" t="str">
         <x:v>Ex99.1 pp1-2; related 8-K Item1.01: IREN parent guarantees subsidiary Dell obligations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="19" t="str">
+        <x:v>SRC-XAI-DB-ZH-20261010</x:v>
+      </x:c>
+      <x:c r="B165" s="45" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C165" s="19" t="str">
+        <x:v>Deutsche Bank Research / ZeroHedge excerpt supplied by user</x:v>
+      </x:c>
+      <x:c r="D165" s="43" t="str">
+        <x:v>SpaceX compute capacity, neocloud deal economics, and annual revenue per GW figures</x:v>
+      </x:c>
+      <x:c r="E165" s="43" t="str">
+        <x:v>User-supplied research screenshots</x:v>
+      </x:c>
+      <x:c r="F165" s="43"/>
+      <x:c r="G165" s="43" t="str">
+        <x:v>xAI / SpaceX compute curve; generation density; hosting $/MW; time-to-MW</x:v>
+      </x:c>
+      <x:c r="H165" s="43" t="str">
+        <x:v>Attributed secondary excerpt</x:v>
+      </x:c>
+      <x:c r="I165" s="43" t="str">
+        <x:v>Raw transcription in raw/2026-10-10-spacex-db-compute-curve.md; underlying bank notes not independently accessed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="19" t="str">
+        <x:v>SRC-AVGO-10K-FY25</x:v>
+      </x:c>
+      <x:c r="B166" s="45" t="d">
+        <x:v>2025-12-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C166" s="19" t="str">
+        <x:v>Broadcom / SEC</x:v>
+      </x:c>
+      <x:c r="D166" s="43" t="str">
+        <x:v>Broadcom fiscal 2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E166" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F166" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1730168/000173016825000121/avgo-20251102.htm</x:v>
+      </x:c>
+      <x:c r="G166" s="43" t="str">
+        <x:v>Broadcom supplier economics and contract baseline</x:v>
+      </x:c>
+      <x:c r="H166" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I166" s="43" t="str">
+        <x:v>Business AI perimeter pp4-7; Risk Factors pp16-19; Note 3 RPO p59; Note 14 commitments and concentration p85</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="19" t="str">
+        <x:v>SRC-AVGO-10Q-Q3FY26</x:v>
+      </x:c>
+      <x:c r="B167" s="45" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C167" s="19" t="str">
+        <x:v>Broadcom / SEC</x:v>
+      </x:c>
+      <x:c r="D167" s="43" t="str">
+        <x:v>Broadcom Q3 fiscal 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E167" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F167" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1730168/000173016826000080/avgo-20260802.htm</x:v>
+      </x:c>
+      <x:c r="G167" s="43" t="str">
+        <x:v>Broadcom supplier economics commitments and financing</x:v>
+      </x:c>
+      <x:c r="H167" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I167" s="43" t="str">
+        <x:v>Note 2 RPO pp9-10; Note 10 commitments guarantee and notes pp20-21; MD&amp;A pp27-31; Risk Factors pp36-43</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="19" t="str">
+        <x:v>SRC-AVGO-EARNINGS-Q3FY26</x:v>
+      </x:c>
+      <x:c r="B168" s="45" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C168" s="19" t="str">
+        <x:v>Broadcom / SEC</x:v>
+      </x:c>
+      <x:c r="D168" s="43" t="str">
+        <x:v>Broadcom Q3 fiscal 2026 financial results</x:v>
+      </x:c>
+      <x:c r="E168" s="43" t="str">
+        <x:v>8-K exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="F168" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1730168/000173016826000076/avgo-08022026x8kxex99.htm</x:v>
+      </x:c>
+      <x:c r="G168" s="43" t="str">
+        <x:v>Broadcom AI revenue and cash flow</x:v>
+      </x:c>
+      <x:c r="H168" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I168" s="43" t="str">
+        <x:v>Exhibit 99.1 pp1-3: AI semiconductor revenue segment revenue cash flow capex and Q4 guidance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="19" t="str">
+        <x:v>SRC-AVGO-XPV-20260609</x:v>
+      </x:c>
+      <x:c r="B169" s="45" t="d">
+        <x:v>2026-06-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C169" s="19" t="str">
+        <x:v>Broadcom</x:v>
+      </x:c>
+      <x:c r="D169" s="43" t="str">
+        <x:v>Broadcom Apollo and Blackstone AI XPV platform</x:v>
+      </x:c>
+      <x:c r="E169" s="43" t="str">
+        <x:v>issuer_release</x:v>
+      </x:c>
+      <x:c r="F169" s="43" t="str">
+        <x:v>https://investors.broadcom.com/news-releases/news-release-details/broadcom-apollo-and-blackstone-establish-landmark-strategic</x:v>
+      </x:c>
+      <x:c r="G169" s="43" t="str">
+        <x:v>Broadcom rack-financing platform and capacity</x:v>
+      </x:c>
+      <x:c r="H169" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I169" s="43" t="str">
+        <x:v>Opening: more than 20GW platform; $35B initial tranche for more than 1GW Anthropic capacity at Fluidstack</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="19" t="str">
+        <x:v>SRC-APOLLO-AVGO-XPV-20260609</x:v>
+      </x:c>
+      <x:c r="B170" s="45" t="d">
+        <x:v>2026-06-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C170" s="19" t="str">
+        <x:v>Apollo</x:v>
+      </x:c>
+      <x:c r="D170" s="43" t="str">
+        <x:v>Apollo-led $35 billion capital solution for Broadcom AI XPV platform</x:v>
+      </x:c>
+      <x:c r="E170" s="43" t="str">
+        <x:v>counterparty_release</x:v>
+      </x:c>
+      <x:c r="F170" s="43" t="str">
+        <x:v>https://www.apollo.com/insights-news/pressreleases/2026/06/apollo-leads-35-billion-capital-solution-for-broadcom-ai-xpv-platform-in-partnership-with-blackstone-and-leading-global-banks-3308896</x:v>
+      </x:c>
+      <x:c r="G170" s="43" t="str">
+        <x:v>Broadcom rack-financing capital structure</x:v>
+      </x:c>
+      <x:c r="H170" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I170" s="43" t="str">
+        <x:v>Opening and advisor list: multi-year draw schedule more than 1GW Anthropic compute and bank roles</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="19" t="str">
+        <x:v>SRC-AVGO-META-20260414</x:v>
+      </x:c>
+      <x:c r="B171" s="45" t="d">
+        <x:v>2026-04-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C171" s="19" t="str">
+        <x:v>Broadcom / Meta</x:v>
+      </x:c>
+      <x:c r="D171" s="43" t="str">
+        <x:v>Extended MTIA partnership through 2029</x:v>
+      </x:c>
+      <x:c r="E171" s="43" t="str">
+        <x:v>issuer_counterparty_release</x:v>
+      </x:c>
+      <x:c r="F171" s="43" t="str">
+        <x:v>https://investors.broadcom.com/news-releases/news-release-details/broadcom-announces-extended-partnership-meta-deploy-technology</x:v>
+      </x:c>
+      <x:c r="G171" s="43" t="str">
+        <x:v>Broadcom future custom accelerator and networking deployments</x:v>
+      </x:c>
+      <x:c r="H171" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I171" s="43" t="str">
+        <x:v>Opening: 2nm MTIA; initial more-than-1GW commitment; XPU and Ethernet scope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="19" t="str">
+        <x:v>SRC-AVGO-OPENAI-20251013</x:v>
+      </x:c>
+      <x:c r="B172" s="45" t="d">
+        <x:v>2025-10-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C172" s="19" t="str">
+        <x:v>Broadcom / OpenAI</x:v>
+      </x:c>
+      <x:c r="D172" s="43" t="str">
+        <x:v>10GW OpenAI-designed accelerator collaboration</x:v>
+      </x:c>
+      <x:c r="E172" s="43" t="str">
+        <x:v>issuer_counterparty_release</x:v>
+      </x:c>
+      <x:c r="F172" s="43" t="str">
+        <x:v>https://investors.broadcom.com/news-releases/news-release-details/openai-and-broadcom-announce-strategic-collaboration-deploy-10</x:v>
+      </x:c>
+      <x:c r="G172" s="43" t="str">
+        <x:v>Broadcom future custom accelerator and networking deployments</x:v>
+      </x:c>
+      <x:c r="H172" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I172" s="43" t="str">
+        <x:v>Opening: accelerator and Ethernet systems; term sheet; rack delivery H2 2026 through end-2029</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="19" t="str">
+        <x:v>SRC-BE-10K-FY25</x:v>
+      </x:c>
+      <x:c r="B173" s="45" t="d">
+        <x:v>2026-02-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C173" s="19" t="str">
+        <x:v>Bloom Energy / SEC</x:v>
+      </x:c>
+      <x:c r="D173" s="43" t="str">
+        <x:v>Bloom Energy fiscal 2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E173" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F173" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1664703/000162828026006516/be-20251231.htm</x:v>
+      </x:c>
+      <x:c r="G173" s="43" t="str">
+        <x:v>Bloom supplier economics revenue concentration financing and commitments</x:v>
+      </x:c>
+      <x:c r="H173" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I173" s="43" t="str">
+        <x:v>Statements of Operations; Note 3 revenue concentration and RPO; Note 11 Fund JVs and Brookfield framework; debt and commitments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" s="19" t="str">
+        <x:v>SRC-BE-10QA-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B174" s="45" t="d">
+        <x:v>2026-07-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C174" s="19" t="str">
+        <x:v>Bloom Energy / SEC</x:v>
+      </x:c>
+      <x:c r="D174" s="43" t="str">
+        <x:v>Bloom Energy Q2 2026 Form 10-Q/A</x:v>
+      </x:c>
+      <x:c r="E174" s="43" t="str">
+        <x:v>10-Q/A</x:v>
+      </x:c>
+      <x:c r="F174" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1664703/000162828026050325/be-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G174" s="43" t="str">
+        <x:v>Bloom quarterly revenue concentration cash debt RPO JVs and Oracle warrant</x:v>
+      </x:c>
+      <x:c r="H174" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I174" s="43" t="str">
+        <x:v>Statements of Operations; Notes 3 11 12 and 13; liquidity and debt tables</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" s="19" t="str">
+        <x:v>SRC-BE-EARNINGS-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B175" s="45" t="d">
+        <x:v>2026-07-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C175" s="19" t="str">
+        <x:v>Bloom Energy / SEC</x:v>
+      </x:c>
+      <x:c r="D175" s="43" t="str">
+        <x:v>Bloom Energy Q2 2026 financial results</x:v>
+      </x:c>
+      <x:c r="E175" s="43" t="str">
+        <x:v>8-K exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="F175" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1664703/000162828026050150/ex991_q226financialresults.htm</x:v>
+      </x:c>
+      <x:c r="G175" s="43" t="str">
+        <x:v>Bloom quarterly results cash flow and guidance</x:v>
+      </x:c>
+      <x:c r="H175" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I175" s="43" t="str">
+        <x:v>Financial highlights revenue table cash-flow summary and fiscal 2026 outlook</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="19" t="str">
+        <x:v>SRC-NBIS-BE-CAPACITY-20260520</x:v>
+      </x:c>
+      <x:c r="B176" s="45" t="d">
+        <x:v>2026-05-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C176" s="19" t="str">
+        <x:v>Nebius / SEC</x:v>
+      </x:c>
+      <x:c r="D176" s="43" t="str">
+        <x:v>Nebius Capacity Agreement with Bloom Energy</x:v>
+      </x:c>
+      <x:c r="E176" s="43" t="str">
+        <x:v>6-K</x:v>
+      </x:c>
+      <x:c r="F176" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/0001965040/000121390026052737/ea0243376-6k_nebius.htm</x:v>
+      </x:c>
+      <x:c r="G176" s="43" t="str">
+        <x:v>Bloom contracted generation and capacity-service economics</x:v>
+      </x:c>
+      <x:c r="H176" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I176" s="43" t="str">
+        <x:v>Agreement entered May 14; three 10-year phases; about250MW guaranteed and328MW installed generation; up to2.6B aggregate service fees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="19" t="str">
+        <x:v>SRC-NBIS-BE-RELEASE-20260520</x:v>
+      </x:c>
+      <x:c r="B177" s="45" t="d">
+        <x:v>2026-05-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C177" s="19" t="str">
+        <x:v>Nebius</x:v>
+      </x:c>
+      <x:c r="D177" s="43" t="str">
+        <x:v>Nebius and Bloom Energy partner for AI infrastructure power</x:v>
+      </x:c>
+      <x:c r="E177" s="43" t="str">
+        <x:v>counterparty_release</x:v>
+      </x:c>
+      <x:c r="F177" s="43" t="str">
+        <x:v>https://nebius.com/newsroom/nebius-and-bloom-energy-partner-to-power-ai-infrastructure-build-out</x:v>
+      </x:c>
+      <x:c r="G177" s="43" t="str">
+        <x:v>Bloom deployment timing and behind-the-meter boundary</x:v>
+      </x:c>
+      <x:c r="H177" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I177" s="43" t="str">
+        <x:v>Opening:328MW installed behind-the-meter generation expected operational in 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="19" t="str">
+        <x:v>SRC-IDF-OAKTREE-BE-20260716</x:v>
+      </x:c>
+      <x:c r="B178" s="45" t="d">
+        <x:v>2026-07-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C178" s="19" t="str">
+        <x:v>IDF / Oaktree</x:v>
+      </x:c>
+      <x:c r="D178" s="43" t="str">
+        <x:v>$1.7 billion project investment for Bloom fuel cells serving Nebius</x:v>
+      </x:c>
+      <x:c r="E178" s="43" t="str">
+        <x:v>project_finance_release</x:v>
+      </x:c>
+      <x:c r="F178" s="43" t="str">
+        <x:v>https://www.prnewswire.com/news-releases/industrial-development-funding-and-oaktree-announce-1-7-billion-project-investment-in-bloom-energy-fuel-cells-for-nebius-ai-infrastructure-build-out-302827566.html</x:v>
+      </x:c>
+      <x:c r="G178" s="43" t="str">
+        <x:v>Bloom Nebius project-finance capital stack</x:v>
+      </x:c>
+      <x:c r="H178" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I178" s="43" t="str">
+        <x:v>IDF developer; Oaktree minority equity; Morgan Stanley tax equity and placement agent; MUFG senior debt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" s="19" t="str">
+        <x:v>SRC-BE-BROOKFIELD-20260630</x:v>
+      </x:c>
+      <x:c r="B179" s="45" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C179" s="19" t="str">
+        <x:v>Bloom Energy / Brookfield</x:v>
+      </x:c>
+      <x:c r="D179" s="43" t="str">
+        <x:v>Brookfield and Bloom expand AI infrastructure financing framework to $25 billion</x:v>
+      </x:c>
+      <x:c r="E179" s="43" t="str">
+        <x:v>issuer_release</x:v>
+      </x:c>
+      <x:c r="F179" s="43" t="str">
+        <x:v>https://investor.bloomenergy.com/press-releases/press-release-details/2026/Brookfield-and-Bloom-Energy-Expand-AI-Infrastructure-Partnership-to-25-Billion-Fivefold-Increase-to-Build-and-Finance-Rapid-Power-for-AI-Infrastructure/default.aspx</x:v>
+      </x:c>
+      <x:c r="G179" s="43" t="str">
+        <x:v>Bloom financing framework</x:v>
+      </x:c>
+      <x:c r="H179" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I179" s="43" t="str">
+        <x:v>Framework expanded from5B to25B over five years; not recognized revenue or RPO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" s="19" t="str">
+        <x:v>SRC-BE-ORCL-20260413</x:v>
+      </x:c>
+      <x:c r="B180" s="45" t="d">
+        <x:v>2026-04-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C180" s="19" t="str">
+        <x:v>Bloom Energy / Oracle</x:v>
+      </x:c>
+      <x:c r="D180" s="43" t="str">
+        <x:v>Bloom and Oracle expand strategic partnership to up to 2.8 GW</x:v>
+      </x:c>
+      <x:c r="E180" s="43" t="str">
+        <x:v>issuer_release</x:v>
+      </x:c>
+      <x:c r="F180" s="43" t="str">
+        <x:v>https://investor.bloomenergy.com/press-releases/press-release-details/2026/Bloom-Energy-and-Oracle-Expand-Strategic-Partnership-to-Deploy-up-to-2-8-GW-to-Accelerate-AI-Infrastructure-Build-Out/default.aspx</x:v>
+      </x:c>
+      <x:c r="G180" s="43" t="str">
+        <x:v>Bloom future Oracle generation deployment</x:v>
+      </x:c>
+      <x:c r="H180" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I180" s="43" t="str">
+        <x:v>Up to2.8GW;1.2GW contracted and deploying into next year; first system delivered in55 days</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" s="19" t="str">
+        <x:v>SRC-ORCL-JUPITER-BE-20260427</x:v>
+      </x:c>
+      <x:c r="B181" s="45" t="d">
+        <x:v>2026-04-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C181" s="19" t="str">
+        <x:v>Oracle / BorderPlex</x:v>
+      </x:c>
+      <x:c r="D181" s="43" t="str">
+        <x:v>Oracle BorderPlex and Bloom to power Project Jupiter</x:v>
+      </x:c>
+      <x:c r="E181" s="43" t="str">
+        <x:v>counterparty_release</x:v>
+      </x:c>
+      <x:c r="F181" s="43" t="str">
+        <x:v>https://www.oracle.com/news/announcement/oracle-borderplex-and-bloom-energy-to-power-project-jupiter-with-fuel-cell-technology-2026-04-27/</x:v>
+      </x:c>
+      <x:c r="G181" s="43" t="str">
+        <x:v>Bloom Project Jupiter generation perimeter</x:v>
+      </x:c>
+      <x:c r="H181" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I181" s="43" t="str">
+        <x:v>Up to2.45GW installed fuel-cell generation; Oracle bears energy costs; no IT-load or PUE disclosure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" s="19" t="str">
+        <x:v>SRC-BE-800V-20260916</x:v>
+      </x:c>
+      <x:c r="B182" s="45" t="d">
+        <x:v>2026-09-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C182" s="19" t="str">
+        <x:v>Bloom Energy</x:v>
+      </x:c>
+      <x:c r="D182" s="43" t="str">
+        <x:v>Bloom 800V DC-native power cost model</x:v>
+      </x:c>
+      <x:c r="E182" s="43" t="str">
+        <x:v>issuer_modeled_claim</x:v>
+      </x:c>
+      <x:c r="F182" s="43" t="str">
+        <x:v>https://investor.bloomenergy.com/press-releases/press-release-details/2026/Bloom-Energys-800V-DC-Native-Power-Can-Cut-Billions-from-AI-Data-Center-Costs-Reduce-Power-Use-and-Eliminate-Need-for-Transformers/default.aspx</x:v>
+      </x:c>
+      <x:c r="G182" s="43" t="str">
+        <x:v>Bloom company modeled DC power economics</x:v>
+      </x:c>
+      <x:c r="H182" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I182" s="43" t="str">
+        <x:v>Illustrative1GW site claims3.6B non-compute capex and5.5B five-year TCO savings; not audited realized economics or PUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" s="19" t="str">
+        <x:v>SRC-PLTR-10K-FY25</x:v>
+      </x:c>
+      <x:c r="B183" s="45" t="d">
+        <x:v>2026-02-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C183" s="19" t="str">
+        <x:v>Palantir Technologies Inc.</x:v>
+      </x:c>
+      <x:c r="D183" s="43" t="str">
+        <x:v>Palantir FY2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="E183" s="43" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F183" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</x:v>
+      </x:c>
+      <x:c r="G183" s="43" t="str">
+        <x:v>Palantir company review</x:v>
+      </x:c>
+      <x:c r="H183" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I183" s="43" t="str">
+        <x:v>Statements of Operations p86; Material Cash Requirements p78; Note 2 pp93-95; Notes 6-8 pp100-103; Item 15 exhibit index; </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" s="19" t="str">
+        <x:v>SRC-PLTR-10Q-Q2FY26</x:v>
+      </x:c>
+      <x:c r="B184" s="45" t="d">
+        <x:v>2026-08-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C184" s="19" t="str">
+        <x:v>Palantir Technologies Inc.</x:v>
+      </x:c>
+      <x:c r="D184" s="43" t="str">
+        <x:v>Palantir Q2 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E184" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F184" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000041/pltr-20260630.htm</x:v>
+      </x:c>
+      <x:c r="G184" s="43" t="str">
+        <x:v>Palantir company review</x:v>
+      </x:c>
+      <x:c r="H184" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I184" s="43" t="str">
+        <x:v>Balance Sheet p3; Operations p4; Note 3 p11; Notes 6-7 pp13-14; MD&amp;A pp29-33; investment risk p55; cloud-provider risk pp58-59; Item 6 p88; SEC filing date is August 4; document signatures and issuer PDF are dated August 3. Both HTML and issuer PDF read.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" s="19" t="str">
+        <x:v>SRC-PLTR-10Q-Q1FY26</x:v>
+      </x:c>
+      <x:c r="B185" s="45" t="d">
+        <x:v>2026-05-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C185" s="19" t="str">
+        <x:v>Palantir Technologies Inc.</x:v>
+      </x:c>
+      <x:c r="D185" s="43" t="str">
+        <x:v>Palantir Q1 2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="E185" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F185" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000028/pltr-20260331.htm</x:v>
+      </x:c>
+      <x:c r="G185" s="43" t="str">
+        <x:v>Palantir company review</x:v>
+      </x:c>
+      <x:c r="H185" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I185" s="43" t="str">
+        <x:v>Note 7 Purchase Commitments; Item 6 exhibit index p86; Read to establish first disclosure of March amendment; not an additional commitment on top of Q2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" s="19" t="str">
+        <x:v>SRC-PLTR-Q2FY26-ER</x:v>
+      </x:c>
+      <x:c r="B186" s="45" t="d">
+        <x:v>2026-08-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C186" s="19" t="str">
+        <x:v>Palantir Technologies Inc.</x:v>
+      </x:c>
+      <x:c r="D186" s="43" t="str">
+        <x:v>Palantir Q2 2026 earnings release furnished as Exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="E186" s="43" t="str">
+        <x:v>8-K_exhibit</x:v>
+      </x:c>
+      <x:c r="F186" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000039/a2026q2ex991pressrelease.htm</x:v>
+      </x:c>
+      <x:c r="G186" s="43" t="str">
+        <x:v>Palantir company review</x:v>
+      </x:c>
+      <x:c r="H186" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I186" s="43" t="str">
+        <x:v>Q2 Highlights; Financial Summary; Statements of Operations; Reconciliation of Adjusted Free Cash Flow; </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" s="19" t="str">
+        <x:v>SRC-PLTR-Q2FY26-DECK</x:v>
+      </x:c>
+      <x:c r="B187" s="45" t="d">
+        <x:v>2026-08-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C187" s="19" t="str">
+        <x:v>Palantir Technologies Inc.</x:v>
+      </x:c>
+      <x:c r="D187" s="43" t="str">
+        <x:v>Palantir Q2 2026 Business Update</x:v>
+      </x:c>
+      <x:c r="E187" s="43" t="str">
+        <x:v>issuer_presentation</x:v>
+      </x:c>
+      <x:c r="F187" s="43" t="str">
+        <x:v>https://investors.palantir.com/files/Palantir%20-%20Q2%202026%20Business%20Update.pdf</x:v>
+      </x:c>
+      <x:c r="G187" s="43" t="str">
+        <x:v>Palantir company review</x:v>
+      </x:c>
+      <x:c r="H187" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I187" s="43" t="str">
+        <x:v>Slides 4-5, 11, 14, 19-20, 23-24, 27, 29; Full PDF retrieved directly and text extracted; web renderer rejected 16.3MB size. Company strategy statements are claims, not measured token economics.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="A188" s="19" t="str">
+        <x:v>SRC-PLTR-FILING-INDEX-20261011</x:v>
+      </x:c>
+      <x:c r="B188" s="45" t="d">
+        <x:v>2026-10-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C188" s="19" t="str">
+        <x:v>Palantir Technologies Inc.</x:v>
+      </x:c>
+      <x:c r="D188" s="43" t="str">
+        <x:v>Palantir SEC submissions index checked October 11 2026</x:v>
+      </x:c>
+      <x:c r="E188" s="43" t="str">
+        <x:v>regulator_index</x:v>
+      </x:c>
+      <x:c r="F188" s="43" t="str">
+        <x:v>https://data.sec.gov/submissions/CIK0001321655.json</x:v>
+      </x:c>
+      <x:c r="G188" s="43" t="str">
+        <x:v>Palantir company review</x:v>
+      </x:c>
+      <x:c r="H188" s="43" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I188" s="43" t="str">
+        <x:v>filings.recent form, filingDate, accessionNumber and primaryDocument; Latest 10-K FY2025 and 10-Q June 30 2026. Latest indexed 8-K August 3 earnings; Q1/Q2 exhibit lists contain no full cloud-hosting amendment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="A189" s="20" t="str">
+        <x:v>SRC-PLTR-NVDA-SOVEREIGN-20260910</x:v>
+      </x:c>
+      <x:c r="B189" s="46" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C189" s="20" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="D189" s="44" t="str">
+        <x:v>NVIDIA and Palantir Bring Sovereign Intelligence to Critical Supply Chains</x:v>
+      </x:c>
+      <x:c r="E189" s="44" t="str">
+        <x:v>counterparty_release</x:v>
+      </x:c>
+      <x:c r="F189" s="44" t="str">
+        <x:v>https://nvidianews.nvidia.com/news/nvidia-and-palantir-bring-sovereign-intelligence-to-critical-supply-chains</x:v>
+      </x:c>
+      <x:c r="G189" s="44" t="str">
+        <x:v>Palantir company review</x:v>
+      </x:c>
+      <x:c r="H189" s="44" t="str">
+        <x:v>Primary read</x:v>
+      </x:c>
+      <x:c r="I189" s="44" t="str">
+        <x:v>News Summary; Open Models; Built for Sovereign Enterprise-Scale Deployment; Deployment begins inside NVIDIA operations. No contract value, GPU count, IT MW, PUE, deployment revenue or measured savings disclosed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R070ca4829cd643e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa6a7d51a254518"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Review Oracle OCI: CPU/GPU economics, financing and matched-MW gaps (2026-10-12)
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R622505dd11384eaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rf1824ba6b2534017"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R44b3f18795ec405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rd8f3833de5a24437"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R743bdc6f50cf47f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rf56c81c5f7584230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rd03a833525ae40d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb09d3df6532b43c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rbeae67b6cf4843bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R0bc4dd3fe1514461"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R9bf7915467d34fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R506850f379554c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R4da699e3358d41b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Re735e3d4a2cd4fcd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I189" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I199" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1516,7 +1516,7 @@
         <x:v>Q1 FY2027</x:v>
       </x:c>
       <x:c r="D9" s="27" t="n">
-        <x:v>7400000000</x:v>
+        <x:v>6500000000</x:v>
       </x:c>
       <x:c r="E9" s="29" t="n">
         <x:v>4</x:v>
@@ -1529,13 +1529,13 @@
       <x:c r="K9" s="35"/>
       <x:c r="L9" s="35"/>
       <x:c r="M9" s="19" t="str">
-        <x:v>SRC-ORCL-Q1FY27-20260910</x:v>
+        <x:v>SRC-ORCL-Q1FY27-DECK</x:v>
       </x:c>
       <x:c r="N9" s="19" t="str">
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O9" s="43" t="str">
-        <x:v>IaaS only; AI share and average IT MW missing. 850MW additions excluded; PUE undisclosed.</x:v>
+        <x:v>Rounded CPU/GPU revenue excludes database; AI share, hardware adjustment, average active IT MW and physical utilization missing. 97.9% issuer utilization undefined; 850MW additions excluded; matched PUE undisclosed.</x:v>
       </x:c>
       <x:c r="P9" s="37" t="str">
         <x:f>IF(OR(D9="",E9="",F9=""),"",D9*E9*F9)</x:f>
@@ -2227,16 +2227,16 @@
         <x:v>Hyperscaler</x:v>
       </x:c>
       <x:c r="D9" s="43" t="str">
-        <x:v>Recognized AI compute within OCI less hardware pass-through</x:v>
+        <x:v>Annualized AI-attributable CPU/GPU revenue less hardware pass-through</x:v>
       </x:c>
       <x:c r="E9" s="43" t="str">
-        <x:v>Time-weighted active AI IT MW and matching utilization</x:v>
+        <x:v>Time-weighted active AI IT MW times matching physical utilization</x:v>
       </x:c>
       <x:c r="F9" s="43" t="str">
-        <x:v>Exclude RPO and prepayment cash; no use of capacity additions as denominator</x:v>
+        <x:v>Exclude database, RPO, prepayment cash and undefined utilization; require dated active AI IT capacity</x:v>
       </x:c>
       <x:c r="G9" s="43" t="str">
-        <x:v>Partial 2026-09-11; PUE not disclosed</x:v>
+        <x:v>Partial 2026-10-12; AI attribution, active IT MW, physical utilization and matched PUE open</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2472,7 +2472,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9506ee048adb424a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55534733680843de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3444,7 +3444,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34de0e430cb84fff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a5614bebfb14fc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9197,38 +9197,324 @@
       </x:c>
     </x:row>
     <x:row r="189">
-      <x:c r="A189" s="20" t="str">
+      <x:c r="A189" s="19" t="str">
         <x:v>SRC-PLTR-NVDA-SOVEREIGN-20260910</x:v>
       </x:c>
-      <x:c r="B189" s="46" t="d">
+      <x:c r="B189" s="45" t="d">
         <x:v>2026-09-10T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C189" s="20" t="str">
+      <x:c r="C189" s="19" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
-      <x:c r="D189" s="44" t="str">
+      <x:c r="D189" s="43" t="str">
         <x:v>NVIDIA and Palantir Bring Sovereign Intelligence to Critical Supply Chains</x:v>
       </x:c>
-      <x:c r="E189" s="44" t="str">
+      <x:c r="E189" s="43" t="str">
         <x:v>counterparty_release</x:v>
       </x:c>
-      <x:c r="F189" s="44" t="str">
+      <x:c r="F189" s="43" t="str">
         <x:v>https://nvidianews.nvidia.com/news/nvidia-and-palantir-bring-sovereign-intelligence-to-critical-supply-chains</x:v>
       </x:c>
-      <x:c r="G189" s="44" t="str">
+      <x:c r="G189" s="43" t="str">
         <x:v>Palantir company review</x:v>
       </x:c>
-      <x:c r="H189" s="44" t="str">
+      <x:c r="H189" s="43" t="str">
         <x:v>Primary read</x:v>
       </x:c>
-      <x:c r="I189" s="44" t="str">
+      <x:c r="I189" s="43" t="str">
         <x:v>News Summary; Open Models; Built for Sovereign Enterprise-Scale Deployment; Deployment begins inside NVIDIA operations. No contract value, GPU count, IT MW, PUE, deployment revenue or measured savings disclosed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="A190" s="19" t="str">
+        <x:v>SRC-ORCL-Q1FY27-DECK</x:v>
+      </x:c>
+      <x:c r="B190" s="45" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C190" s="19" t="str">
+        <x:v>Oracle (issuer presentation on third-party mirror)</x:v>
+      </x:c>
+      <x:c r="D190" s="43" t="str">
+        <x:v>Q1 FY2027 earnings presentation</x:v>
+      </x:c>
+      <x:c r="E190" s="43" t="str">
+        <x:v>issuer_presentation</x:v>
+      </x:c>
+      <x:c r="F190" s="43" t="str">
+        <x:v>https://csv-storage.forexpros.com/slides/597927154e234fcd26fe6003bd5d184554884a6499af9b3bf8ed3ef5bf2d8d24.pdf</x:v>
+      </x:c>
+      <x:c r="G190" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H190" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I190" s="43" t="str">
+        <x:v>Full 15-slide issuer-authored document read. Oracle IR endpoint unavailable; mirror provenance explicit. Rounded financial totals reconcile to SEC filing; utilization and renewal premium are management claims.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191">
+      <x:c r="A191" s="19" t="str">
+        <x:v>SRC-ORCL-CDP-2025-READ20261012</x:v>
+      </x:c>
+      <x:c r="B191" s="45"/>
+      <x:c r="C191" s="19" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D191" s="43" t="str">
+        <x:v>CDP climate questionnaire 2025</x:v>
+      </x:c>
+      <x:c r="E191" s="43" t="str">
+        <x:v>issuer_sustainability_questionnaire</x:v>
+      </x:c>
+      <x:c r="F191" s="43" t="str">
+        <x:v>https://www.oracle.com/a/ocom/docs/cdp-climate-change-questionnaire.pdf</x:v>
+      </x:c>
+      <x:c r="G191" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H191" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I191" s="43" t="str">
+        <x:v>Copyright 2026 does not establish publication date. Oracle describes invoice-based IT power and site-average PUE inputs for leased-site non-IT emissions estimation, but does not publish usable matched site PUE inputs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" s="19" t="str">
+        <x:v>SRC-ORCL-PUE-BLOG-20201204</x:v>
+      </x:c>
+      <x:c r="B192" s="45" t="d">
+        <x:v>2020-12-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C192" s="19" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D192" s="43" t="str">
+        <x:v>Sustainability 2025: Oracle renews commitment to environmental goals</x:v>
+      </x:c>
+      <x:c r="E192" s="43" t="str">
+        <x:v>issuer_blog</x:v>
+      </x:c>
+      <x:c r="F192" s="43" t="str">
+        <x:v>https://blogs.oracle.com/sustainability/sustainability-2025-oracle-renews-commitment-to-environmental-goals</x:v>
+      </x:c>
+      <x:c r="G192" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H192" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I192" s="43" t="str">
+        <x:v>2025 in title is target year, not publication year. Best-case historical site claim only; not a current fleet average.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" s="19" t="str">
+        <x:v>SRC-ORCL-PLANET-READ20261012</x:v>
+      </x:c>
+      <x:c r="B193" s="45"/>
+      <x:c r="C193" s="19" t="str">
+        <x:v>Oracle</x:v>
+      </x:c>
+      <x:c r="D193" s="43" t="str">
+        <x:v>Planet sustainability goals</x:v>
+      </x:c>
+      <x:c r="E193" s="43" t="str">
+        <x:v>issuer_webpage</x:v>
+      </x:c>
+      <x:c r="F193" s="43" t="str">
+        <x:v>https://www.oracle.com/social-impact/planet/</x:v>
+      </x:c>
+      <x:c r="G193" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H193" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I193" s="43" t="str">
+        <x:v>Current webpage read; does not give numeric matched PUE. Separate 2035 custom-cluster goal must not be collapsed into public-cloud goal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" s="19" t="str">
+        <x:v>SRC-ORCL-SEC-INDEX-20261012</x:v>
+      </x:c>
+      <x:c r="B194" s="45" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C194" s="19" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D194" s="43" t="str">
+        <x:v>Oracle submissions index through October 12</x:v>
+      </x:c>
+      <x:c r="E194" s="43" t="str">
+        <x:v>regulatory_index</x:v>
+      </x:c>
+      <x:c r="F194" s="43" t="str">
+        <x:v>https://data.sec.gov/submissions/CIK0001341439.json</x:v>
+      </x:c>
+      <x:c r="G194" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H194" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I194" s="43" t="str">
+        <x:v>Latest 10-K June22, 10-Q September11 and 8-K September14. Retrieval date is snapshot date, not filing publication date.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195">
+      <x:c r="A195" s="19" t="str">
+        <x:v>SRC-ORCL-8K-20260914</x:v>
+      </x:c>
+      <x:c r="B195" s="45" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C195" s="19" t="str">
+        <x:v>Oracle / SEC</x:v>
+      </x:c>
+      <x:c r="D195" s="43" t="str">
+        <x:v>September 14 Form 8-K</x:v>
+      </x:c>
+      <x:c r="E195" s="43" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="F195" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389753/d20034d8k.htm</x:v>
+      </x:c>
+      <x:c r="G195" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H195" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I195" s="43" t="str">
+        <x:v>Entire short filing read. Larry Ellison canceled trading plan; no sales. Does not disclose disposition of September lessor guarantee.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" s="19" t="str">
+        <x:v>SRC-ORCL-424B5-20260623</x:v>
+      </x:c>
+      <x:c r="B196" s="45" t="d">
+        <x:v>2026-06-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C196" s="19" t="str">
+        <x:v>Oracle / SEC</x:v>
+      </x:c>
+      <x:c r="D196" s="43" t="str">
+        <x:v>ATM prospectus supplement adding sales agents</x:v>
+      </x:c>
+      <x:c r="E196" s="43" t="str">
+        <x:v>424B5</x:v>
+      </x:c>
+      <x:c r="F196" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526278585/d120346d424b5.htm</x:v>
+      </x:c>
+      <x:c r="G196" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H196" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I196" s="43" t="str">
+        <x:v>Adds agents, not another $20B authorization; Q1 10-Q subsequently reports full utilization.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="19" t="str">
+        <x:v>SRC-ORCL-Q1FY27-TRANSCRIPT</x:v>
+      </x:c>
+      <x:c r="B197" s="45" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C197" s="19" t="str">
+        <x:v>The Motley Fool (transcript of Oracle management)</x:v>
+      </x:c>
+      <x:c r="D197" s="43" t="str">
+        <x:v>Oracle Q1 FY2027 earnings-call transcript</x:v>
+      </x:c>
+      <x:c r="E197" s="43" t="str">
+        <x:v>secondary_transcript</x:v>
+      </x:c>
+      <x:c r="F197" s="43" t="str">
+        <x:v>https://www.fool.com/earnings/call-transcripts/2026/09/11/oracle-orcl-q1-2027-earnings-call-transcript/</x:v>
+      </x:c>
+      <x:c r="G197" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H197" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I197" s="43" t="str">
+        <x:v>Prepared remarks and Q&amp;A read; not checked against audio. Obvious 3 thousand GPUs transcription discrepancy is overridden by primary earnings release &gt;300,000. Management delivery claims are not independently verified energized capacity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198">
+      <x:c r="A198" s="19" t="str">
+        <x:v>SRC-NMED-JUPITER-20261012</x:v>
+      </x:c>
+      <x:c r="B198" s="45" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C198" s="19" t="str">
+        <x:v>New Mexico Environment Department</x:v>
+      </x:c>
+      <x:c r="D198" s="43" t="str">
+        <x:v>Project Jupiter microgrid permit stay: October12 snapshot</x:v>
+      </x:c>
+      <x:c r="E198" s="43" t="str">
+        <x:v>regulatory_status_snapshot</x:v>
+      </x:c>
+      <x:c r="F198" s="43" t="str">
+        <x:v>https://www.env.nm.gov/</x:v>
+      </x:c>
+      <x:c r="G198" s="43" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H198" s="43" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I198" s="43" t="str">
+        <x:v>Date is observation date; page says Supreme Court has stayed process. No signed judicial order or final permit independently obtained; does not prove cancellation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" s="20" t="str">
+        <x:v>SRC-NMED-JUPITER-DOCKET-20261012</x:v>
+      </x:c>
+      <x:c r="B199" s="46" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C199" s="20" t="str">
+        <x:v>New Mexico Environment Department</x:v>
+      </x:c>
+      <x:c r="D199" s="44" t="str">
+        <x:v>Yucca Growth Infrastructure microgrid permit docket snapshot</x:v>
+      </x:c>
+      <x:c r="E199" s="44" t="str">
+        <x:v>regulatory_docket_snapshot</x:v>
+      </x:c>
+      <x:c r="F199" s="44" t="str">
+        <x:v>https://www.env.nm.gov/public-notices/yucca-growth-infrastructure-llc-ygi-microgrid/</x:v>
+      </x:c>
+      <x:c r="G199" s="44" t="str">
+        <x:v>Oracle OCI review</x:v>
+      </x:c>
+      <x:c r="H199" s="44" t="str">
+        <x:v>Read 2026-10-12</x:v>
+      </x:c>
+      <x:c r="I199" s="44" t="str">
+        <x:v>Docket read; no final permit seen in displayed documents. Dynamic hearing-calendar link did not expose order text.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa6a7d51a254518"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52d0400268834e2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Review CoreWeave pricing, leases, and MW economics (2026-10-13)
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb09d3df6532b43c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rbeae67b6cf4843bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R0bc4dd3fe1514461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R9bf7915467d34fc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R506850f379554c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R4da699e3358d41b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Re735e3d4a2cd4fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rca3fda7210954635"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R648eda0c68b84666"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rce54bc8aeec14764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rbfc03ddeccc04104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R4177d54573ce4436"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Ra611178303ae425d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rc21230771eaa45ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I199" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I207" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1571,11 +1571,9 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F10" s="31"/>
-      <x:c r="G10" s="33" t="n">
-        <x:v>1250</x:v>
-      </x:c>
+      <x:c r="G10" s="33"/>
       <x:c r="H10" s="23" t="str">
-        <x:v>Facility power</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="I10" s="35"/>
       <x:c r="J10" s="35"/>
@@ -1588,7 +1586,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O10" s="43" t="str">
-        <x:v>All-cloud revenue and modeled period-average active-power proxy; compute mix power boundary PUE and utilization remain missing so normalized output stays blank</x:v>
+        <x:v>All-cloud recognized revenue ceiling; June-heavy activation invalidates midpoint selection. Compute mix, dated IT-MW, power boundary, matched PUE and physical utilization remain missing. Recent ~$40M/MW-year short-contract rate is separate.</x:v>
       </x:c>
       <x:c r="P10" s="37" t="str">
         <x:f>IF(OR(D10="",E10="",F10=""),"",D10*E10*F10)</x:f>
@@ -2250,16 +2248,16 @@
         <x:v>Neocloud</x:v>
       </x:c>
       <x:c r="D10" s="43" t="str">
-        <x:v>Annualized compute-only revenue</x:v>
+        <x:v>Annualized external AI compute recognized revenue</x:v>
       </x:c>
       <x:c r="E10" s="43" t="str">
-        <x:v>Weighted-average active IT MW times utilization</x:v>
+        <x:v>Time-weighted active AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F10" s="43" t="str">
-        <x:v>Remove storage networking and software; reconstruct average capacity; resolve active-power boundary and PUE</x:v>
+        <x:v>Remove storage networking and software; keep ~$40M/MW-year recent 3-6 month signed-contract rate separate from recognized revenue; no generic PUE or utilization</x:v>
       </x:c>
       <x:c r="G10" s="43" t="str">
-        <x:v>Partial 2026-09-12; canonical output open</x:v>
+        <x:v>Partial 2026-10-13; canonical output open</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2472,7 +2470,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55534733680843de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb706819416fc43eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3444,7 +3442,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a5614bebfb14fc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fabf5fe30a849de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9483,38 +9481,270 @@
       </x:c>
     </x:row>
     <x:row r="199">
-      <x:c r="A199" s="20" t="str">
+      <x:c r="A199" s="19" t="str">
         <x:v>SRC-NMED-JUPITER-DOCKET-20261012</x:v>
       </x:c>
-      <x:c r="B199" s="46" t="d">
+      <x:c r="B199" s="45" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C199" s="20" t="str">
+      <x:c r="C199" s="19" t="str">
         <x:v>New Mexico Environment Department</x:v>
       </x:c>
-      <x:c r="D199" s="44" t="str">
+      <x:c r="D199" s="43" t="str">
         <x:v>Yucca Growth Infrastructure microgrid permit docket snapshot</x:v>
       </x:c>
-      <x:c r="E199" s="44" t="str">
+      <x:c r="E199" s="43" t="str">
         <x:v>regulatory_docket_snapshot</x:v>
       </x:c>
-      <x:c r="F199" s="44" t="str">
+      <x:c r="F199" s="43" t="str">
         <x:v>https://www.env.nm.gov/public-notices/yucca-growth-infrastructure-llc-ygi-microgrid/</x:v>
       </x:c>
-      <x:c r="G199" s="44" t="str">
+      <x:c r="G199" s="43" t="str">
         <x:v>Oracle OCI review</x:v>
       </x:c>
-      <x:c r="H199" s="44" t="str">
+      <x:c r="H199" s="43" t="str">
         <x:v>Read 2026-10-12</x:v>
       </x:c>
-      <x:c r="I199" s="44" t="str">
+      <x:c r="I199" s="43" t="str">
         <x:v>Docket read; no final permit seen in displayed documents. Dynamic hearing-calendar link did not expose order text.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" s="19" t="str">
+        <x:v>SRC-CRWV-SEC-INDEX-20261013</x:v>
+      </x:c>
+      <x:c r="B200" s="45" t="d">
+        <x:v>2026-10-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C200" s="19" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D200" s="43" t="str">
+        <x:v>CoreWeave submissions index checked October 13 2026</x:v>
+      </x:c>
+      <x:c r="E200" s="43" t="str">
+        <x:v>regulator_index</x:v>
+      </x:c>
+      <x:c r="F200" s="43" t="str">
+        <x:v>https://data.sec.gov/submissions/CIK0001769628.json</x:v>
+      </x:c>
+      <x:c r="G200" s="43" t="str">
+        <x:v>CoreWeave review</x:v>
+      </x:c>
+      <x:c r="H200" s="43" t="str">
+        <x:v>Read 2026-10-13</x:v>
+      </x:c>
+      <x:c r="I200" s="43" t="str">
+        <x:v>Latest material financial filing is September 22 convertible close; October 13 entries are Forms 144.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" s="19" t="str">
+        <x:v>SRC-CRWV-Q2FY26-DECK</x:v>
+      </x:c>
+      <x:c r="B201" s="45" t="d">
+        <x:v>2026-08-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C201" s="19" t="str">
+        <x:v>CoreWeave</x:v>
+      </x:c>
+      <x:c r="D201" s="43" t="str">
+        <x:v>Q2 2026 Earnings Presentation</x:v>
+      </x:c>
+      <x:c r="E201" s="43" t="str">
+        <x:v>issuer_presentation</x:v>
+      </x:c>
+      <x:c r="F201" s="43" t="str">
+        <x:v>https://s205.q4cdn.com/133937190/files/doc_financials/2026/q2/CoreWeave-Q2-26-Earnings-Presentation.pdf</x:v>
+      </x:c>
+      <x:c r="G201" s="43" t="str">
+        <x:v>CoreWeave review</x:v>
+      </x:c>
+      <x:c r="H201" s="43" t="str">
+        <x:v>Read 2026-10-13</x:v>
+      </x:c>
+      <x:c r="I201" s="43" t="str">
+        <x:v>Full 23-page presentation; active power boundary remains undefined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" s="19" t="str">
+        <x:v>SRC-CRWV-Q2FY26-OUTLOOK</x:v>
+      </x:c>
+      <x:c r="B202" s="45" t="d">
+        <x:v>2026-08-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C202" s="19" t="str">
+        <x:v>CoreWeave</x:v>
+      </x:c>
+      <x:c r="D202" s="43" t="str">
+        <x:v>Q2 2026 Earnings Outlook Presentation</x:v>
+      </x:c>
+      <x:c r="E202" s="43" t="str">
+        <x:v>issuer_presentation</x:v>
+      </x:c>
+      <x:c r="F202" s="43" t="str">
+        <x:v>https://s205.q4cdn.com/133937190/files/doc_financials/2026/q2/CoreWeave-Q2-26-Earnings-Outlook-Presentation.pdf</x:v>
+      </x:c>
+      <x:c r="G202" s="43" t="str">
+        <x:v>CoreWeave review</x:v>
+      </x:c>
+      <x:c r="H202" s="43" t="str">
+        <x:v>Read 2026-10-13</x:v>
+      </x:c>
+      <x:c r="I202" s="43" t="str">
+        <x:v>Guidance and ARR kept separate from Q2 recognized revenue.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" s="19" t="str">
+        <x:v>SRC-CRWV-Q2FY26-CALL</x:v>
+      </x:c>
+      <x:c r="B203" s="45" t="d">
+        <x:v>2026-08-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C203" s="19" t="str">
+        <x:v>CoreWeave</x:v>
+      </x:c>
+      <x:c r="D203" s="43" t="str">
+        <x:v>Corrected transcript of Q2 2026 earnings call</x:v>
+      </x:c>
+      <x:c r="E203" s="43" t="str">
+        <x:v>issuer_hosted_transcript</x:v>
+      </x:c>
+      <x:c r="F203" s="43" t="str">
+        <x:v>https://s205.q4cdn.com/133937190/files/doc_financials/2026/q2/CRWV-US-CORRECTED-TRANSCRIPT-CoreWeave-Q2-2026-Earnings-Call-11August2026.pdf</x:v>
+      </x:c>
+      <x:c r="G203" s="43" t="str">
+        <x:v>CoreWeave review</x:v>
+      </x:c>
+      <x:c r="H203" s="43" t="str">
+        <x:v>Read 2026-10-13</x:v>
+      </x:c>
+      <x:c r="I203" s="43" t="str">
+        <x:v>Management claims labeled; more than 300MW activated in June.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" s="19" t="str">
+        <x:v>SRC-CRWV-CONVERT-DECK-20260917</x:v>
+      </x:c>
+      <x:c r="B204" s="45" t="d">
+        <x:v>2026-09-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C204" s="19" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D204" s="43" t="str">
+        <x:v>Convertible offering supplemental presentation</x:v>
+      </x:c>
+      <x:c r="E204" s="43" t="str">
+        <x:v>8-K Exhibit 99.2</x:v>
+      </x:c>
+      <x:c r="F204" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000429/crwv2026convertpresentat.htm</x:v>
+      </x:c>
+      <x:c r="G204" s="43" t="str">
+        <x:v>CoreWeave review</x:v>
+      </x:c>
+      <x:c r="H204" s="43" t="str">
+        <x:v>Read 2026-10-13</x:v>
+      </x:c>
+      <x:c r="I204" s="43" t="str">
+        <x:v>Full deck; $40M/MW is scoped signed-contract rate not recognized revenue per effective IT MW.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205">
+      <x:c r="A205" s="19" t="str">
+        <x:v>SRC-CRWV-8K-CONVERT-20260917</x:v>
+      </x:c>
+      <x:c r="B205" s="45" t="d">
+        <x:v>2026-09-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C205" s="19" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D205" s="43" t="str">
+        <x:v>Convertible notes and equity distribution Form 8-K</x:v>
+      </x:c>
+      <x:c r="E205" s="43" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="F205" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000429/crwv-20260917.htm</x:v>
+      </x:c>
+      <x:c r="G205" s="43" t="str">
+        <x:v>CoreWeave review</x:v>
+      </x:c>
+      <x:c r="H205" s="43" t="str">
+        <x:v>Read 2026-10-13</x:v>
+      </x:c>
+      <x:c r="I205" s="43" t="str">
+        <x:v>Initial offering and equity distribution terms read.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206">
+      <x:c r="A206" s="19" t="str">
+        <x:v>SRC-CRWV-424B5-CONVERT-20260918</x:v>
+      </x:c>
+      <x:c r="B206" s="45" t="d">
+        <x:v>2026-09-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C206" s="19" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D206" s="43" t="str">
+        <x:v>Prospectus supplement for 2.875% convertible senior notes due 2033</x:v>
+      </x:c>
+      <x:c r="E206" s="43" t="str">
+        <x:v>424B5</x:v>
+      </x:c>
+      <x:c r="F206" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000162828026062362/coreweave-424b5.htm</x:v>
+      </x:c>
+      <x:c r="G206" s="43" t="str">
+        <x:v>CoreWeave review</x:v>
+      </x:c>
+      <x:c r="H206" s="43" t="str">
+        <x:v>Read 2026-10-13</x:v>
+      </x:c>
+      <x:c r="I206" s="43" t="str">
+        <x:v>Final prospectus; general-purpose use and capped-call terms.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207">
+      <x:c r="A207" s="20" t="str">
+        <x:v>SRC-CRWV-8K-CONVERT-CLOSE-20260922</x:v>
+      </x:c>
+      <x:c r="B207" s="46" t="d">
+        <x:v>2026-09-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C207" s="20" t="str">
+        <x:v>CoreWeave / SEC</x:v>
+      </x:c>
+      <x:c r="D207" s="44" t="str">
+        <x:v>Convertible senior notes closing Form 8-K</x:v>
+      </x:c>
+      <x:c r="E207" s="44" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="F207" s="44" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000432/crwv-20260917.htm</x:v>
+      </x:c>
+      <x:c r="G207" s="44" t="str">
+        <x:v>CoreWeave review</x:v>
+      </x:c>
+      <x:c r="H207" s="44" t="str">
+        <x:v>Read 2026-10-13</x:v>
+      </x:c>
+      <x:c r="I207" s="44" t="str">
+        <x:v>$4.2B principal; $4.137B net before other expenses; $566.2M capped-call cost.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52d0400268834e2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R197961cb4dfb454d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
research: complete Nebius commissioning and collateral review (2026-10-15)
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rca3fda7210954635"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R648eda0c68b84666"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rce54bc8aeec14764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rbfc03ddeccc04104"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R4177d54573ce4436"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Ra611178303ae425d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rc21230771eaa45ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8812293c34754c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R7e8c69089d164425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R4639024501684d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R00f6bde1f09f418b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R4c45c7c7241b4031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R7ead8152e2844d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rfdbe23b4a5c449e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I207" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I211" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1635,7 +1635,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O11" s="43" t="str">
-        <x:v>Raw segment includes internal/noncompute; Q2 active IT MW and utilization open. PUE 1.25 is 2025 only.</x:v>
+        <x:v>Compute attribution and Q2 active IT MW/utilization open. PUE 1.25 is 2025 only. June $7.8364B not-in-use PP&amp;E includes prepayments; not idle GPU collateral.</x:v>
       </x:c>
       <x:c r="P11" s="37" t="str">
         <x:f>IF(OR(D11="",E11="",F11=""),"",D11*E11*F11)</x:f>
@@ -2470,7 +2470,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb706819416fc43eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R030bd63f38594766"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3442,7 +3442,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fabf5fe30a849de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re79cab3823864295"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9713,38 +9713,154 @@
       </x:c>
     </x:row>
     <x:row r="207">
-      <x:c r="A207" s="20" t="str">
+      <x:c r="A207" s="19" t="str">
         <x:v>SRC-CRWV-8K-CONVERT-CLOSE-20260922</x:v>
       </x:c>
-      <x:c r="B207" s="46" t="d">
+      <x:c r="B207" s="45" t="d">
         <x:v>2026-09-22T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C207" s="20" t="str">
+      <x:c r="C207" s="19" t="str">
         <x:v>CoreWeave / SEC</x:v>
       </x:c>
-      <x:c r="D207" s="44" t="str">
+      <x:c r="D207" s="43" t="str">
         <x:v>Convertible senior notes closing Form 8-K</x:v>
       </x:c>
-      <x:c r="E207" s="44" t="str">
+      <x:c r="E207" s="43" t="str">
         <x:v>8-K</x:v>
       </x:c>
-      <x:c r="F207" s="44" t="str">
+      <x:c r="F207" s="43" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1769628/000176962826000432/crwv-20260917.htm</x:v>
       </x:c>
-      <x:c r="G207" s="44" t="str">
+      <x:c r="G207" s="43" t="str">
         <x:v>CoreWeave review</x:v>
       </x:c>
-      <x:c r="H207" s="44" t="str">
+      <x:c r="H207" s="43" t="str">
         <x:v>Read 2026-10-13</x:v>
       </x:c>
-      <x:c r="I207" s="44" t="str">
+      <x:c r="I207" s="43" t="str">
         <x:v>$4.2B principal; $4.137B net before other expenses; $566.2M capped-call cost.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208">
+      <x:c r="A208" s="19" t="str">
+        <x:v>SRC-NBIS-SEC-INDEX-20261015</x:v>
+      </x:c>
+      <x:c r="B208" s="45" t="d">
+        <x:v>2026-10-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C208" s="19" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D208" s="43" t="str">
+        <x:v>Nebius submissions index checked October 15 2026</x:v>
+      </x:c>
+      <x:c r="E208" s="43" t="str">
+        <x:v>regulator_index</x:v>
+      </x:c>
+      <x:c r="F208" s="43" t="str">
+        <x:v>https://data.sec.gov/submissions/CIK0001513845.json</x:v>
+      </x:c>
+      <x:c r="G208" s="43" t="str">
+        <x:v>Nebius commissioning, financing and idle-capacity economics</x:v>
+      </x:c>
+      <x:c r="H208" s="43" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="I208" s="43" t="str">
+        <x:v>filings.recent: form, filingDate, accessionNumber, primaryDocument. Latest issuer material 6-K October 1 Inferize; October 13 Form 4 and October 7 Schedule 13G/A do not replace quarterly financials.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209">
+      <x:c r="A209" s="19" t="str">
+        <x:v>SRC-NBIS-INFERIZE-20261001</x:v>
+      </x:c>
+      <x:c r="B209" s="45" t="d">
+        <x:v>2026-10-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C209" s="19" t="str">
+        <x:v>Nebius</x:v>
+      </x:c>
+      <x:c r="D209" s="43" t="str">
+        <x:v>Nebius acquires Inferize to strengthen Token Factory production inference</x:v>
+      </x:c>
+      <x:c r="E209" s="43" t="str">
+        <x:v>issuer_release</x:v>
+      </x:c>
+      <x:c r="F209" s="43" t="str">
+        <x:v>https://nebius.com/newsroom/nebius-acquires-inferize-to-strengthen-nebius-token-factorys-production-inference-stack</x:v>
+      </x:c>
+      <x:c r="G209" s="43" t="str">
+        <x:v>Nebius commissioning, financing and idle-capacity economics</x:v>
+      </x:c>
+      <x:c r="H209" s="43" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="I209" s="43" t="str">
+        <x:v>Opening acquisition paragraphs; cold-start and standby GPU discussion; transaction terms paragraph. Company claims about reducing idle launch/scale time; no quantified fleet utilization, GPU count, savings or purchase price. Also furnished in October 1 6-K accession 0001104659-26-112824.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210">
+      <x:c r="A210" s="19" t="str">
+        <x:v>SRC-NBIS-NEWSROOM-20261015</x:v>
+      </x:c>
+      <x:c r="B210" s="45" t="d">
+        <x:v>2026-10-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C210" s="19" t="str">
+        <x:v>Nebius</x:v>
+      </x:c>
+      <x:c r="D210" s="43" t="str">
+        <x:v>Nebius issuer news and financial-results indices checked October 15</x:v>
+      </x:c>
+      <x:c r="E210" s="43" t="str">
+        <x:v>issuer_index</x:v>
+      </x:c>
+      <x:c r="F210" s="43" t="str">
+        <x:v>https://nebius.com/newsroom</x:v>
+      </x:c>
+      <x:c r="G210" s="43" t="str">
+        <x:v>Nebius commissioning, financing and idle-capacity economics</x:v>
+      </x:c>
+      <x:c r="H210" s="43" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="I210" s="43" t="str">
+        <x:v>Latest releases: October 1 Inferize; financials index latest Q2 August 12. Index retrieval date is not a new publication date for the underlying releases. https://nebius.com/financials also checked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211">
+      <x:c r="A211" s="20" t="str">
+        <x:v>SRC-NBIS-STATUS-EUWEST2-20261015</x:v>
+      </x:c>
+      <x:c r="B211" s="46" t="d">
+        <x:v>2026-10-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C211" s="20" t="str">
+        <x:v>Nebius service status</x:v>
+      </x:c>
+      <x:c r="D211" s="44" t="str">
+        <x:v>InfiniBand connectivity issues for GPU clusters in eu-west2</x:v>
+      </x:c>
+      <x:c r="E211" s="44" t="str">
+        <x:v>issuer_status_incident</x:v>
+      </x:c>
+      <x:c r="F211" s="44" t="str">
+        <x:v>https://status.nebius.com/incidents/sdb2htxgyprr</x:v>
+      </x:c>
+      <x:c r="G211" s="44" t="str">
+        <x:v>Nebius availability; no quantified MW impact</x:v>
+      </x:c>
+      <x:c r="H211" s="44" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="I211" s="44" t="str">
+        <x:v>Incident sdb2htxgyprr; Investigating 05:34, Update 09:32, Monitoring 13:13 UTC. Issuer says recovery still in progress in 13:13 UTC update. Affected service EU-WEST2 Compute Cloud. No GPU count, MW, fleet-wide outage percentage, lost revenue or SLA credit amount disclosed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R197961cb4dfb454d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10e370b215594803"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research IREN acceptance risk, pledged GPUs and parent recourse (2026-10-16)
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8812293c34754c7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="R7e8c69089d164425"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R4639024501684d4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R00f6bde1f09f418b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R4c45c7c7241b4031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R7ead8152e2844d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Rfdbe23b4a5c449e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R59d81a709ab64bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rd6ac2691c59c488f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R57b6d850e387484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R8373101135494ebd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R155c9f989e3f4908"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rb9a56a9930dd4cfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R5a487a3e5e894414"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I211" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I214" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1670,9 +1670,7 @@
       <x:c r="E12" s="29" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F12" s="31" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="F12" s="31"/>
       <x:c r="G12" s="33"/>
       <x:c r="H12" s="23"/>
       <x:c r="I12" s="35"/>
@@ -1686,11 +1684,10 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O12" s="43" t="str">
-        <x:v>AI Cloud revenue only derived from FY less nine months; Q4 average active IT MW, utilization and fleet PUE missing. The 40MW June 30 exit capacity is excluded.</x:v>
-      </x:c>
-      <x:c r="P12" s="37" t="n">
+        <x:v>Q4 AI Cloud bundle $70.515M; compute attribution, average IT MW and utilization missing. PUE 1.1 is site-only. June pledged GPUs $1.487B are not an October idle-chip estimate.</x:v>
+      </x:c>
+      <x:c r="P12" s="37" t="str">
         <x:f>IF(OR(D12="",E12="",F12=""),"",D12*E12*F12)</x:f>
-        <x:v>282060000</x:v>
       </x:c>
       <x:c r="Q12" s="39" t="str">
         <x:f>IF(G12="","",IF(H12="IT load",G12,IF(H12="Facility power",IF(I12="","",G12/I12),IF(H12="Generation",IF(OR(I12="",J12="",K12=""),"",G12*J12*K12/I12),IF(H12="Effective utilized IT",G12,"")))))</x:f>
@@ -2294,16 +2291,16 @@
         <x:v>Neocloud</x:v>
       </x:c>
       <x:c r="D12" s="43" t="str">
-        <x:v>Annualized AI cloud and services revenue only</x:v>
+        <x:v>Annualized external compute after AI Cloud bundle attribution</x:v>
       </x:c>
       <x:c r="E12" s="43" t="str">
-        <x:v>Average active AI IT MW times physical utilization</x:v>
+        <x:v>Time-weighted active AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F12" s="43" t="str">
-        <x:v>Exclude Bitcoin mining revenue and mining power</x:v>
+        <x:v>Exclude mining and noncompute ancillaries; acceptance differs from utilization</x:v>
       </x:c>
       <x:c r="G12" s="43" t="str">
-        <x:v>Q4 FY2026 numerator established; average active IT MW utilization and matched PUE open</x:v>
+        <x:v>Compute attribution and matched active IT MW utilization PUE open</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2470,7 +2467,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R030bd63f38594766"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R161e8ba56d2148e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3442,7 +3439,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re79cab3823864295"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R901fa90c522842b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5428,7 +5425,7 @@
         <x:v>SRC-IREN-Q3FY26-ER</x:v>
       </x:c>
       <x:c r="B58" s="45" t="d">
-        <x:v>2026-05-08T00:00:00.000Z</x:v>
+        <x:v>2026-05-07T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C58" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5449,7 +5446,7 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="I58" s="43" t="str">
-        <x:v>pp.1-4 operating and contract update; p.9 revenue table</x:v>
+        <x:v>Release dated May 7; SEC filing May 8. Opening highlights explicitly identify NVIDIA, five years, $3.4B and 60MW existing Childress capacity. May 26 Dell exhibit alone did not identify the customer.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -5573,7 +5570,7 @@
         <x:v>SRC-IREN-GPUFIN-8K-20260529</x:v>
       </x:c>
       <x:c r="B63" s="45" t="d">
-        <x:v>2026-05-29T00:00:00.000Z</x:v>
+        <x:v>2026-06-01T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C63" s="19" t="str">
         <x:v>IREN Limited / SEC</x:v>
@@ -5594,7 +5591,7 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="I63" s="43" t="str">
-        <x:v>Item 1.01 financing collateral covenants 1.05x ongoing DSCR and guarantees</x:v>
+        <x:v>SEC filing date June 1; agreement/event date May 29. Preserve separate dates.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -5768,7 +5765,7 @@
         <x:v>active</x:v>
       </x:c>
       <x:c r="I69" s="43" t="str">
-        <x:v>Re-read 8-K Item1.01 and Ex99.1: guarantee is IREN parent for its subsidiary, not NVIDIA. This exhibit describes an unnamed $3.4B customer contract and does not identify 60MW or NVIDIA as the customer; prior locator/title alone cannot establish those claims. See SRC-IREN-DELL-EX991-20260526.</x:v>
+        <x:v>May 26 exhibit alone names no customer or 60MW. May 7 Q3 release and August 27 10-K independently confirm NVIDIA customer attribution. Dell procurement guarantee is IREN parent, not NVIDIA.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -9829,38 +9826,125 @@
       </x:c>
     </x:row>
     <x:row r="211">
-      <x:c r="A211" s="20" t="str">
+      <x:c r="A211" s="19" t="str">
         <x:v>SRC-NBIS-STATUS-EUWEST2-20261015</x:v>
       </x:c>
-      <x:c r="B211" s="46" t="d">
+      <x:c r="B211" s="45" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C211" s="20" t="str">
+      <x:c r="C211" s="19" t="str">
         <x:v>Nebius service status</x:v>
       </x:c>
-      <x:c r="D211" s="44" t="str">
+      <x:c r="D211" s="43" t="str">
         <x:v>InfiniBand connectivity issues for GPU clusters in eu-west2</x:v>
       </x:c>
-      <x:c r="E211" s="44" t="str">
+      <x:c r="E211" s="43" t="str">
         <x:v>issuer_status_incident</x:v>
       </x:c>
-      <x:c r="F211" s="44" t="str">
+      <x:c r="F211" s="43" t="str">
         <x:v>https://status.nebius.com/incidents/sdb2htxgyprr</x:v>
       </x:c>
-      <x:c r="G211" s="44" t="str">
+      <x:c r="G211" s="43" t="str">
         <x:v>Nebius availability; no quantified MW impact</x:v>
       </x:c>
-      <x:c r="H211" s="44" t="str">
+      <x:c r="H211" s="43" t="str">
         <x:v>Primary</x:v>
       </x:c>
-      <x:c r="I211" s="44" t="str">
+      <x:c r="I211" s="43" t="str">
         <x:v>Incident sdb2htxgyprr; Investigating 05:34, Update 09:32, Monitoring 13:13 UTC. Issuer says recovery still in progress in 13:13 UTC update. Affected service EU-WEST2 Compute Cloud. No GPU count, MW, fleet-wide outage percentage, lost revenue or SLA credit amount disclosed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212">
+      <x:c r="A212" s="19" t="str">
+        <x:v>SRC-IREN-SEC-INDEX-20261016</x:v>
+      </x:c>
+      <x:c r="B212" s="45" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C212" s="19" t="str">
+        <x:v>IREN / SEC</x:v>
+      </x:c>
+      <x:c r="D212" s="43" t="str">
+        <x:v>IREN SEC submissions index checked October 16</x:v>
+      </x:c>
+      <x:c r="E212" s="43" t="str">
+        <x:v>regulator_index</x:v>
+      </x:c>
+      <x:c r="F212" s="43" t="str">
+        <x:v>https://data.sec.gov/submissions/CIK0001878848.json</x:v>
+      </x:c>
+      <x:c r="G212" s="43" t="str">
+        <x:v>IREN acceptance and collateral economics</x:v>
+      </x:c>
+      <x:c r="H212" s="43" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="I212" s="43" t="str">
+        <x:v>Latest 10-K filed August 27 for June 30; latest 10-Q filed May 8 for March 31. October 13 annual/proxy packet does not supply a later quarterly period. Financing 8-K filed June 1 reports May 29 agreements.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213">
+      <x:c r="A213" s="19" t="str">
+        <x:v>SRC-IREN-NEWS-20261016</x:v>
+      </x:c>
+      <x:c r="B213" s="45" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C213" s="19" t="str">
+        <x:v>IREN / SEC</x:v>
+      </x:c>
+      <x:c r="D213" s="43" t="str">
+        <x:v>IREN news index checked October 16</x:v>
+      </x:c>
+      <x:c r="E213" s="43" t="str">
+        <x:v>issuer_index</x:v>
+      </x:c>
+      <x:c r="F213" s="43" t="str">
+        <x:v>https://iren.com/investors/news</x:v>
+      </x:c>
+      <x:c r="G213" s="43" t="str">
+        <x:v>IREN acceptance and collateral economics</x:v>
+      </x:c>
+      <x:c r="H213" s="43" t="str">
+        <x:v>Primary</x:v>
+      </x:c>
+      <x:c r="I213" s="43" t="str">
+        <x:v>Retrieval date, not a new economic announcement date. No later earnings release or tranche acceptance found in the index at retrieval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214">
+      <x:c r="A214" s="20" t="str">
+        <x:v>SRC-IREN-ARS-20261013</x:v>
+      </x:c>
+      <x:c r="B214" s="46" t="d">
+        <x:v>2026-10-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C214" s="20" t="str">
+        <x:v>IREN / SEC</x:v>
+      </x:c>
+      <x:c r="D214" s="44" t="str">
+        <x:v>IREN FY2026 annual report shareholder packet</x:v>
+      </x:c>
+      <x:c r="E214" s="44" t="str">
+        <x:v>annual_report</x:v>
+      </x:c>
+      <x:c r="F214" s="44" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000114036126039453/ny20078226x3_ars.pdf</x:v>
+      </x:c>
+      <x:c r="G214" s="44" t="str">
+        <x:v>IREN acceptance and collateral economics</x:v>
+      </x:c>
+      <x:c r="H214" s="44" t="str">
+        <x:v>Primary; ARS text unreadable</x:v>
+      </x:c>
+      <x:c r="I214" s="44" t="str">
+        <x:v>Retrieved successfully but font mapping produced unusable extracted text. No incremental facts attributed to this wrapper. Read August 27 original SEC HTML 10-K for latest annual financial period; wrapper identity/content equivalence not asserted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10e370b215594803"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6ad833067f6462c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Research Azure: Maia rack economics, funding boundaries and October 18 handoff
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R59d81a709ab64bf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rd6ac2691c59c488f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="R57b6d850e387484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R8373101135494ebd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R155c9f989e3f4908"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rb9a56a9930dd4cfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R5a487a3e5e894414"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R15e81dfde8b04538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Ra71326954c8446ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rddf3c215bd8d48b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R8df89e8aa3314fb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R0a992bc8fadf4544"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R064227a7fbf5465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Redf8e0a10ebc4e62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I214" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I219" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1339,7 +1339,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O5" s="43" t="str">
-        <x:v>Restated Azure revenue; AI share, period-average active AI IT MW, physical utilization and matched full-fleet PUE missing. FY2025 PUE 1.17 and implied 1.55GW owned-fleet IT load are boundary diagnostics only; Q4 1GW addition excluded.</x:v>
+        <x:v>AI revenue share, average active AI IT MW and physical utilization missing. FY25 owned-fleet PUE 1.17 is historical. Maia300 575 accelerators/MW is a 2027 rack-design ratio, not current fleet capacity or PUE.</x:v>
       </x:c>
       <x:c r="P5" s="37" t="str">
         <x:f>IF(OR(D5="",E5="",F5=""),"",D5*E5*F5)</x:f>
@@ -2136,10 +2136,10 @@
         <x:v>Time-weighted average active Azure AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F5" s="43" t="str">
-        <x:v>Use September 2026 restated Azure perimeter; remove virtual desktop and non-AI consumption; include owned, leased, colocated and purchased capacity; never use quarterly added MW or PPA generation</x:v>
+        <x:v>Restated Azure perimeter; exclude internal Copilot and revenue-share income without attribution. Time-weight owned/leased/purchased AI IT MW. Maia rack density and token efficiency are separate design diagnostics.</x:v>
       </x:c>
       <x:c r="G5" s="43" t="str">
-        <x:v>Partial 2026-09-17; exact Azure revenue established; AI attribution and effective-MW denominator open</x:v>
+        <x:v>Partial 2026-10-18; Maia design separated; AI attribution and active-MW denominator open</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2467,7 +2467,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R161e8ba56d2148e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fd43c745a724159"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3439,7 +3439,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R901fa90c522842b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c478d0603074478"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9913,38 +9913,183 @@
       </x:c>
     </x:row>
     <x:row r="214">
-      <x:c r="A214" s="20" t="str">
+      <x:c r="A214" s="19" t="str">
         <x:v>SRC-IREN-ARS-20261013</x:v>
       </x:c>
-      <x:c r="B214" s="46" t="d">
+      <x:c r="B214" s="45" t="d">
         <x:v>2026-10-13T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C214" s="20" t="str">
+      <x:c r="C214" s="19" t="str">
         <x:v>IREN / SEC</x:v>
       </x:c>
-      <x:c r="D214" s="44" t="str">
+      <x:c r="D214" s="43" t="str">
         <x:v>IREN FY2026 annual report shareholder packet</x:v>
       </x:c>
-      <x:c r="E214" s="44" t="str">
+      <x:c r="E214" s="43" t="str">
         <x:v>annual_report</x:v>
       </x:c>
-      <x:c r="F214" s="44" t="str">
+      <x:c r="F214" s="43" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1878848/000114036126039453/ny20078226x3_ars.pdf</x:v>
       </x:c>
-      <x:c r="G214" s="44" t="str">
+      <x:c r="G214" s="43" t="str">
         <x:v>IREN acceptance and collateral economics</x:v>
       </x:c>
-      <x:c r="H214" s="44" t="str">
+      <x:c r="H214" s="43" t="str">
         <x:v>Primary; ARS text unreadable</x:v>
       </x:c>
-      <x:c r="I214" s="44" t="str">
+      <x:c r="I214" s="43" t="str">
         <x:v>Retrieved successfully but font mapping produced unusable extracted text. No incremental facts attributed to this wrapper. Read August 27 original SEC HTML 10-K for latest annual financial period; wrapper identity/content equivalence not asserted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215">
+      <x:c r="A215" s="19" t="str">
+        <x:v>SRC-MSFT-MAIA-20261012</x:v>
+      </x:c>
+      <x:c r="B215" s="45" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C215" s="19" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="D215" s="43" t="str">
+        <x:v>Maia production and multi-gigawatt roadmap</x:v>
+      </x:c>
+      <x:c r="E215" s="43" t="str">
+        <x:v>issuer_technology_announcement</x:v>
+      </x:c>
+      <x:c r="F215" s="43" t="str">
+        <x:v>https://blogs.microsoft.com/blog/2026/10/12/microsoft-to-expand-azure-maia-system-to-multi-gigawatt-deployments/</x:v>
+      </x:c>
+      <x:c r="G215" s="43" t="str">
+        <x:v>Azure economics and disclosure boundaries</x:v>
+      </x:c>
+      <x:c r="H215" s="43" t="str">
+        <x:v>Primary reviewed</x:v>
+      </x:c>
+      <x:c r="I215" s="43" t="str">
+        <x:v>Issuer claims, not independently measured fleet efficiency or paid Azure consumption.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216">
+      <x:c r="A216" s="19" t="str">
+        <x:v>SRC-MSFT-MAIA-ARCH-20261012</x:v>
+      </x:c>
+      <x:c r="B216" s="45" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C216" s="19" t="str">
+        <x:v>Microsoft Azure</x:v>
+      </x:c>
+      <x:c r="D216" s="43" t="str">
+        <x:v>Deep dive into Azure Maia 300 architecture</x:v>
+      </x:c>
+      <x:c r="E216" s="43" t="str">
+        <x:v>issuer_technical_architecture</x:v>
+      </x:c>
+      <x:c r="F216" s="43" t="str">
+        <x:v>https://azure.microsoft.com/en-us/blog/deep-dive-into-azure-maia-300-architecture/</x:v>
+      </x:c>
+      <x:c r="G216" s="43" t="str">
+        <x:v>Azure economics and disclosure boundaries</x:v>
+      </x:c>
+      <x:c r="H216" s="43" t="str">
+        <x:v>Primary reviewed</x:v>
+      </x:c>
+      <x:c r="I216" s="43" t="str">
+        <x:v>Read through web extraction; direct download returned a short access response. Rack design includes host/memory/storage and rack switches; not total facility energy. No disclosed standardized comparative workload.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217">
+      <x:c r="A217" s="19" t="str">
+        <x:v>SRC-MSFT-SEC-INDEX-20261018</x:v>
+      </x:c>
+      <x:c r="B217" s="45" t="d">
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C217" s="19" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D217" s="43" t="str">
+        <x:v>Microsoft submissions index checked October 18</x:v>
+      </x:c>
+      <x:c r="E217" s="43" t="str">
+        <x:v>regulator_index</x:v>
+      </x:c>
+      <x:c r="F217" s="43" t="str">
+        <x:v>https://data.sec.gov/submissions/CIK0000789019.json</x:v>
+      </x:c>
+      <x:c r="G217" s="43" t="str">
+        <x:v>Azure economics and disclosure boundaries</x:v>
+      </x:c>
+      <x:c r="H217" s="43" t="str">
+        <x:v>Primary reviewed</x:v>
+      </x:c>
+      <x:c r="I217" s="43" t="str">
+        <x:v>Latest 10-K July29, latest 10-Q April29, latest material 8-K September2. No September-quarter results yet.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218">
+      <x:c r="A218" s="19" t="str">
+        <x:v>SRC-MSFT-EARNINGS-DATE-20261007</x:v>
+      </x:c>
+      <x:c r="B218" s="45" t="d">
+        <x:v>2026-10-07T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C218" s="19" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="D218" s="43" t="str">
+        <x:v>FY2027 first-quarter earnings date</x:v>
+      </x:c>
+      <x:c r="E218" s="43" t="str">
+        <x:v>issuer_calendar_announcement</x:v>
+      </x:c>
+      <x:c r="F218" s="43" t="str">
+        <x:v>https://news.microsoft.com/source/2026/10/07/microsoft-announces-quarterly-earnings-release-date-69/</x:v>
+      </x:c>
+      <x:c r="G218" s="43" t="str">
+        <x:v>Azure economics and disclosure boundaries</x:v>
+      </x:c>
+      <x:c r="H218" s="43" t="str">
+        <x:v>Primary reviewed</x:v>
+      </x:c>
+      <x:c r="I218" s="43" t="str">
+        <x:v>Results scheduled October28 after market close; call 2:30PM Pacific. Not a results release.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219">
+      <x:c r="A219" s="20" t="str">
+        <x:v>SRC-CEG-CRANE-UPDATE-20260806</x:v>
+      </x:c>
+      <x:c r="B219" s="46" t="d">
+        <x:v>2026-08-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C219" s="20" t="str">
+        <x:v>Constellation Energy</x:v>
+      </x:c>
+      <x:c r="D219" s="44" t="str">
+        <x:v>Q2 2026 Crane restart progress</x:v>
+      </x:c>
+      <x:c r="E219" s="44" t="str">
+        <x:v>counterparty_earnings_release</x:v>
+      </x:c>
+      <x:c r="F219" s="44" t="str">
+        <x:v>https://www.constellationenergy.com/news/2026/08/constellation-reports-second-quarter-2026-results.html</x:v>
+      </x:c>
+      <x:c r="G219" s="44" t="str">
+        <x:v>Azure economics and disclosure boundaries</x:v>
+      </x:c>
+      <x:c r="H219" s="44" t="str">
+        <x:v>Primary reviewed</x:v>
+      </x:c>
+      <x:c r="I219" s="44" t="str">
+        <x:v>FERC interconnection-rights waiver and NRC fuel-license amendment reported; 2027 restart target supersedes original 2028, not actual commissioning.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6ad833067f6462c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15a255f592ac4353"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Review AWS financing, chip idle-risk boundaries and power delivery (2026-10-19)
</commit_message>
<xml_diff>
--- a/data/ai-compute-economics.xlsx
+++ b/data/ai-compute-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R15e81dfde8b04538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Ra71326954c8446ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Rddf3c215bd8d48b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="R8df89e8aa3314fb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R0a992bc8fadf4544"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R064227a7fbf5465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="Redf8e0a10ebc4e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra9d44ed11adc4432"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Models" sheetId="2" r:id="Rda2c48d0b1534d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="3" r:id="Re9c0d97b80574012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Economics" sheetId="4" r:id="Rd46225592b404892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" r:id="R7cd71d1c77cb4b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R7f9545ba729f44a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R784835897c244ce9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I219" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceRegisterTable" displayName="SourceRegisterTable" ref="A4:I228" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -1388,7 +1388,7 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="O6" s="43" t="str">
-        <x:v>AWS all services; AI/chips run rates overlap and are not Q2 AI revenue. Active AI IT MW and utilization missing. 2025 PUE 1.14 is historical only.</x:v>
+        <x:v>Q2 AI revenue attribution, average active IT MW and utilization missing. PUE 1.14 is FY2025 only. Usage and fixed-term billing differ; no measured idle-chip stock.</x:v>
       </x:c>
       <x:c r="P6" s="37" t="str">
         <x:f>IF(OR(D6="",E6="",F6=""),"",D6*E6*F6)</x:f>
@@ -2159,10 +2159,10 @@
         <x:v>Time-weighted active AI IT MW times physical utilization</x:v>
       </x:c>
       <x:c r="F6" s="43" t="str">
-        <x:v>Separate Trainium Inferentia and NVIDIA; exclude internal/noncompute revenue and run-rate overlap; PUE only for matched facility-power conversion</x:v>
+        <x:v>Separate metered usage and ratable fixed capacity; Trainium/Inferentia versus NVIDIA; matched AI revenue and active cohorts; corporate unsecured debt is not chip collateral.</x:v>
       </x:c>
       <x:c r="G6" s="43" t="str">
-        <x:v>Partial 2026-09-19; matched numerator and denominator open</x:v>
+        <x:v>Partial 2026-10-19; funding and PPA timing verified; idle cohorts and matched MW economics open</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2467,7 +2467,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fd43c745a724159"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd00a1bf002154d8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3439,7 +3439,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c478d0603074478"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e87473255834297"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10058,38 +10058,297 @@
       </x:c>
     </x:row>
     <x:row r="219">
-      <x:c r="A219" s="20" t="str">
+      <x:c r="A219" s="19" t="str">
         <x:v>SRC-CEG-CRANE-UPDATE-20260806</x:v>
       </x:c>
-      <x:c r="B219" s="46" t="d">
+      <x:c r="B219" s="45" t="d">
         <x:v>2026-08-06T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C219" s="20" t="str">
+      <x:c r="C219" s="19" t="str">
         <x:v>Constellation Energy</x:v>
       </x:c>
-      <x:c r="D219" s="44" t="str">
+      <x:c r="D219" s="43" t="str">
         <x:v>Q2 2026 Crane restart progress</x:v>
       </x:c>
-      <x:c r="E219" s="44" t="str">
+      <x:c r="E219" s="43" t="str">
         <x:v>counterparty_earnings_release</x:v>
       </x:c>
-      <x:c r="F219" s="44" t="str">
+      <x:c r="F219" s="43" t="str">
         <x:v>https://www.constellationenergy.com/news/2026/08/constellation-reports-second-quarter-2026-results.html</x:v>
       </x:c>
-      <x:c r="G219" s="44" t="str">
+      <x:c r="G219" s="43" t="str">
         <x:v>Azure economics and disclosure boundaries</x:v>
       </x:c>
-      <x:c r="H219" s="44" t="str">
+      <x:c r="H219" s="43" t="str">
         <x:v>Primary reviewed</x:v>
       </x:c>
-      <x:c r="I219" s="44" t="str">
+      <x:c r="I219" s="43" t="str">
         <x:v>FERC interconnection-rights waiver and NRC fuel-license amendment reported; 2027 restart target supersedes original 2028, not actual commissioning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220">
+      <x:c r="A220" s="19" t="str">
+        <x:v>SRC-AMZN-SEC-INDEX-20261019</x:v>
+      </x:c>
+      <x:c r="B220" s="45"/>
+      <x:c r="C220" s="19" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D220" s="43" t="str">
+        <x:v>Amazon SEC submissions freshness check</x:v>
+      </x:c>
+      <x:c r="E220" s="43" t="str">
+        <x:v>filing_index</x:v>
+      </x:c>
+      <x:c r="F220" s="43" t="str">
+        <x:v>https://data.sec.gov/submissions/CIK0001018724.json</x:v>
+      </x:c>
+      <x:c r="G220" s="43" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H220" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I220" s="43" t="str">
+        <x:v>filings.recent: form, filingDate, accessionNumber, primaryDocument</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221">
+      <x:c r="A221" s="19" t="str">
+        <x:v>SRC-AMZN-GBP-CLOSE-20260914</x:v>
+      </x:c>
+      <x:c r="B221" s="45" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C221" s="19" t="str">
+        <x:v>Amazon / SEC</x:v>
+      </x:c>
+      <x:c r="D221" s="43" t="str">
+        <x:v>Sterling notes closing</x:v>
+      </x:c>
+      <x:c r="E221" s="43" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="F221" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1018724/000110465926107526/tm2624614d5_8k.htm</x:v>
+      </x:c>
+      <x:c r="G221" s="43" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H221" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I221" s="43" t="str">
+        <x:v>Item 8.01 p.3; Item 9.01 p.4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222">
+      <x:c r="A222" s="19" t="str">
+        <x:v>SRC-AMZN-GBP-PROSPECTUS-20260911</x:v>
+      </x:c>
+      <x:c r="B222" s="45" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C222" s="19" t="str">
+        <x:v>Amazon / SEC</x:v>
+      </x:c>
+      <x:c r="D222" s="43" t="str">
+        <x:v>Sterling notes final prospectus supplement</x:v>
+      </x:c>
+      <x:c r="E222" s="43" t="str">
+        <x:v>424B5</x:v>
+      </x:c>
+      <x:c r="F222" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1018724/000110465926107122/tm2624614-3_424b5.htm</x:v>
+      </x:c>
+      <x:c r="G222" s="43" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H222" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I222" s="43" t="str">
+        <x:v>Cover pricing/proceeds table; S-3 Ranking; S-7 Risk Factors; Use of Proceeds</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223">
+      <x:c r="A223" s="19" t="str">
+        <x:v>SRC-AMZN-GBP-CERT-20260914</x:v>
+      </x:c>
+      <x:c r="B223" s="45" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C223" s="19" t="str">
+        <x:v>Amazon / SEC</x:v>
+      </x:c>
+      <x:c r="D223" s="43" t="str">
+        <x:v>Officers certificate and sterling note forms</x:v>
+      </x:c>
+      <x:c r="E223" s="43" t="str">
+        <x:v>8-K_Exhibit_4.1</x:v>
+      </x:c>
+      <x:c r="F223" s="43" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1018724/000110465926107526/tm2624614d5_ex4-1.htm</x:v>
+      </x:c>
+      <x:c r="G223" s="43" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H223" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I223" s="43" t="str">
+        <x:v>Sections 6(b)-(e) p.2 principal, maturities, coupons; 6(k) no sinking fund; note forms</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224">
+      <x:c r="A224" s="19" t="str">
+        <x:v>SRC-AMZN-EARNINGS-DATE-20261015</x:v>
+      </x:c>
+      <x:c r="B224" s="45" t="d">
+        <x:v>2026-10-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C224" s="19" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="D224" s="43" t="str">
+        <x:v>Q3 2026 earnings date</x:v>
+      </x:c>
+      <x:c r="E224" s="43" t="str">
+        <x:v>issuer_calendar</x:v>
+      </x:c>
+      <x:c r="F224" s="43" t="str">
+        <x:v>https://press.aboutamazon.com/2026/10/amazon-com-to-webcast-third-quarter-2026-financial-results-conference-call</x:v>
+      </x:c>
+      <x:c r="G224" s="43" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H224" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I224" s="43" t="str">
+        <x:v>Opening announcement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225">
+      <x:c r="A225" s="19" t="str">
+        <x:v>SRC-AWS-TORCHNEURON-20261019</x:v>
+      </x:c>
+      <x:c r="B225" s="45" t="d">
+        <x:v>2026-10-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C225" s="19" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="D225" s="43" t="str">
+        <x:v>TorchNeuron native PyTorch support announcement</x:v>
+      </x:c>
+      <x:c r="E225" s="43" t="str">
+        <x:v>issuer_technology_announcement</x:v>
+      </x:c>
+      <x:c r="F225" s="43" t="str">
+        <x:v>https://www.aboutamazon.com/news/innovation-at-amazon/torchneuron-pytorch-aws-trainium-chips-ai</x:v>
+      </x:c>
+      <x:c r="G225" s="43" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H225" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I225" s="43" t="str">
+        <x:v>What does no code change mean; Why TorchNeuron matters; What is next</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226">
+      <x:c r="A226" s="19" t="str">
+        <x:v>SRC-AWS-BUILT-TOGETHER-20261002</x:v>
+      </x:c>
+      <x:c r="B226" s="45" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C226" s="19" t="str">
+        <x:v>Amazon / Matt Garman</x:v>
+      </x:c>
+      <x:c r="D226" s="43" t="str">
+        <x:v>AWS community and data center commitment</x:v>
+      </x:c>
+      <x:c r="E226" s="43" t="str">
+        <x:v>issuer_policy_announcement</x:v>
+      </x:c>
+      <x:c r="F226" s="43" t="str">
+        <x:v>https://www.aboutamazon.com/news/company-news/amazon-data-centers-built-together</x:v>
+      </x:c>
+      <x:c r="G226" s="43" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H226" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I226" s="43" t="str">
+        <x:v>Our Data Center Commitment items 1, 3, 4; Built Together</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227">
+      <x:c r="A227" s="19" t="str">
+        <x:v>SRC-TALEN-AWS-10Q-20260805</x:v>
+      </x:c>
+      <x:c r="B227" s="45" t="d">
+        <x:v>2026-08-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C227" s="19" t="str">
+        <x:v>Talen / SEC</x:v>
+      </x:c>
+      <x:c r="D227" s="43" t="str">
+        <x:v>Talen Q2 2026 AWS PPA transition disclosure</x:v>
+      </x:c>
+      <x:c r="E227" s="43" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F227" s="43" t="str">
+        <x:v>https://ir.talenenergy.com/node/9536/html</x:v>
+      </x:c>
+      <x:c r="G227" s="43" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H227" s="43" t="str">
+        <x:v>primary_read</x:v>
+      </x:c>
+      <x:c r="I227" s="43" t="str">
+        <x:v>p.44 Glossary: AWS PPA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228">
+      <x:c r="A228" s="20" t="str">
+        <x:v>SRC-AWS-BI-LEAD-20261019</x:v>
+      </x:c>
+      <x:c r="B228" s="46" t="d">
+        <x:v>2026-10-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C228" s="20" t="str">
+        <x:v>Business Insider</x:v>
+      </x:c>
+      <x:c r="D228" s="44" t="str">
+        <x:v>Amazon AI buildout constraints reporting lead</x:v>
+      </x:c>
+      <x:c r="E228" s="44" t="str">
+        <x:v>secondary_search_excerpt</x:v>
+      </x:c>
+      <x:c r="F228" s="44" t="str">
+        <x:v>https://www.businessinsider.com/amazon-220-billion-ai-bet-data-centers-spending-challenges-2026-10</x:v>
+      </x:c>
+      <x:c r="G228" s="44" t="str">
+        <x:v>amazon_aws;contract_economics</x:v>
+      </x:c>
+      <x:c r="H228" s="44" t="str">
+        <x:v>secondary_excerpt_only</x:v>
+      </x:c>
+      <x:c r="I228" s="44" t="str">
+        <x:v>Search excerpt on power and warehouse staging</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15a255f592ac4353"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raadce362295f45c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>